<commit_message>
feat(enterprise): add -PruneShadowsOnly mode to strip sheet-scoped shadow names
</commit_message>
<xml_diff>
--- a/Excel/9_Refrigerants_WIP_v02.xlsx
+++ b/Excel/9_Refrigerants_WIP_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D31B6EF2-FC2B-490F-A665-B5F02DC7A181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B592100-A9E1-49C2-984D-5A459EF2A56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" firstSheet="2" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1575" yWindow="540" windowWidth="36255" windowHeight="19140" firstSheet="2" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -258,15 +258,6 @@
     <definedName name="Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary_Unit">_xlfn.LAMBDA("t CO2-e")</definedName>
     <definedName name="Fuel_Equations.VEERG_8_2_1_1__1_FuelCombustionStationary_Variable">_xlfn.LAMBDA("E_g")</definedName>
     <definedName name="Fuel_Equations.VEERG_8_FuelCombustion">_xlfn.LAMBDA(_xlpm.Q,_xlpm.EC,_xlpm.EF, (_xlpm.Q * _xlpm.EC * _xlpm.EF) * 10 ^ -3)</definedName>
-    <definedName name="Fuel_Equations.VEERG_8_X_FuelCombustionGeneric">_xlfn.LAMBDA(_xlpm.Q_GCq,_xlpm.EC_GCq,_xlpm.EF_GC1qg, Fuel_Equations.VEERG_8_FuelCombustion(_xlpm.Q_GCq, _xlpm.EC_GCq, _xlpm.EF_GC1qg))</definedName>
-    <definedName name="Fuel_Equations.VEERG_8_X_FuelCombustionGeneric_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(7, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Q_GCq","Amount of fuel type q used for generic combustion operations","Varies based on fuel type: kL, m3, GJ","Input";"EC_GCq","Energy content factor for generic combustion operations","GJ / unit of fuel","Constant";"EF_GC1qg","Scope 1 emission factor for generic combustion for each greenhouse gas","kg CO2e / GJ","Constant";"q","Fuel type","","Constant";"GC","Generic combustion","","Constant";"g","Greenhouse gas","","Constant";"1","Scope 1","","Constant"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="Fuel_Equations.VEERG_8_X_FuelCombustionGeneric_LatexEquation">_xlfn.LAMBDA("E_g=\sum\nolimits_t \sum\nolimits_q\left(Q_{GC,q}\times EC_{GC,q}\times EF_{GC,1,qg}\right)\times 10^{-3}")</definedName>
-    <definedName name="Fuel_Equations.VEERG_8_X_FuelCombustionGeneric_NIRReference">_xlfn.LAMBDA("Australian National Greenhouse Accounts Factors 2025 - 2.2 Estimating emissions from generic energy sources - Calculating emissions from generic combustion of liquid fuels and 2.3 Estimating emissions from transport fuels")</definedName>
-    <definedName name="Fuel_Equations.VEERG_8_X_FuelCombustionGeneric_Source">_xlfn.LAMBDA("Uses VEERG 2026: 8.1.1.1, Equation (1), 8.2.1.1, Equation (1) and everages the Australian National Greenhouse Accounts Factors 2025 for transport and stationary fuel combustion")</definedName>
-    <definedName name="Fuel_Equations.VEERG_8_X_FuelCombustionGeneric_Title">_xlfn.LAMBDA("Emissions for each GHG from the generic combustion of fuels")</definedName>
-    <definedName name="Fuel_Equations.VEERG_8_X_FuelCombustionGeneric_Unit">_xlfn.LAMBDA("t CO2-e")</definedName>
-    <definedName name="Fuel_Equations.VEERG_8_X_FuelCombustionGeneric_Variable">_xlfn.LAMBDA("E_g")</definedName>
-    <definedName name="Fuel_Equations.VEERG_8_X_FuelCombustionGeneric_Variation">_xlfn.LAMBDA("VARIATION ON SOURCE: This calculation uses averages of transport and stationary emission factors for fuel combustion where the usage is not known.")</definedName>
     <definedName name="Fuel_InputFunctions.Fuel_GetStationaryFuelString">_xlfn.LAMBDA(_xlpm.Cell,
     RIGHT(_xlpm.Cell,LEN(_xlpm.Cell)-FIND(", ",_xlpm.Cell))
 )</definedName>
@@ -359,7 +350,7 @@
     <definedName name="Refrigerants_SourceData.Refrigerants_ChemicalGWP_Source">_xlfn.LAMBDA(("Australian National Greenhouse Accounts Factors 2025 - Appendix 2 - Table 23"))</definedName>
     <definedName name="Refrigerants_SourceData.Refrigerants_ChemicalGWP_Title">_xlfn.LAMBDA(("Global Warming Potentials"))</definedName>
     <definedName name="Refrigerants_SourceData.Refrigerants_ChemicalGWP_Variation">_xlfn.LAMBDA(("VARIATION OF SOURCE DATA: Added 'GAS - FC name' column with truncated gas name to allow matching with other tables. Added extra gases from IPCC Global Warming Potential Values v2.0 - (AR5). Added 'Additional data source' column."))</definedName>
-    <definedName name="Refrigerants_SourceData.Refrigerants_LeakageRates_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(81, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Annual leakage rate (%)";"Domestic refrigerators",1.7;"Transport refrigeration",15.7;"Domestic A/C portable",2.5;"Domestic A/C split",3.5;"Domestic A/C packaged",2.5;"Light vehicle A/C",6.7;"Heavy vehicle A/C",10.8}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="Refrigerants_SourceData.Refrigerants_LeakageRates_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(8, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Product","Annual leakage rate (%)";"Domestic refrigerators",1.7;"Transport refrigeration",15.7;"Domestic A/C portable",2.5;"Domestic A/C split",3.5;"Domestic A/C packaged",2.5;"Light vehicle A/C",6.7;"Heavy vehicle A/C",10.8}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Refrigerants_SourceData.Refrigerants_LeakageRates_Description">_xlfn.LAMBDA((""))</definedName>
     <definedName name="Refrigerants_SourceData.Refrigerants_LeakageRates_Source">_xlfn.LAMBDA(("Australian National Greenhouse Accounts Factors 2025 - Table 10"))</definedName>
     <definedName name="Refrigerants_SourceData.Refrigerants_LeakageRates_Title">_xlfn.LAMBDA(("Indicative leakage rates for common refrigeration and air - conditioning equipment"))</definedName>
@@ -5577,7 +5568,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="866" row="4">
+  <wetp:taskpane dockstate="right" visibility="0" width="750" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -19296,6 +19287,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
@@ -19306,20 +19306,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACkAKgAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADIAKQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlACkAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwBlAGwAbAAsACAARABlAGwAaQBtAGkAdABlAHIALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEAXQAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgBdACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgBYAE0ATAAoAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAHQAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMAcwBcAHUAMAAwADMAZQBcACIAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFMAVQBCAFMAVABJAFQAVQBUAEUAKABDAGUAbABsACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEALABcACIAXAAiACkALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABEAGUAbABpAG0AaQB0AGUAcgAsAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMAcwBcAHUAMAAwADMAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAApACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAC8AdABcAHUAMAAwADMAZQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAvAC8AcwBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAGEAdgBnAFQAZQBtAHAALABhAHYAZwBSAGEAaQBuACwAZgByAG8AcwB0AEQAYQB5AHMALABlAGwAZQB2ACwAbQBhAHAAXwBwAGUAdAAsAFwAbgAgACAAIAAgAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACwAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkALABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUABFAFQAQQByAHIAYQB5ACwAbQBhAHgAUABFAFQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AG0AYQBwAF8AcABlAHQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABQAEUAVABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AG0AYQBwAF8AcABlAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABBAEsARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgADEAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAE0AaQBuAEEAcgByAGEAeQAsACAATQBhAHgAQQByAHIAYQB5ACwAIABJAHQAZQBtAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AaQBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABJAHQAZQBtAEEAcgByAGEAeQAsACAAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwByAGkAdABlAHIAaQBhADEALAAgAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5ACwAIABRAHUAYQBuAHQAaQB0AHkALAAgAFsATQB1AGwAdABpAHAAbABpAGUAcgBdACwAIABbAEMAcgBpAHQAZQByAGkAYQAyAF0ALABbAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQBdACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgATQB1AGwAdABpAHAAbABpAGUAcgApACwAMQAsAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsAFwAbgAgACAAIAAgAHEAdQBhAG4AdABpAHQAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACoATQB1AGwAdABpAHAAbABpAGUAcgAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMQApACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADIALABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAcgBpAHQAZQByAGkAYQAyACkALAAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADIAKQApACwAXABuACAAIAAgACAAUwBVAE0AUABSAE8ARABVAEMAVAAoAGMAcgBpAHQAZQByAGkAYQAxACoAYwByAGkAdABlAHIAaQBhADIAKgBxAHUAYQBuAHQAaQB0AHkAKQBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjACAAUwApACwAXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAG4AZQB4AHQAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAUwApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBiACAAcwB0AGEAcgB0AHMAIABhAGYAdABlAHIAIABFACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUARQApACwAXABuACAAIAAgACAAIAAgACAAIABuACwATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAcgBzACwAUwBFAFEAVQBFAE4AQwBFACgAbgAsADEALABmAGkAcgBzAHQAWQBlAGEAcgAsADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALABEAEEAVABFACgAeQByAHMALABtACwAZAApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzACwATQBBAFAAKABzAHQAYQByAHQAcwAsAFAAZQByAGkAbwBkAEUAbgBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAHQAYQBnACwASQBGACgAcwB0AGEAcgB0AHMAPQBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXAAiACAAKABUAGgAaQBzACAAcgBlAHAAbwByAHQAaQBuAGcAIABjAHkAYwBsAGUAKQBcACIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzAFQAZQB4AHQALABUAEUAWABUACgAcwB0AGEAcgB0AHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzAFQAZQB4AHQALABUAEUAWABUACgAZQBuAGQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAXAAiACAAdABvACAAXAAiACAAXAB1ADAAMAAyADYAIABlAG4AZABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAHQAYQBnACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQBcAG4APQBMAEEATQBCAEQAQQAoAEYAdQBuAGMAdABpAG8AbgAsACAAVABFAFgAVABCAEUARgBPAFIARQAoAEYATwBSAE0AVQBMAEEAVABFAFgAVAAoAEYAdQBuAGMAdABpAG8AbgApACwAIABcACIAKABcACIAKQApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5ACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkALABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAA9AFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACAAPQAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5AD0AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkAPQBJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkAPQBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAFwAdQAwADAAMwBlADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAdQAwADAAMgA3AFwAIgAgAFwAdQAwADAAMgA2ACAAcwBoACAAXAB1ADAAMAAyADYAIABcACIAXAB1ADAAMAAyADcAIQBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsARABpAGYAZgBlAHIAZQBuAHQAUwBoAGUAZQB0AFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADEALAAgADIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADMALAAgADQAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAATQBNAFMALAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFwAbgAgACAAIAAgACAAIAAgACAATQBFAEQASQBBAE4AKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFUATgBEACgAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIAAwACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAE0ATQBTACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAaQB0AGwAZQBDAGUAbABsACwAIABTAG8AdQByAGMAZQBDAGUAbABsACwAXABuACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAEwARQBGAFQAKABTAG8AdQByAGMAZQBDAGUAbABsACwAIABGAEkATgBEACgAXAAiACwAXAAiACwAIABTAG8AdQByAGMAZQBDAGUAbABsACkAIAAtADEAKQAsACAAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFwAIgAsACAAXAAiAFwAIgApACAAXAB1ADAAMAAyADYAIABcACIAIABcACIAIABcAHUAMAAwADIANgAgAFQAaQB0AGwAZQBDAGUAbABsAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBEAGkAcgBlAGMAdAAgACgAUwBjAG8AcABlACAAMQApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzACAAaQBuAGMAbAB1AGQAaQBuAGcAIABsAGkAcQB1AGUAZgBpAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAgACAAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAA1AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAANwAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAHUAZQBsACAAYwBvAG0AYgB1AHMAdABlAGQAXAAiACwAIABcACIARQBuAGUAcgBnAHkAIABDAG8AbgB0AGUAbgB0ACAARgBhAGMAdABvAHIAIAAoAEcASgAgAHAAZQByACAAdQBuAGkAdAAgAG8AZgAgAGYAdQBlAGwAKQBcACIALAAgAFwAIgBGAHUAZQBsACAAdQBuAGkAdABcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAE8AMgBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAEgANABcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABOADIATwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAG8AbQBiAGkAbgBlAGQAIABnAGEAcwBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBhAHQAdQByAGEAbAAgAGcAYQBzACAAZABpAHMAdAByAGkAYgB1AHQAZQBkACAAaQBuACAAYQAgAHAAaQBwAGUAbABpAG4AZQBcACIALAAgADAALgAwADMAOQAzACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBhAGwAIABzAGUAYQBtACAAbQBlAHQAaABhAG4AZQAgAHQAaABhAHQAIABpAHMAIABjAGEAcAB0AHUAcgBlAGQAIABmAG8AcgAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AXAAiACwAIAAwAC4AMAAzADcANwAsACAAXAAiAG0AMwBcACIALAAgADUAMQAuADQALAAgADAALgAyACwAIAAwAC4AMAAzACwAIAA1ADEALgA2ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AYQBsACAAbQBpAG4AZQAgAHcAYQBzAHQAZQAgAGcAYQBzACAAdABoAGEAdAAgAGkAcwAgAGMAYQBwAHQAdQByAGUAZAAgAGYAbwByACAAYwBvAG0AYgB1AHMAdABpAG8AbgBcACIALAAgADAALgAwADMANwA3ACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4AOQAsACAANAAuADYALAAgADAALgAzACwAIAA1ADYALgA4ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcAByAGUAcwBzAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAoAHIAZQB2AGUAcgB0AGkAbgBnACAAdABvACAAcwB0AGEAbgBkAGEAcgBkACAAYwBvAG4AZABpAHQAaQBvAG4AcwApAFwAIgAsACAAMAAuADAAMwA5ADMALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAANQAxAC4ANQAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVQBuAHAAcgBvAGMAZQBzAHMAZQBkACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAFwAIgAsACAAMAAuADAAMwA5ADMALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAANQAxAC4ANQAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIARQB0AGgAYQBuAGUAXAAiACwAIAAwAC4AMAA2ADIAOQAsACAAXAAiAG0AMwBcACIALAAgADUANgAuADUALAAgADAALgAwADMALAAgADAALgAwADMALAAgADUANgAuADUANgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBrAGUAIABvAHYAZQBuACAAZwBhAHMAXAAiACwAIAAwAC4AMAAxADgAMQAsACAAXAAiAG0AMwBcACIALAAgADMANwAuADAALAAgADAALgAwADMALAAgADAALgAwADUALAAgADMANwAuADAAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEIAbABhAHMAdAAgAGYAdQByAG4AYQBjAGUAIABnAGEAcwBcACIALAAgADAALgAwADAANAAwACwAIABcACIAbQAzAFwAIgAsACAAMgAzADQALgAwACwAIAAwAC4AMAAzACwAIAAwAC4AMAAyACwAIAAyADMANAAuADAANQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAbwB3AG4AIABnAGEAcwBcACIALAAgADAALgAwADMAOQAwACwAIABcACIAbQAzAFwAIgAsACAANgAwAC4AMgAsACAAMAAuADAANAAsACAAMAAuADAAMwAsACAANgAwAC4AMgA3ADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAXAAiACwAIAAyADUALgAzACwAIABcACIAawBMAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAGUAbwB1AHMAIABmAG8AcwBzAGkAbAAgAGYAdQBlAGwAcwAgAG8AdABoAGUAcgAgAHQAaABhAG4AIAB0AGgAbwBzAGUAIABtAGUAbgB0AGkAbwBuAGUAZAAgAGkAbgAgAHQAaABlACAAaQB0AGUAbQBzACAAYQBiAG8AdgBlAFwAIgAsACAAMAAuADAAMwA5ADAALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAANQAxAC4ANQAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsACAAYgBpAG8AZwBhAHMAIAB0AGgAYQB0ACAAaQBzACAAYwBhAHAAdAB1AHIAZQBkACAAZgBvAHIAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAKABtAGUAdABoAGEAbgBlACAAbwBuAGwAeQApAFwAIgAsACAAMAAuADAAMwA3ADcALAAgAFwAIgBtADMAXAAiACwAIAAwAC4AMAAsACAANgAuADQALAAgADAALgAwADMALAAgADYALgA0ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAGwAdQBkAGcAZQAgAGIAaQBvAGcAYQBzACAAdABoAGEAdAAgAGkAcwAgAGMAYQBwAHQAdQByAGUAZAAgAGYAbwByACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgACgAbQBlAHQAaABhAG4AZQAgAG8AbgBsAHkAKQBcACIALAAgADAALgAwADMANwA3ACwAIABcACIAbQAzAFwAIgAsACAAMAAuADAALAAgADYALgA0ACwAIAAwAC4AMAAzACwAIAA2AC4ANAAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQAgAGIAaQBvAGcAYQBzACAAdABoAGEAdAAgAGkAcwAgAGMAYQBwAHQAdQByAGUAZAAgAGYAbwByACAAYwBvAG0AYgB1AHMAdABpAG8AbgAsACAAbwB0AGgAZQByACAAdABoAGEAbgAgAHQAaABvAHMAZQAgAG0AZQBuAHQAaQBvAG4AZQBkACAAaQBuACAAdABoAGUAIABpAHQAZQBtAHMAIABhAGIAbwB2AGUAXAAiACwAIAAwAC4AMAAzADcAMAAsACAAXAAiAG0AMwBcACIALAAgADAALgAwACwAIAA2AC4ANAAsACAAMAAuADAAMwAsACAANgAuADQAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEIAaQBvAG0AZQB0AGgAYQBuAGUAXAAiACwAIAAwAC4AMAAzADkAMwAsACAAXAAiAG0AMwBcACIALAAgADAALgAwACwAIAAwAC4AMQAsACAAMAAuADAAMwAsACAAMAAuADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAeQBkAHIAbwBnAGUAbgBcACIALAAgADAALgAwADEAMgAyACwAIABcACIAbQAzAFwAIgAsACAAMAAuADAALAAgADAALgAwACwAIAAwAC4ANQAsACAAMAAuADUAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAGEAdAB1AHIAYQBsACAAZwBhAHMAIABkAGkAcwB0AHIAaQBiAHUAdABlAGQAIABpAG4AIABhACAAcABpAHAAZQBsAGkAbgBlACAALQAgAEcAaQBnAGEAagBvAHUAbABlAHMAXAAiACwAIAAxACwAIABcACIARwBKAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAbwB3AG4AIABnAGEAcwAgAC0AIABHAGkAZwBhAGoAbwB1AGwAZQBzAFwAIgAsACAAMQAsACAAXAAiAEcASgBcACIALAAgADYAMAAuADIALAAgADAALgAwADQALAAgADAALgAwADMALAAgADYAMAAuADIANwBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAFwAdQAwADAAMgA3AE4AYQB0AHUAcgBhAGwAIABnAGEAcwAgAGQAaQBzAHQAcgBpAGIAdQB0AGUAZAAgAGkAbgAgAGEAIABwAGkAcABlAGwAaQBuAGUAIAAtACAARwBpAGcAYQBqAG8AdQBsAGUAcwBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAVABvAHcAbgAgAGcAYQBzACAALQAgAEcAaQBnAGEAagBvAHUAbABlAHMAXAB1ADAAMAAyADcAIAB3AGUAcgBlACAAYQBkAGQAZQBkACwAIABlAGEAYwBoACAAdwBpAHQAaAAgAGEAbgAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAGYAYQBjAHQAbwByACAAbwBmACAAMQAgAEcASgAgAHAAZQByACAAdQBuAGkAdAAgAG8AZgAgAGYAdQBlAGwALgAgAFQAaABpAHMAIABpAHMAIABmAG8AcgAgAHUAcwBlAHIAcwAgAHcAaABvACAAaABhAHYAZQAgAGYAdQBlAGwAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABkAGEAdABhACAAaQBuACAARwBKACAAcgBhAHQAaABlAHIAIAB0AGgAYQBuACAAbQAzAC4AXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ARgB1AGUAbAAgAHMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARgB1AGUAbAAgAHMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBJAG4AZABpAHIAZQBjAHQAIAAoAFMAYwBvAHAAZQAgADMAKQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAC4AXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAA2AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAdABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMwAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIABmAG8AcgAgAE4AYQB0AHUAcgBhAGwAIABHAGEAcwAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAE0AZQB0AHIAbwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAcwAgAGYAbwByACAATgBhAHQAdQByAGEAbAAgAEcAYQBzACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAATgBvAG4AIAAtACAATQBlAHQAcgBvAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAMQAzAC4AMQAsACAAMQA0AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAQwBUAFwAIgAsACAAMQAzAC4AMQAsACAAMQA0AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgADQALgAwACwAIAA0AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIAA4AC4AOAAsACAANwAuADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgADEAMAAuADcALAAgADEAMAAuADYAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIAA0AC4AMQAsACAANAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIAA0AC4AMAAsACAANAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgADQALgAxACwAIAA0AC4AMABcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAE4AUwBXACAAYQBuAGQAIABBAEMAVAAgAHMAcABsAGkAdAAgAGkAbgB0AG8AIABzAGUAcABhAHIAYQB0AGUAIAByAG8AdwBzAC4AIABcAHUAMAAwADIANwBDAFwAdQAwADAAMgA3ACAAVgBhAGwAdQBlAHMAIABmAG8AcgAgAFQAYQBzAG0AYQBuAGkAYQAgAGEAbgBkACAATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAIAByAGUAcABsAGEAYwBlAGQAIAB3AGkAdABoACAAdABoAG8AcwBlACAAZgBvAHIAIABWAGkAYwB0AG8AcgBpAGEAIABhAG4AZAAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAHIAZQBzAHAAZQBjAHQAaQB2AGUAbAB5AC4AIAAoAFMAZQBlACAAYQBwAHAAZQBuAGQAaQBjAGUAcwApAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMgAsACAAMgAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAEEAcwAgAFMAYwBvAHAAZQAgADMAIABmAGEAYwB0AG8AcgBzACAAYQByAGUAIABjAGEAbABjAHUAbABhAHQAZQBkACAAYQB0ACAAdABoAGUAIABwAG8AaQBuAHQAIAB3AGgAZQByAGUAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAIABpAHMAIABkAGUAbABpAHYAZQByAGUAZAAgAHQAbwAgAGUAbgBkACAAdQBzAGUAcgBzACwAIABpAHQAIABpAHMAIABuAGUAYwBlAHMAcwBhAHIAeQAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAYQB0ACAAZQBhAGMAaAAgAG8AZgAgAHQAaABlACAAbABvAGEAZAAgAGMAZQBuAHQAcgBlAHMALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBHAGEAcwAgAHIAZQBhAGMAaABlAHMAIABlAG4AZAAgAHUAcwBlAHIAcwAgAGUAaQB0AGgAZQByACAAZgByAG8AbQAgAHQAaABlACAAbQBlAHQAcgBvACAAZABpAHMAdAByAGkAYgB1AHQAaQBvAG4AIABuAGUAdAB3AG8AcgBrAHMAIABvAHIAIABkAGkAcgBlAGMAdAAgAGYAcgBvAG0AIAB0AGgAZQAgAGgAaQBnAGgAIAAtACAAcAByAGUAcwBzAHUAcgBlACAAZABpAHMAdAByAGkAYgB1AHQAaQBvAG4AIABwAGkAcABlAGwAaQBuAGUAcwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAEgAbwB1AHMAZQBoAG8AbABkAHMAIABhAG4AZAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB1AHMAZQByAHMAIAB0AGUAbgBkACAAdABvACAAYgBlACAAcwBlAHIAdgBlAGQAIABiAHkAIAB0AGgAZQAgAGYAbwByAG0AZQByACwAIABhAG4AZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAGcAZQBuAGUAcgBhAHQAbwByAHMAIABhAG4AZAAgAGwAYQByAGcAZQAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIABwAGwAYQBuAHQAcwAgAGYAcgBvAG0AIAB0AGgAZQAgAGwAYQB0AHQAZQByAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAFwAIgBNAGUAdAByAG8AIABpAHMAIABkAGUAZgBpAG4AZQBkACAAYQBzACAAbABvAGMAYQB0AGUAZAAgAG8AbgAgAG8AcgAgAGUAYQBzAHQAIABvAGYAIAB0AGgAZQAgAGQAaQB2AGkAZABpAG4AZwAgAHIAYQBuAGcAZQAgAGkAbgAgAE4AUwBXACwAIABpAG4AYwBsAHUAZABpAG4AZwAgAEMAYQBuAGIAZQByAHIAYQAgAGEAbgBkACAAUQB1AGUAYQBuAGIAZQB5AGEAbgAsACAATQBlAGwAYgBvAHUAcgBuAGUALAAgAEIAcgBpAHMAYgBhAG4AZQAsACAAQQBkAGUAbABhAGkAZABlACAAbwByACAAUABlAHIAdABoAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIATwB0AGgAZQByAHcAaQBzAGUALAAgAHQAaABlACAAbgBvAG4AIAAtACAAbQBlAHQAcgBvACAAZgBhAGMAdABvAHIAIABzAGgAbwB1AGwAZAAgAGIAZQAgAHUAcwBlAGQALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAEYAYQBjAHQAbwByAHMAIABhAHIAZQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAG8AcgAgAGEAbABsACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzACAAZABpAHMAdAByAGkAYgB1AHQAZQBkACAAaQBuACAAYQAgAHAAaQBwAGUAbABpAG4AZQAgAHcAaABpAGMAaAAgAG0AYQB5ACAAaQBuAGMAbAB1AGQAZQAgAGMAbwBhAGwAIABzAGUAYQBtACAAbQBlAHQAaABhAG4AZQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC0AXAAiACwAIABcACIAVABhAGIAbABlACAANgAgAGkAcwAgAG4AbwB0ACAAYQBwAHAAbABpAGMAYQBiAGwAZQAgAHQAbwAgAGUAdABoAGEAbgBlAC4AIABTAGUAZQAgAFQAYQBiAGwAZQAgADcAIABJAG4AZABpAHIAZQBjAHQAIAAoAFMAYwBvAHAAZQAgADMAKQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAZQB0AGgAYQBuAGUALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAEMAIAA9ACAAQwBvAG4AZgBpAGQAZQBuAHQAaQBhAGwALgAgAFMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABUAGEAcwBtAGEAbgBpAGEAIABhAG4AZAAgAHQAaABlACAATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAIABhAHIAZQAgAG4AbwB0ACAAYQB2AGEAaQBsAGEAYgBsAGUAIABkAHUAZQAgAHQAbwAgAGMAbwBuAGYAaQBkAGUAbgB0AGkAYQBsAGkAdAB5ACAAYwBvAG4AcwB0AHIAYQBpAG4AdABzACAAdABoAGEAdAAgAGEAcgBpAHMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBmAHIAbwBtACAAdABoAGUAIAB1AHMAZQAgAG8AZgAgAGEAIABsAGkAbQBpAHQAZQBkACAAbgB1AG0AYgBlAHIAIABvAGYAIABOAEcARQBSACAAZABhAHQAYQAgAGkAbgBwAHUAdABzAC4AIABJAHQAIABpAHMAIABzAHUAZwBnAGUAcwB0AGUAZAAgAHQAaABhAHQAIABmAG8AcgAgAFQAYQBzAG0AYQBuAGkAYQAgAHQAaABlACAAdQBzAGUAIABvAGYAIAB0AGgAZQAgAFYAaQBjAHQAbwByAGkAYQBuACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGkAcwAgAGEAcABwAHIAbwBwAHIAaQBhAHQAZQAsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAHcAaABpAGwAZQAgAGYAbwByACAATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAIAB0AGgAZQAgAHUAcwBlACAAbwBmACAAdABoAGUAIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABpAHMAIABhAHAAcAByAG8AcAByAGkAYQB0AGUALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZABvACAAbgBvAHQAIABpAG4AYwBsAHUAZABlACAAZgB1AGcAaQB0AGkAdgBlACAAZQBtAGkAcwBzAGkAbwBuACAAbABlAGEAawBhAGcAZQAgAGYAcgBvAG0AIABsAG8AdwAgAHAAcgBlAHMAcwB1AHIAZQAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAgAGQAaQBzAHQAcgBpAGIAdQB0AGkAbwBuACAAcABpAHAAZQBsAGkAbgBlACAAbgBlAHQAdwBvAHIAawBzACAAdwBoAGkAbABlACAAdABoAG8AcwBlACAAZgByAG8AbQAgAGgAaQBnAGgAIABwAHIAZQBzAHMAdQByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAZwBhAHMAIABuAGUAdAB3AG8AcgBrAHMAIABhAHIAZQAgAGMAbwBuAHMAaQBkAGUAcgBlAGQAIABuAGUAZwBsAGkAZwBpAGIAbABlAC4AXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBGAHUAZQBsACAAcwBjAG8AcABlACAAMQAgAGEAbgBkACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAUwB0AGEAdABpAG8AbgBhAHIAeQAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAYQBuAGQAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABTAHQAYQB0AGkAbwBuAGEAcgB5ACAAbABpAHEAdQBpAGQAIABmAHUAZQBsAHMAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBEAGkAcgBlAGMAdAAgACgAUwBjAG8AcABlACAAMQApACAAYQBuAGQAIABpAG4AZABpAHIAZQBjAHQAIAAoAHMAYwBvAHAAZQAgADMAKQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAbABpAHEAdQBpAGQAIABmAHUAZQBsAHMALAAgAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBlAHIAdABhAGkAbgAgAHAAZQB0AHIAbwBsAGUAdQBtACAAYgBhAHMAZQBkACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMALgBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAA4AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyADUALAAgADgALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIARgB1AGUAbAAgAGMAbwBtAGIAdQBzAHQAZQBkAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAQwBvAG4AdABlAG4AdAAgAEYAYQBjAHQAbwByACAAKABHAEoAIABwAGUAcgAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsACkAXAAiACwAIABcACIARgB1AGUAbAAgAHUAbgBpAHQAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBPADIAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBIADQAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAATgAyAE8AXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBvAG0AYgBpAG4AZQBkACAAZwBhAHMAZQBzAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAdAByAG8AbABlAHUAbQAgAGIAYQBzAGUAZAAgAG8AaQBsAHMAIAAoAG8AdABoAGUAcgAgAHQAaABhAG4AIABwAGUAdAByAG8AbABlAHUAbQAgAGIAYQBzAGUAZAAgAG8AaQBsACAAdQBzAGUAZAAgAGEAcwAgAGYAdQBlAGwAKQAsACAAZQAuAGcALgAgAGwAdQBiAHIAaQBjAGEAbgB0AHMAXAAiACwAIAAzADgALgA4ACwAIABcACIAawBsAFwAIgAsACAAMQAzAC4AOQAsACAAMAAuADAALAAgADAALgAwACwAIAAxADMALgA5ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABlAHQAcgBvAGwAZQB1AG0AIABiAGEAcwBlAGQAIABnAHIAZQBhAHMAZQBzAFwAIgAsACAAMwA4AC4AOAAsACAAXAAiAGsAbABcACIALAAgADMALgA1ACwAIAAwAC4AMAAsACAAMAAuADAALAAgADMALgA1ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwByAHUAZABlACAAbwBpAGwAIABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgB1AGQAZQAgAG8AaQBsACAAYwBvAG4AZABlAG4AcwBhAHQAZQBzAFwAIgAsACAANAA1AC4AMwAsACAAXAAiAHQAXAAiACwAIAA2ADkALgA2ACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAANgA5AC4AOAA4ACwAIABcACIATgBFAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAgAGwAaQBxAHUAaQBkAHMAXAAiACwAIAA0ADYALgA1ACwAIABcACIAdABcACIALAAgADYAMQAuADAALAAgADAALgAwADgALAAgADAALgAyACwAIAA2ADEALgAyADgALAAgAFwAIgBOAEUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQB1AHQAbwBtAG8AdABpAHYAZQAgAGcAYQBzAG8AbABpAG4AZQAgAC8AIABwAGUAdAByAG8AbAAgACgAbwB0AGgAZQByACAAdABoAGEAbgAgAGYAbwByACAAdQBzAGUAIABhAHMAIABmAHUAZQBsACAAaQBuACAAYQBuACAAYQBpAHIAYwByAGEAZgB0ACkAXAAiACwAIAAzADQALgAyACwAIABcACIAawBMAFwAIgAsACAANgA3AC4ANAAsACAAMAAuADIALAAgADAALgAyACwAIAA2ADcALgA4ADAALAAgADEANwAuADIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAHYAaQBhAHQAaQBvAG4AIABnAGEAcwBvAGwAaQBuAGUAXAAiACwAIAAzADMALgAxACwAIABcACIAawBMAFwAIgAsACAANgA3ACwAIAAwAC4AMgAsACAAMAAuADIALAAgADYANwAuADQAMAAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEsAZQByAG8AcwBlAG4AZQAgACgAbwB0AGgAZQByACAAdABoAGEAbgAgAGYAbwByACAAdQBzAGUAIABhAHMAIABmAHUAZQBsACAAaQBuACAAYQBuACAAYQBpAHIAYwByAGEAZgB0ACkAXAAiACwAIAAzADcALgA1ACwAIABcACIAawBMAFwAIgAsACAANgA4AC4AOQAsACAAMAAuADAAMQAsACAAMAAuADIALAAgADYAOQAuADEAMQAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAdgBpAGEAdABpAG8AbgAgAHQAdQByAGIAaQBuAGUAIABmAHUAZQBsACAALwAgAGsAZQByAG8AcwBlAG4AZQBcACIALAAgADMANgAuADgALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA2ACwAIAAwAC4AMAAyACwAIAAwAC4AMgAsACAANgA5AC4AOAAyACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdABpAG4AZwAgAG8AaQBsAFwAIgAsACAAMwA3AC4AMwAsACAAXAAiAGsATABcACIALAAgADYAOQAuADUALAAgADAALgAwADMALAAgADAALgAyACwAIAA2ADkALgA3ADMALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAZQBzAGUAbAAgAG8AaQBsAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsATABcACIALAAgADYAOQAuADkALAAgADAALgAxACwAIAAwAC4AMgAsACAANwAwAC4AMgAwACwAIAAxADcALgAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIARgB1AGUAbAAgAG8AaQBsAFwAIgAsACAAMwA5AC4ANwAsACAAXAAiAGsATABcACIALAAgADcAMwAuADYALAAgADAALgAwADQALAAgADAALgAyACwAIAA3ADMALgA4ADQALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGkAcQB1AGUAZgBpAGUAZAAgAGEAcgBvAG0AYQB0AGkAYwAgAGgAeQBkAHIAbwBjAGEAcgBiAG8AbgBzAFwAIgAsACAAMwA0AC4ANAAsACAAXAAiAGsATABcACIALAAgADYAOQAuADcALAAgADAALgAwADMALAAgADAALgAyACwAIAA2ADkALgA5ADMALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AbAB2AGUAbgB0AHMAOgAgAG0AaQBuAGUAcgBhAGwAIAB0AHUAcgBwAGUAbgB0AGkAbgBlACAAbwByACAAdwBoAGkAdABlACAAcwBwAGkAcgBpAHQAcwBcACIALAAgADMANAAuADQALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA3ACwAIAAwAC4AMAAzACwAIAAwAC4AMgAsACAANgA5AC4AOQAzACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABwAGUAdAByAG8AbABlAHUAbQAgAGcAYQBzACAAKABMAFAARwApAFwAIgAsACAAMgA1AC4ANwAsACAAXAAiAGsATABcACIALAAgADYAMAAuADIALAAgADAALgAyACwAIAAwAC4AMgAsACAANgAwAC4ANgAwACwAIAAyADAALgAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBhAHAAaAB0AGgAYQBcACIALAAgADMAMQAuADQALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAA2ADkALgA4ADIALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAdAByAG8AbABlAHUAbQAgAGMAbwBrAGUAXAAiACwAIAAzADQALgAyACwAIABcACIAdABcACIALAAgADkAMgAuADYALAAgADAALgAwADgALAAgADAALgAyACwAIAA5ADIALgA4ADgALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAZgBpAG4AZQByAHkAIABnAGEAcwAgAGEAbgBkACAAbABpAHEAdQBpAGQAcwBcACIALAAgADQAMgAuADkALAAgAFwAIgB0AFwAIgAsACAANQA0AC4ANwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAANQA0AC4ANwA2ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgBlAGYAaQBuAGUAcgB5ACAAYwBvAGsAZQBcACIALAAgADMANAAuADIALAAgAFwAIgB0AFwAIgAsACAAOQAyAC4ANgAsACAAMAAuADAAOAAsACAAMAAuADIALAAgADkAMgAuADgAOAAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAAZQB0AHIAbwBsAGUAdQBtACAAYgBhAHMAZQBkACAAcAByAG8AZAB1AGMAdABzACAAbwB0AGgAZQByACAAdABoAGEAbgAgAG0AZQBuAHQAaQBvAG4AZQBkACAAaQBuACAAdABoAGUAIABpAHQAZQBtAHMAIABhAGIAbwB2AGUAXAAiACwAIAAzADQALgA0ACwAIABcACIAawBMAFwAIgAsACAANgA5AC4AOAAsACAAMAAuADAAMgAsACAAMAAuADEALAAgADYAOQAuADkAMgAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEIAaQBvAGQAaQBlAHMAZQBsAFwAIgAsACAAMwA0AC4ANgAsACAAXAAiAGsATABcACIALAAgADAALgAwACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAAMAAuADIAOAAsACAAXAAiAE4ARQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBFAHQAaABhAG4AbwBsACAAZgBvAHIAIAB1AHMAZQAgAGEAcwAgAGEAIABmAHUAZQBsACAAaQBuACAAYQBuACAAaQBuAHQAZQByAG4AYQBsACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAGUAbgBnAGkAbgBlAFwAIgAsACAAMgAzAC4ANAAsACAAXAAiAGsATABcACIALAAgADAALgAwACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAAMAAuADIAOAAsACAAXAAiAE4ARQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBCAGkAbwBmAHUAZQBsAHMAIABvAHQAaABlAHIAIAB0AGgAYQBuACAAdABoAG8AcwBlACAAbQBlAG4AdABpAG8AbgBlAGQAIABpAG4AIAB0AGgAZQAgAGkAdABlAG0AcwAgAGEAYgBvAHYAZQAgAGEAbgBkACAAYgBlAGwAbwB3AFwAIgAsACAAMgAzAC4ANAAsACAAXAAiAGsATABcACIALAAgADAALgAwACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAAMAAuADIAOAAsACAAXAAiAE4ARQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAGEAdgBpAGEAdABpAG8AbgAgAGsAZQByAG8AcwBlAG4AZQBcACIALAAgADMANgAuADgALAAgAFwAIgBrAEwAXAAiACwAIAAwAC4AMAAsACAAMAAuADAAMgAsACAAMAAuADIALAAgADAALgAyADIALAAgAFwAIgBOAEUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABkAGkAZQBzAGUAbABcACIALAAgADMAOAAuADYALAAgAFwAIgBrAEwAXAAiACwAIAAwAC4AMAAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMwAwACwAIABcACIATgBFAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAXAB1ADAAMAAyADcATgBFAFwAdQAwADAAMgA3ACAAdgBhAGwAdQBlAHMAIAByAGUAdAB1AHIAbgBlAGQAIABhAHMAIAB6AGUAcgBvACAAZgBvAHIAIABjAGEAbABjAHUAbABhAHQAaQBvAG4AcwAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAYQBuAGQAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABUAHIAYQBuAHMAcABvAHIAdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABhAG4AZAAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFQAcgBhAG4AcwBwAG8AcgB0AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEQAaQByAGUAYwB0ACAAKABzAGMAbwBwAGUAIAAxACkAIABhAG4AZAAgAGkAbgBkAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMwApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGYAdQBlAGwAcwAgAGkAbgAgAGQAaQBmAGYAZQByAGUAbgB0ACAAdAByAGEAbgBzAHAAbwByAHQAIABlAHEAdQBpAHAAbQBlAG4AdABcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAQQBjAGMAbwB1AG4AdABzACAARgBhAGMAdABvAHIAcwAgADIAMAAyADUAIAAtACAAVABhAGIAbABlACAAOQBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIANgAsACAAMQAwACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBhAG4AcwBwAG8AcgB0ACAAdAB5AHAAZQBcACIALAAgAFwAIgBGAHUAZQBsACAAYwBvAG0AYgB1AHMAdABlAGQAXAAiACwAIABcACIARQBuAGUAcgBnAHkAIABDAG8AbgB0AGUAbgB0ACAARgBhAGMAdABvAHIAKABHAEoAIABwAGUAcgAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsACkAXAAiACwAIABcACIARgB1AGUAbAAgAHUAbgBpAHQAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBPADIAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBIADQAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAATgAyAE8AXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBvAG0AYgBpAG4AZQBkACAAZwBhAHMAZQBzAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQBcACIALAAgAFwAIgBTAG8AdQByAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBzACAAYQBuAGQAIABsAGkAZwBoAHQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEcAYQBzAG8AbABpAG4AZQBcACIALAAgADMANAAuADIALAAgAFwAIgBrAGwAXAAiACwAIAA2ADcALgA0ACwAIAAwAC4AMAAyACwAIAAwAC4AMgAsACAANgA3AC4ANgAyACwAIAAxADcALgAyACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBEAGkAZQBzAGUAbAAgAG8AaQBsAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADYAOQAuADkALAAgADAALgAwADEALAAgADAALgA1ACwAIAA3ADAALgA0ADEALAAgADEANwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBzACAAYQBuAGQAIABsAGkAZwBoAHQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAZQBmAGkAZQBkACAAcABlAHQAcgBvAGwAZQB1AG0AIABnAGEAcwAgACgATABQAEcAKQBcACIALAAgADIANgAuADIALAAgAFwAIgBrAGwAXAAiACwAIAA2ADAALgAyACwAIAAwAC4ANQAsACAAMAAuADMALAAgADYAMQAuADAAMAAsACAAMgAwAC4AMgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAHMAIABhAG4AZAAgAGwAaQBnAGgAdAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIARgB1AGUAbAAgAG8AaQBsAFwAIgAsACAAMwA5AC4ANwAsACAAXAAiAGsAbABcACIALAAgADcAMwAuADYALAAgADAALgAwADgALAAgADAALgA1ACwAIAA3ADQALgAxADgALAAgADEAOAAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBzACAAYQBuAGQAIABsAGkAZwBoAHQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEUAdABoAGEAbgBvAGwAXAAiACwAIAAyADMALgA0ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgAyACwAIAAwAC4AMgAsACAAMAAuADQALAAgAFwAIgBOAEUAXAAiACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBCAGkAbwBkAGkAZQBzAGUAbABcACIALAAgADMANAAuADYALAAgAFwAIgBrAGwAXAAiACwAIAAwAC4AMAAsACAAMAAuADgALAAgADEALgA3ACwAIAAyAC4ANQAsACAAXAAiAE4ARQBcACIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBzACAAYQBuAGQAIABsAGkAZwBoAHQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAFIAZQBuAGUAdwBhAGIAbABlACAAZABpAGUAcwBlAGwAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgAwADEALAAgADAALgA1ACwAIAAwAC4ANQAxACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAHMAIABhAG4AZAAgAGwAaQBnAGgAdAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIATwB0AGgAZQByACAAYgBpAG8AZgB1AGUAbABzAFwAIgAsACAAMgAzAC4ANAAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AOAAsACAAMQAuADcALAAgADIALgA1ACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAaQBnAGgAdAAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIAQwBvAG0AcAByAGUAcwBzAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwBcACIALAAgADAALgAwADMAOQAzACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4ANAAsACAANwAuADMALAAgADAALgAzACwAIAA1ADkALgAwACwAIAAxADgALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABpAGcAaAB0ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBMAGkAcQB1AGUAZgBpAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwBcACIALAAgADIANQAuADMALAAgAFwAIgBrAGwAXAAiACwAIAA1ADEALgA0ACwAIAA3AC4AMwAsACAAMAAuADMALAAgADUAOQAuADAALAAgADEAOAAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAYQB2AHkAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEMAbwBtAHAAcgBlAHMAcwBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAXAAiACwAIAAwAC4AMAAzADkAMwAsACAAXAAiAG0AMwBcACIALAAgADUAMQAuADQALAAgADIALgA4ACwAIAAwAC4AMwAsACAANQA0AC4ANQAsACAAMQA4AC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAXAAiACwAIAAyADUALgAzACwAIABcACIAawBsAFwAIgAsACAANQAxAC4ANAAsACAAMgAuADgALAAgADAALgAzACwAIAA1ADQALgA1ACwAIAAxADgALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBEAGkAZQBzAGUAbAAgAG8AaQBsACAALQAgAEUAdQByAG8AIABpAHYAIABvAHIAIABoAGkAZwBoAGUAcgBcACIALAAgADMAOAAuADYALAAgAFwAIgBrAGwAXAAiACwAIAA2ADkALgA5ACwAIAAwAC4AMAA3ACwAIAAwAC4ANAAsACAANwAwAC4AMwA3ACwAIAAxADcALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBEAGkAZQBzAGUAbAAgAG8AaQBsACAALQAgAEUAdQByAG8AIABpAGkAaQBcACIALAAgADMAOAAuADYALAAgAFwAIgBrAGwAXAAiACwAIAA2ADkALgA5ACwAIAAwAC4AMQAsACAAMAAuADQALAAgADcAMAAuADQALAAgADEANwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAYQB2AHkAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsACAAbwBpAGwAIAAtACAARQB1AHIAbwAgAGkAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAANgA5AC4AOQAsACAAMAAuADIALAAgADAALgA0ACwAIAA3ADAALgA1ACwAIAAxADcALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAGQAaQBlAHMAZQBsACAAEyAgAEUAdQByAG8AIABpAHYAIABvAHIAIABoAGkAZwBoAGUAcgBcACIALAAgADMAOAAuADYALAAgAFwAIgBrAGwAXAAiACwAIAAwAC4AMAAsACAAMAAuADAANwAsACAAMAAuADQALAAgADAALgA0ADcALAAgAFwAIgBOAEUAXAAiACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAGQAaQBlAHMAZQBsACAAEyAgAEUAdQByAG8AIABpAGkAaQBcACIALAAgADMAOAAuADYALAAgAFwAIgBrAGwAXAAiACwAIAAwAC4AMAAsACAAMAAuADEALAAgADAALgA0ACwAIAAwAC4ANQAsACAAXAAiAE4ARQBcACIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAYQB2AHkAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAFIAZQBuAGUAdwBhAGIAbABlACAAZABpAGUAcwBlAGwAIAATICAARQB1AHIAbwAgAGkAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgAyACwAIAAwAC4ANAAsACAAMAAuADYALAAgAFwAIgBOAEUAXAAiACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQB2AGkAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEcAYQBzAG8AbABpAG4AZQAgAGYAbwByACAAdQBzAGUAIABhAHMAIABmAHUAZQBsACAAaQBuACAAYQBuACAAYQBpAHIAYwByAGEAZgB0AFwAIgAsACAAMwAzAC4AMQAsACAAXAAiAGsAbABcACIALAAgADYANwAuADAALAAgADAALgAwADYALAAgADAALgA2ACwAIAA2ADcALgA2ADYALAAgADEAOAAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAHYAaQBhAHQAaQBvAG4AXAAiACwAIABcACIASwBlAHIAbwBzAGUAbgBlACAAZgBvAHIAIAB1AHMAZQAgAGEAcwAgAGYAdQBlAGwAIABpAG4AIABhAG4AIABhAGkAcgBjAHIAYQBmAHQAXAAiACwAIAAzADYALgA4ACwAIABcACIAawBsAFwAIgAsACAANgA5AC4ANgAsACAAMAAuADAAMQAsACAAMAAuADYALAAgADcAMAAuADIAMQAsACAAMQA4AC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAdgBpAGEAdABpAG8AbgBcACIALAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAGEAdgBpAGEAdABpAG8AbgAgAGsAZQByAG8AcwBlAG4AZQBcACIALAAgADMANgAuADgALAAgAFwAIgBrAGwAXAAiACwAIAAwAC4AMAAsACAAMAAuADAAMQAsACAAMAAuADYALAAgADAALgA2ADEALAAgAFwAIgBOAEUAXAAiACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBlAHMAcwBlAGwAcwBcACIALAAgAFwAIgBHAGEAcwBvAGwAaQBuAGUAXAAiACwAIAAzADQALgAyACwAIABcACIAawBMAFwAIgAsACAANgA3AC4ANAAsACAAMQAwAC4AMQAsACAAMAAuADMALAAgAFwAIgBcACIALAAgADEANwAuADIALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADIALgAxAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAZQBzAHMAZQBsAHMAXAAiACwAIABcACIARABpAGUAcwBlAGwAIABvAGkAbABcACIALAAgADMAOAAuADYALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA5ACwAIAAwAC4AMgAsACAAMAAuADUALAAgAFwAIgBcACIALAAgADEANwAuADMALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADIALgAxAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAZQBzAHMAZQBsAHMAXAAiACwAIABcACIARgB1AGUAbAAgAE8AaQBsAFwAIgAsACAAMwA5AC4ANwAsACAAXAAiAGsATABcACIALAAgADcAMwAuADYALAAgADAALgAyACwAIAAwAC4ANQAsACAAXAAiAFwAIgAsACAAMQA4AC4AMAAsACAAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMgAuADEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATwBmAGYALQByAG8AYQBkACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACAAYQBuAGQAIABmAG8AcgBlAHMAdAByAHkAIABlAHEAdQBpAHAAbQBlAG4AdABcACIALAAgAFwAIgBEAGkAZQBzAGUAbAAgAG8AaQBsAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsATABcACIALAAgADYAOQAuADkALAAgADAALgAzACwAIAAwAC4ANQAsACAAXAAiAFwAIgAsACAAMQA3AC4AMwAsACAAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMgAuADEAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAXAB1ADAAMAAyADcATgBFAFwAdQAwADAAMgA3ACAAdgBhAGwAdQBlAHMAIAByAGUAdAB1AHIAbgBlAGQAIABhAHMAIAB6AGUAcgBvACAAZgBvAHIAIABjAGEAbABjAHUAbABhAHQAaQBvAG4AcwAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBGAHUAZQBsACAAcwBjAG8AcABlACAAMQAgAGEAbgBkACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAATwBmAGYALQByAGEAZAAgAGUAcQB1AGkAcABtAGUAbgB0ACAAYQBuAGQAIAB2AGUAcwBzAGUAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAYQBuAGQAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABPAGYAZgAtAHIAbwBhAGQAIABlAHEAdQBpAHAAbQBlAG4AdAAgAGEAbgBkACAAdgBlAHMAcwBlAGwAcwBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEQAaQByAGUAYwB0ACAAKABzAGMAbwBwAGUAIAAxACkAIABhAG4AZAAgAGkAbgBkAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMwApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIABmAHUAZQBsAHMAIABpAG4AIABvAGYAZgAtAHIAbwBhAGQAIABlAHEAdQBpAHAAbQBlAG4AdAAgAGEAbgBkACAAdgBlAHMAcwBlAGwAcwBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAyAC4AMQBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAANwAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAYQBuAHMAcABvAHIAdAAgAHQAeQBwAGUAIAB0AFwAIgAsACAAXAAiAEYAdQBlAGwAIAB0AHkAcABlACAAcQBcACIALAAgAFwAIgBFAEMAVAByAGEAbgBzACwAcQAgACgARwBKAC8AawBMACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEMATwAyACAARQBGAFQAcgBhAG4ALAAxACwAdABxAGcAIAAoAGsAZwAgAEMATwAyAC0AZQAvAEcASgApAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABDAEgANAAgAEUARgBUAHIAYQBuACwAMQAsAHQAZwBnACAAKABrAGcAIABDAE8AMgAtAGUALwBHAEoAKQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAATgAyAE8AIABFAEYAVAByAGEAbgAsADEALAB0AGcAZwAgACgAawBnACAAQwBPADIALQBlAC8ARwBKACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMwAgAEUARgBUAHIAYQBuAHMALAAzACwAcQAgACgAawBnACAAQwBPADIALQBlAC8ARwBKACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBlAHMAcwBlAGwAXAAiACwAIABcACIAUABlAHQAcgBvAGwAXAAiACwAIAAzADQALgAyACwAIAA2ADcALgA0ACwAIAAxADAALgAxACwAIAAwAC4AMwAsACAAMQA3AC4AMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAZQBzAHMAZQBsAFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsAFwAIgAsACAAMwA4AC4ANgAsACAANgA5AC4AOQAsACAAMAAuADIALAAgADAALgA1ACwAIAAxADcALgAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBlAHMAcwBlAGwAXAAiACwAIABcACIARgB1AGUAbAAgAE8AaQBsAFwAIgAsACAAMwA5AC4ANwAsACAANwAzAC4ANgAsACAAMAAuADIALAAgADAALgA1ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIATwBmAGYALQByAG8AYQBkACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACAAYQBuAGQAIABmAG8AcgBlAHMAdAByAHkAIABlAHEAdQBpAHAAbQBlAG4AdABcACIALAAgAFwAIgBEAGkAZQBzAGUAbABcACIALAAgADMAOAAuADYALAAgADYAOQAuADkALAAgADAALgAzACwAIAAwAC4ANQAsACAAMQA3AC4AMwBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEYAdQBlAGwAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBGAHUAZQBsAF8ARwBlAHQAVAByAGEAbgBzAHAAbwByAHQARgB1AGUAbABTAHQAcgBpAG4AZwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALABcAG4AIAAgACAAIABMAEUARgBUACgAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsACAAXAAiACwAQwBlAGwAbAApACAALQAxACkAXABuACkAOwBcAG4AXABuAEYAdQBlAGwAXwBHAGUAdABTAHQAYQB0AGkAbwBuAGEAcgB5AEYAdQBlAGwAUwB0AHIAaQBuAGcAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAXABuACAAIAAgACAAUgBJAEcASABUACgAQwBlAGwAbAAsAEwARQBOACgAQwBlAGwAbAApAC0ARgBJAE4ARAAoAFwAIgAsACAAXAAiACwAQwBlAGwAbAApACkAXABuACkAOwBcAG4AXABuAEYAdQBlAGwAXwBUAG8AdABhAGwAQwBvAG4AcwB1AG0AcAB0AGkAbwBuAFwAbgA9ACAATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABGAHUAZQBsAEMAbwBuAHMAdQBtAHAAdABpAG8AbgBBAHIAcgBhAHkALAAgAEYAdQBlAGwAVQBzAGUAQQByAHIAYQB5ACwAIABGAHUAZQBsAFUAcwBlACwAIABGAHUAZQBsAFQAeQBwAGUAQQByAHIAYQB5ACwAIABGAHUAZQBsAFQAeQBwAGUALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAUwBVAE0AKABcAG4AIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAEYAdQBlAGwAQwBvAG4AcwB1AG0AcAB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAKABGAHUAZQBsAFQAeQBwAGUAQQByAHIAYQB5ACAAPQAgAEYAdQBlAGwAVAB5AHAAZQApACAAKgAgAFwAbgAgACAAIAAgACAAIAAgACAAKABGAHUAZQBsAFUAcwBlAEEAcgByAGEAeQAgAD0AIABGAHUAZQBsAFUAcwBlACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQAsAFwAbgAgACAAIAAgADAAXABuACAAIAApAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AOAA6ACAARgB1AGUAbAAgAFUAcwBlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADgALgAxACAARgB1AGUAbAAgAFUAcwBlACAALQAgAFQAcgBhAG4AcwBwAG8AcgB0ACAAZgB1AGUAbABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRACwAIABFAEMALAAgAEUARgAsAFwAbgAgACAAIAAgACgAUQAgACoAIABFAEMAIAAqACAARQBGACkAIAAqACAAMQAwACAAXgAgAC0AIAAzAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBmACAAZgB1AGUAbABzACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzAFwAbgBRACAAOgAgAEEAbQBvAHUAbgB0ACAAbwBmACAAZgB1AGUAbAAgAHQAeQBwAGUAIABxACAAYwBvAG0AYgB1AHMAdABlAGQAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAIAA6ACAAawBMAFwAbgBFAEMAIAA6ACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAIAA6ACAARwBKAC8AawBMAFwAbgBFAEYAIAA6ACAAUwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzACAAZgBvAHIAIABlAGEAYwBoACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAOgAgAGsAZwAgAEMATwAyAGUAIAAvACAARwBKAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwBUAHIAYQBuAHMAdABxACwAIABFAEMAXwBUAHIAYQBuAHMAcQAsACAARQBGAF8AVAByAGEAbgBzADEAdABxAGcALABcAG4AIAAgACAAIABWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACgAUQBfAFQAcgBhAG4AcwB0AHEALAAgAEUAQwBfAFQAcgBhAG4AcwBxACwAIABFAEYAXwBUAHIAYQBuAHMAMQB0AHEAZwApAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBmACAAZgB1AGUAbABzACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgAtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAOAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIAAyAC4AMwAgAEUAcwB0AGkAbQBhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB0AHIAYQBuAHMAcABvAHIAdAAgAGYAdQBlAGwAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBnAD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB0ACAAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBxAFwAXABsAGUAZgB0ACgAUQBfAHsAVAByAGEAbgBzACwAdABxAH0AXABcAHQAaQBtAGUAcwAgAEUAQwBfAHsAVAByAGEAbgBzACwAcQB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFQAcgBhAG4AcwAsADEALAB0AHEAZwB9AFwAXAByAGkAZwBoAHQAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAFQAcgBhAG4AcwB0AHEAXAAiACwAIABcACIAQQBtAG8AdQBuAHQAIABvAGYAIABmAHUAZQBsACAAdAB5AHAAZQAgAHEAIABjAG8AbQBiAHUAcwB0AGUAZAAgAGYAbwByACAAdAByAGEAbgBzAHAAbwByAHQAIABlAG4AZQByAGcAeQAgAHAAdQByAHAAbwBzAGUAcwBcACIALAAgAFwAIgBWAGEAcgBpAGUAcwAgAGIAYQBzAGUAZAAgAG8AbgAgAGYAdQBlAGwAIAB0AHkAcABlADoAIABrAEwALAAgAG0AMwAsACAARwBKAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAF8AVAByAGEAbgBzAHEAXAAiACwAIABcACIARQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAXAAiACwAIABcACIARwBKACAALwAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AVAByAGEAbgBzADEAdABxAGcAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzACAAZgBvAHIAIABlAGEAYwBoACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAGsAZwAgAEMATwAyAGUAIAAvACAARwBKAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcQBcACIALAAgAFwAIgBGAHUAZQBsACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBhAG4AcwBcACIALAAgAFwAIgBUAHIAYQBuAHMAcABvAHIAdAAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AZgAgAGYAdQBlAGwAcwBcAG4AUQAgADoAIABBAG0AbwB1AG4AdAAgAG8AZgAgAGYAdQBlAGwAIAB0AHkAcABlACAAcQAgAHUAcwBlAGQAIABmAG8AcgAgAHMAdABhAHQAaQBvAG4AYQByAHkAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBwAGUAcgBhAHQAaQBvAG4AcwAgADoAIABrAEwAXABuAEUAQwAgADoAIABFAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABvAHAAZQByAGEAdABpAG8AbgBzACAAOgAgAEcASgAvAGsATABcAG4ARQBGACAAOgAgAFMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIAA6ACAAawBnACAAQwBPADIAZQAgAC8AIABHAEoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AUwBDAHEALAAgAEUAQwBfAFMAQwBxACwAIABFAEYAXwBTAEMAMQBxAGcALABcAG4AIAAgACAAIABWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACgAUQBfAFMAQwBxACwAIABFAEMAXwBTAEMAcQAsACAARQBGAF8AUwBDADEAcQBnACkAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAbwByACAAZQBhAGMAaAAgAEcASABHACAAZgByAG8AbQAgAHQAaABlACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABvAGYAIABmAHUAZQBsAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgAtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA4AC4AMgAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAQQBjAGMAbwB1AG4AdABzACAARgBhAGMAdABvAHIAcwAgADIAMAAyADUAIAAtACAAMgAuADIAIABFAHMAdABpAG0AYQB0AGkAbgBnACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGUAbgBlAHIAZwB5ACAAcwBvAHUAcgBjAGUAcwAgAC0AIABDAGEAbABjAHUAbABhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AZgAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdAAgAFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AcQBcAFwAbABlAGYAdAAoAFEAXwB7AFMAQwAsAHEAfQBcAFwAdABpAG0AZQBzACAARQBDAF8AewBTAEMALABxAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAUwBDACwAMQAsAHEAZwB9AFwAXAByAGkAZwBoAHQAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AUwBDAHEAXAAiACwAIABcACIAQQBtAG8AdQBuAHQAIABvAGYAIABmAHUAZQBsACAAdAB5AHAAZQAgAHEAIAB1AHMAZQBkACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIAVgBhAHIAaQBlAHMAIABiAGEAcwBlAGQAIABvAG4AIABmAHUAZQBsACAAdAB5AHAAZQA6ACAAawBMACwAIABtADMALAAgAEcASgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBfAFMAQwBxAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIARwBKACAALwAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AUwBDADEAcQBnAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAawBnACAAQwBPADIAZQAgAC8AIABHAEoAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBxAFwAIgAsACAAXAAiAEYAdQBlAGwAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBDAFwAIgAsACAAXAAiAFMAdABhAHQAaQBvAG4AYQByAHkAIABjAG8AbQBiAHUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAZwBcACIALAAgAFwAIgBHAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADkAOgAgAFIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAFUAcwBlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADkALgAxACAAUgBlAGYAcgBpAGcAZQByAGEAbgB0ACAAVQBzAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXABuAFQAaABlACAAdABvAHQAYQBsACAAZQBtAGkAcwBzAGkAbwBuAHMAIABvAGYAIAByAGUAZgByAGkAZwBlAHIAYQBuAHQAIABsAGUAYQBrAGkAbgBnACAAZAB1AHIAaQBuAGcAIABvAHAAZQByAGEAdABpAG8AbgAgACgAbgBvAHQAIABkAHUAcgBpAG4AZwAgAGkAbgBzAHQAYQBsAGwAYQB0AGkAbwBuACAAbwByACAAZABpAHMAcABvAHMAYQBsACkAXABuAEcAVwBQAFIAIAA6ACAARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABvAGYAIAByAGUAZgByAGkAZwBlAHIAYQBuAHQAIABSACAAOgAgAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXABuAGMAaABhAHIAZwBlAF8AUgBhACAAOgAgAEEAbQBvAHUAbgB0ACAAbwBmACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0ACAAUgAgAGMAbwBuAHQAYQBpAG4AZQBkACAAaQBuACAAYQBwAHAAbABpAGEAbgBjAGUAIABhACAAOgAgAGsAZwBcAG4AbABlAGEAawBhAGcAZQByAGEAdABlAF8AYQAgADoAIABQAHIAYwBlAG4AdABhAGcAZQAgAG8AZgAgAHQAbwB0AGEAbAAgAGMAaABhAHIAZwBlACAAbABlAGEAawBlAGQAIABmAHIAbwBtACAAYQBwAHAAbABpAGEAbgBjAGUAIABhACAAZQBhAGMAaAAgAHkAZQBhAHIAIAA6ACAAUABlAHIAYwBlAG4AdABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYwBoAGEAcgBnAGUAXwBSAGEALAAgAGwAZQBhAGsAYQBnAGUAcgBhAHQAZQBfAGEALABcAG4AIAAgACAAIAAoAGMAaABhAHIAZwBlAF8AUgBhACAAKgAgACgAbABlAGEAawBhAGcAZQByAGEAdABlAF8AYQAvADEAMAAwACkAKQAgACoAIAAxADAAIABeACAALQAgADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBHAFcAUABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AUgAsACAARwBXAFAAXwBSACwAXABuACAAIAAgACAAKAAoAEUAXwBSACAAKgAgADEAMABeADMAKQAgACoAIABHAFcAUABfAFIAKQAgACoAIAAxADAAXgAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABoAGUAIAB0AG8AdABhAGwAIABlAG0AaQBzAHMAaQBvAG4AcwAgAG8AZgAgAHIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAGwAZQBhAGsAaQBuAGcAIABkAHUAcgBpAG4AZwAgAG8AcABlAHIAYQB0AGkAbwBuACAAKABuAG8AdAAgAGQAdQByAGkAbgBnACAAaQBuAHMAdABhAGwAbABhAHQAaQBvAG4AIABvAHIAIABkAGkAcwBwAG8AcwBhAGwAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAGwAZQBhAGsAYQBnAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAQwBPADIALQBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAFIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0ACAAZwBhAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAC0AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAOQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIAAzAC4AMQAgAEUAcwB0AGkAbQBhAHQAaQBuAGcAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAcAByAG8AYwBlAHMAcwBlAHMAIABlAG0AaQBzAHMAaQBvAG4AcwAgAC0AIABSAGUAZgByAGkAZwBlAHIAYQBuAHQAIABsAGUAYQBrAGEAZwBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAFIAZQBhAGQAYQBiAGwAZQBFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGMAaABhAHIAZwBlAF8AUgBhACAAKgAgACgAbABlAGEAawBhAGcAZQByAGEAdABlAF8AYQAvADEAMAAwACkAIAAqACAAMQAwACAAXgAgAC0AIAAzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBSACAAPQAgAFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AYQAgAFwAXABsAGUAZgB0ACgAIABjAGgAYQByAGcAZQBfAHsAUgBhAH0AIABcAFwAdABpAG0AZQBzACAAXABcAGYAcgBhAGMAewBsAGUAYQBrAGEAZwBlAFwAXAAsAHIAYQB0AGUAXwBhAH0AewAxADAAMAB9ACAAXABcAHIAaQBnAGgAdAApACAAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAEMATwAyAGUAIAA9ACAAXABcAGwAZQBmAHQAKABFAF8AUgAgAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7ADMAfQAgAFwAXAByAGkAZwBoAHQAKQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAFIAIABcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGMAaABhAHIAZwBlAF8AUgBhAFwAIgAsACAAXAAiAEEAbQBvAHUAbgB0ACAAbwBmACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0ACAAUgAgAGMAbwBuAHQAYQBpAG4AZQBkACAAaQBuACAAYQBwAHAAbABpAGEAbgBjAGUAIABhAFwAIgAsACAAXAAiAGsAZwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGwAZQBhAGsAYQBnAGUAcgBhAHQAZQBfAGEAXAAiACwAIABcACIAUAByAGMAZQBuAHQAYQBnAGUAIABvAGYAIAB0AG8AdABhAGwAIABjAGgAYQByAGcAZQAgAGwAZQBhAGsAZQBkACAAZgByAG8AbQAgAGEAcABwAGwAaQBhAG4AYwBlACAAYQAgAGUAYQBjAGgAIAB5AGUAYQByAFwAIgAsACAAXAAiAFAAZQByAGMAZQBuAHQAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBhAFwAIgAsACAAXAAiAEEAcABwAGwAaQBhAG4AYwBlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAXAAiACwAIABcACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAF8AUgBcACIALAAgAFwAIgBUAG8AdABhAGwAIABlAG0AaQBzAHMAaQBvAG4AcwAgAG8AZgAgAHIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAFIAXAAiACwAIABcACIAdAAgAHIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAGcAYQBzAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAOQAuADEALgAxACAAKAAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAF8AUgBcACIALAAgAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAG8AZgAgAHIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAFIAXAAiACwAIABcACIARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABlAHEAdQBhAHQAaQBvAG4AIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0ACAAUgAgAHQAbwAgAEMATwAyAC0AZQAgAHUAcwBpAG4AZwAgAHQAaABlACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0AFwAdQAwADAAMgA3AHMAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgACgARwBXAFAAKQAuAFwAIgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEEAcABwAGUAbgBkAGkAeAAgADIAIABHAGwAbwBiAGEAbAAgAFcAYQByAG0AaQBuAGcAIABQAG8AdABlAG4AdABpAGEAbABzADoAIABUAGEAYgBsAGUAIAAyADMAIABHAGwAbwBiAGEAbAAgAFcAYQByAG0AaQBuAGcAIABQAG8AdABlAG4AdABpAGEAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABHAFcAUABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEcAbABvAGIAYQBsACAAVwBhAHIAbQBpAG4AZwAgAFAAbwB0AGUAbgB0AGkAYQBsAHMAXAAiACkAKQA7AFwAbgBcAG4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBDAGgAZQBtAGkAYwBhAGwARwBXAFAAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABHAFcAUABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABBAHAAcABlAG4AZABpAHgAIAAyACAALQAgAFQAYQBiAGwAZQAgADIAMwBcACIAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABHAFcAUABfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwA5ACwAIAA1ACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAaABlAG0AaQBjAGEAbAAgAGYAbwByAG0AdQBsAGEAXAAiACwAIABcACIARwBsAG8AYgBhAGwAIABXAGEAcgBtAGkAbgBnACAAUABvAHQAZQBuAHQAaQBhAGwAIAAoAEEAUgA1ACkAXAAiACwAIABcACIARwBhAHMAIAAtACAARgBDACAAbgBhAG0AZQBcACIALAAgAFwAIgBBAGQAaQB0AGkAbwBuAGEAbAAgAGQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAXAAiACwAIABcACIAQwBPADIAXAAiACwAIAAxACwAIABcACIAQwBPADIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATQBlAHQAaABhAG4AZQBcACIALAAgAFwAIgBDAEgANABcACIALAAgADIAOAAsACAAXAAiAEMASAA0AFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAXAAiACwAIABcACIATgAyAE8AXAAiACwAIAAyADYANQAsACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBsAHAAaAB1AHIAIABoAGUAeABhAGYAbAB1AG8AcgBpAGQAZQBcACIALAAgAFwAIgBTAEYANgBcACIALAAgADIAMwA1ADAAMAAsACAAXAAiAFMARgA2AFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgARgBDAC0AMgAzACAAKABSAC0AMgAzACkAXAAiACwAIABcACIAQwBIAEYAMwBcACIALAAgACAAMQAyADQAMAAwACwAIABcACIASABGAEMALQAyADMAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQAzADIAIAAoAFIALQAzADIAKQBcACIALAAgAFwAIgBDAEgAMgBGADIAXAAiACwAIAA2ADcANwAsACAAXAAiAEgARgBDAC0AMwAyAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgARgBDAC0ANAAxACAAKABSAC0ANAAxACkAXAAiACwAIABcACIAQwBIADMARgBcACIALAAgACAAMQAxADYALAAgAFwAIgBIAEYAQwAtADQAMQBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEYAQwAtADQAMwAtADEAMABtAGUAZQAgACgAUgAtADQAMwAxADAAbQBlAGUAKQBcACIALAAgAFwAIgBDADUASAAyAEYAMQAwAFwAIgAsACAAMQA2ADUAMAAsACAAXAAiAEgARgBDAC0ANAAzAC0AMQAwAG0AZQBlAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgARgBDAC0AMQAyADUAIAAoAFIALQAxADIANQApAFwAIgAsACAAXAAiAEMAMgBIAEYANQBcACIALAAgACAAMwAxADcAMAAsACAAXAAiAEgARgBDAC0AMQAyADUAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQAxADMANAAgACgAUgAtADEAMwA0ACkAXAAiACwAIABcACIAQwAyAEgAMgBGADQAIAAoAEMASABGADIAQwBIAEYAMgApAFwAIgAsACAAIAAxADEAMgAwACwAIABcACIASABGAEMALQAxADMANABcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEYAQwAtADEAMwA0AGEAIAAoAFIALQAxADMANABhACkAXAAiACwAIABcACIAQwAyAEgAMgBGADQAIAAoAEMASAAyAEYAQwBGADMAKQBcACIALAAgADEAMwAwADAALAAgAFwAIgBIAEYAQwAtADEAMwA0AGEAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQAxADQAMwAgACgAUgAtADEANAAzACkAXAAiACwAIABcACIAQwAyAEgAMwBGADMAIAAoAEMASABGADIAQwBIADIARgApAFwAIgAsACAAMwAyADgALAAgAFwAIgBIAEYAQwAtADEANAAzAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgARgBDAC0AMQA0ADMAYQAgACgAUgAtADEANAAzAGEAKQBcACIALAAgAFwAIgBDADIASAAzAEYAMwAgACgAQwBGADMAQwBIADMAKQBcACIALAAgADQAOAAwADAALAAgAFwAIgBIAEYAQwAtADEANAAzAGEAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQAxADUAMgBhACAAKABSAC0AMQA1ADIAYQApAFwAIgAsACAAXAAiAEMAMgBIADQARgAyACAAKABDAEgAMwBDAEgARgAyACkAXAAiACwAIAAxADMAOAAsACAAXAAiAEgARgBDAC0AMQA1ADIAYQBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEYAQwAtADIAMgA3AGUAYQAgACgAUgAtADIAMgA3AGUAYQApAFwAIgAsACAAXAAiAEMAMwBIAEYANwBcACIALAAgADMAMwA1ADAALAAgAFwAIgBIAEYAQwAtADIAMgA3AGUAYQBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEYAQwAtADIAMwA2AGYAYQAgACgAUgAtADIAMwA2AGYAYQApAFwAIgAsACAAXAAiAEMAMwBIADIARgA2AFwAIgAsACAAOAAwADYAMAAsACAAXAAiAEgARgBDAC0AMgAzADYAZgBhAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgARgBDAC0AMgA0ADUAYwBhACAAKABSAC0AMgA0ADUAYwBhACkAXAAiACwAIABcACIAQwAzAEgAMwBGADUAXAAiACwAIAA3ADEANgAsACAAXAAiAEgARgBDAC0AMgA0ADUAYwBhAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgARgBDAC0AMgA0ADUAZgBhACAAKABSAC0AMgA0ADUAZgBhACkAXAAiACwAIABcACIAQwBIAEYAMgBDAEgAMgBDAEYAMwBcACIALAAgADgANQA4ACwAIABcACIASABGAEMALQAyADQANQBmAGEAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQAzADYANQBtAGYAYwAgACgAUgAtADMANgA1AG0AZgBjACkAXAAiACwAIABcACIAQwBIADMAQwBGADIAQwBIADIAQwBGADMAXAAiACwAIAA4ADAANAAsACAAXAAiAEgARgBDAC0AMwA2ADUAbQBmAGMAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABDAEYAQwAtADIAMgAgACgAUgAtADIAMgApAFwAIgAsACAAXAAiAEMASABDAGwARgAyAFwAIgAsACAAMQA3ADYAMAAsACAAXAAiAEgAQwBGAEMALQAyADIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABDAEYAQwAtADEAMgAzACAAKABSAC0AMQAyADMAKQBcACIALAAgAFwAIgBDAEgAQwBsADIAMgBDAEYAMwBcACIALAAgADcAOQAsACAAXAAiAEgAQwBGAEMALQAxADIAMwBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEMARgBDAC0AMQAyADQAIAAoAFIALQAxADIANAApAFwAIgAsACAAXAAiAEMASABDAGwARgBDAEYAMwBcACIALAAgADUAMgA3ACwAIABcACIASABDAEYAQwAtADEAMgA0AFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAQwBGAEMALQAxADQAMQBiACAAKABSAC0AMQA0ADEAYgApAFwAIgAsACAAXAAiAEMASAAzAEMAQwBsADIARgBcACIALAAgADcAOAAyACwAIABcACIASABDAEYAQwAtADEANAAxAGIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABDAEYAQwAtADEANAAyAGIAIAAoAFIALQAxADQAMgBiACkAXAAiACwAIABcACIAQwBIADIAQwBDAGwARgAyAFwAIgAsACAAMQA5ADgAMAAsACAAXAAiAEgAQwBGAEMALQAxADQAMgBiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAQwBGAEMALQAyADIANQBjAGEAIAAoAFIALQAyADIANQBjAGEAKQBcACIALAAgAFwAIgBDAEgAQwBsADIAQwBGADIAQwBGADMAXAAiACwAIAAxADIANwAsACAAXAAiAEgAQwBGAEMALQAyADIANQBjAGEAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABDAEYAQwAtADIAMgA1AGMAYgAgACgAUgAtADIAMgA1AGMAYgApAFwAIgAsACAAXAAiAEMASABDAGwARgBDAEYAMgBDAEMASQBGADIAXAAiACwAIAA1ADIANQAsACAAXAAiAEgAQwBGAEMALQAyADIANQBjAGIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABGAEMALQAxADQAIABQAGUAcgBmAGwAdQBvAHIAbwBtAGUAdABoAGEAbgBlACAAKAB0AGUAdAByAGEAZgBsAHUAbwByAG8AbQBlAHQAaABhAG4AZQApAFwAIgAsACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAAsACAAXAAiAFAARgBDAC0AMQA0AFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAARgBDAC0AMQAxADYAIABQAGUAcgBmAGwAdQBvAHIAbwBlAHQAaABhAG4AZQAgACgAaABlAHgAYQBmAGwAdQBvAHIAbwBlAHQAaABhAG4AZQApAFwAIgAsACAAXAAiAEMAMgBGADYAXAAiACwAIAAxADEAMQAwADAALAAgAFwAIgBQAEYAQwAtADEAMQA2AFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAARgBDAC0AMgAxADgAIABQAGUAcgBmAGwAdQBvAHIAbwBwAHIAbwBwAGEAbgBlAFwAIgAsACAAXAAiAEMAMwBGADgAXAAiACwAIAA4ADkAMAAwACwAIABcACIAUABGAEMALQAyADEAOABcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAQwAtADMAMQAtADEAMAAgAFAAZQByAGYAbAB1AG8AcgBvAGIAdQB0AGEAbgBlAFwAIgAsACAAXAAiAEMANABGADEAMABcACIALAAgADkAMgAwADAALAAgAFwAIgBQAEYAQwAtADMAMQAtADEAMABcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAQwAtADMAMQA4ACAAUABlAHIAZgBsAHUAbwByAG8AYwB5AGMAbABvAGIAdQB0AGEAbgBlAFwAIgAsACAAXAAiAGMALQBDADQARgA4AFwAIgAsACAAOQA1ADQAMAAsACAAXAAiAFAARgBDAC0AMwAxADgAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABGAEMALQA0ADEALQAxADIAIABQAGUAcgBmAGwAdQBvAHIAbwBwAGUAbgB0AGEAbgBlAFwAIgAsACAAXAAiAEMANQBGADEAMgBcACIALAAgADgANQA1ADAALAAgAFwAIgBQAEYAQwAtADQAMQAtADEAMgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAQwAtADUAMQAtADEANAAgAFAAZQByAGYAbAB1AG8AcgBvAGgAZQB4AGEAbgBlAFwAIgAsACAAXAAiAEMANgBGADEANABcACIALAAgADcAOQAxADAALAAgAFwAIgBQAEYAQwAtADUAMQAtADEANABcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAQwAtADkAMQAtADEAOAAgAFAAZQByAGYAbAB1AG4AYQBmAGUAbgBlAFwAIgAsACAAXAAiAEMAMQAwAEYAMQA4AFwAIgAsACAANwAxADkAMAAsACAAXAAiAFAARgBDAC0AOQAxAC0AMQA4AFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMARgBDAC0AMQAyAFwAIgAsACAAXAAiAEMAQwBsADIARgAyAFwAIgAsACAAMQAwADIAMAAwACwAIABcACIAQwBGAEMALQAxADIAXAAiACwAIABcACIASQBQAEMAQwAgAEcAbABvAGIAYQBsACAAVwBhAHIAbQBpAG4AZwAgAFAAbwB0AGUAbgB0AGkAYQBsACAAVgBhAGwAdQBlAHMAIAB2ADIALgAwACAALQAgACgAQQBSADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAEYAQwAtADEAMwBcACIALAAgAFwAIgBDAEMAbABGADMAXAAiACwAIAAxADMAOQAwADAALAAgAFwAIgBDAEYAQwAtADEAMwBcACIALAAgAFwAIgBJAFAAQwBDACAARwBsAG8AYgBhAGwAIABXAGEAcgBtAGkAbgBnACAAUABvAHQAZQBuAHQAaQBhAGwAIABWAGEAbAB1AGUAcwAgAHYAMgAuADAAIAAtACAAKABBAFIANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMARgBDAC0AMQAxADQAXAAiACwAIABcACIAQwBDAGwARgAyAEMAQwBsAEYAMgBcACIALAAgADgANQA5ADAALAAgAFwAIgBDAEYAQwAtADEAMQA0AFwAIgAsACAAXAAiAEkAUABDAEMAIABHAGwAbwBiAGEAbAAgAFcAYQByAG0AaQBuAGcAIABQAG8AdABlAG4AdABpAGEAbAAgAFYAYQBsAHUAZQBzACAAdgAyAC4AMAAgAC0AIAAoAEEAUgA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBGAEMALQAxADEANQBcACIALAAgAFwAIgBDAEMAbABGADIAQwBGADMAXAAiACwAIAA3ADYANwAwACwAIABcACIAQwBGAEMALQAxADEANQBcACIALAAgAFwAIgBJAFAAQwBDACAARwBsAG8AYgBhAGwAIABXAGEAcgBtAGkAbgBnACAAUABvAHQAZQBuAHQAaQBhAGwAIABWAGEAbAB1AGUAcwAgAHYAMgAuADAAIAAtACAAKABBAFIANQApAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBDAGgAZQBtAGkAYwBhAGwARwBXAFAAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBHAEEAUwAgAC0AIABGAEMAIABuAGEAbQBlAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAdAByAHUAbgBjAGEAdABlAGQAIABnAGEAcwAgAG4AYQBtAGUAIAB0AG8AIABhAGwAbABvAHcAIABtAGEAdABjAGgAaQBuAGcAIAB3AGkAdABoACAAbwB0AGgAZQByACAAdABhAGIAbABlAHMALgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAGcAYQBzAGUAcwAgAGYAcgBvAG0AIABJAFAAQwBDACAARwBsAG8AYgBhAGwAIABXAGEAcgBtAGkAbgBnACAAUABvAHQAZQBuAHQAaQBhAGwAIABWAGEAbAB1AGUAcwAgAHYAMgAuADAAIAAtACAAKABBAFIANQApAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBBAGQAZABpAHQAaQBvAG4AYQBsACAAZABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4ALgBcACIAKQApADsAXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEEAcABwAGUAbgBkAGkAeAAgADIAIABHAGwAbwBiAGEAbAAgAFcAYQByAG0AaQBuAGcAIABQAG8AdABlAG4AdABpAGEAbABzADoAIABCAGwAZQBuAGQAZQBkACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEIAbABlAG4AZABzAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQgBsAGUAbgBkAGUAZAAgAHIAZQBmAHIAaQBnAGUAcgBhAG4AdABzACAAKABtAGEAbgB5ACAAYwBvAG4AdABhAGkAbgBpAG4AZwAgAEgARgBDAFMAIABhAG4AZAAvAG8AcgAgAFAARgBDAFMAKQBcACIAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABCAGwAZQBuAGQAcwBfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEIAbABlAG4AZABzAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAALQAgAEEAcABwAGUAbgBkAGkAeAAgADIAIAAtACAAVABhAGIAbABlACAAMgA0AFwAIgApACkAOwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEIAbABlAG4AZABzAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ADEALAAgADMALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAQgBsAGUAbgBkAFwAIgAsACAAXAAiAEMAbwBuAHMAdABpAHQAdQBlAG4AdABzAFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAGkAdABpAG8AbgAgACgAJQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADAAMABcACIALAAgAFwAIgBDAEYAQwAtADEAMgAvAEMARgBDAC0AMQAxADQAXAAiACwAIABcACIAUgAtADQAMAAwACAAYwBhAG4AIABoAGEAdgBlACAAdgBhAHIAaQBvAHUAcwAgAHAAcgBvAHAAbwByAHQAaQBvAG4AcwAgAG8AZgAgAEMARgBDAC0AMQAyACAAYQBuAGQAIABDAEYAQwAtADEAMQA0AC4AIABUAGgAZQAgAGUAeABhAGMAdAAgAGMAbwBtAHAAbwBzAGkAdABpAG8AbgAgAG4AZQBlAGQAcwAgAHQAbwAgAGIAZQAgAHMAcABlAGMAaQBmAGkAZQBkACwAIABlAC4AZwAuACwAIABSAC0ANAAwADAAIAAoADYAMAAvADQAMAApAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAAxAEEAXAAiACwAIABcACIASABDAEYAQwAtADIAMgAvAEgARgBDAC0AMQA1ADIAYQAvAEgAQwBGAEMALQAxADIANABcACIALAAgAFwAIgAoADUAMwAuADAALwAxADMALgAwAC8AMwA0AC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADAAMQBCAFwAIgAsACAAXAAiAEgAQwBGAEMALQAyADIALwBIAEYAQwAtADEANQAyAGEALwBIAEMARgBDAC0AMQAyADQAXAAiACwAIABcACIAKAA2ADEALgAwAC8AMQAxAC4AMAAvADIAOAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADEAQwBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8ASABGAEMALQAxADUAMgBhAC8ASABDAEYAQwAtADEAMgA0AFwAIgAsACAAXAAiACgAMwAzAC4AMAAvADEANQAuADAALwA1ADIALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAAyAEEAXAAiACwAIABcACIASABGAEMALQAxADIANQAvAEgAQwAtADIAOQAwAC8ASABDAEYAQwAtADIAMgBcACIALAAgAFwAIgAoADYAMAAuADAALwAyAC4AMAAvADMAOAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADIAQgBcACIALAAgAFwAIgBIAEYAQwAtADEAMgA1AC8ASABDAC0AMgA5ADAALwBIAEMARgBDAC0AMgAyAFwAIgAsACAAXAAiACgAMwA4AC4AMAAvADIALgAwAC8ANgAwAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADAAMwBBAFwAIgAsACAAXAAiAEgAQwAtADIAOQAwAC8ASABDAEYAQwAtADIAMgAvAFAARgBDAC0AMgAxADgAXAAiACwAIABcACIAKAA1AC4AMAAvADcANQAuADAALwAyADAALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAAzAEIAXAAiACwAIABcACIASABDAC0AMgA5ADAALwBIAEMARgBDAC0AMgAyAC8AUABGAEMALQAyADEAOABcACIALAAgAFwAIgAoADUALgAwAC8ANQA2AC4AMAAvADMAOQAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADQAQQBcACIALAAgAFwAIgBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADQAMwBhAC8ASABGAEMALQAxADMANABhAFwAIgAsACAAXAAiACgANAA0AC4AMAAvADUAMgAuADAALwA0AC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADAANQBBAFwAIgAsACAAXAAiAEgAQwBGAEMALQAyADIALwAgAEgARgBDAC0AMQA1ADIAYQAvAEgAQwBGAEMALQAxADQAMgBiAC8AUABGAEMALQAzADEAOABcACIALAAgAFwAIgAoADQANQAuADAALwA3AC4AMAAvADUALgA1AC8ANAAyAC4ANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADAANgBBAFwAIgAsACAAXAAiAEgAQwBGAEMALQAyADIALwBIAEMALQA2ADAAMABhAC8ASABDAEYAQwAtADEANAAyAGIAXAAiACwAIABcACIAKAA1ADUALgAwAC8AMQA0AC4AMAAvADQAMQAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADcAQQBcACIALAAgAFwAIgBIAEYAQwAtADMAMgAvAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEAXAAiACwAIABcACIAKAAyADAALgAwAC8ANAAwAC4AMAAvADQAMAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADcAQgBcACIALAAgAFwAIgBIAEYAQwAtADMAMgAvAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEAXAAiACwAIABcACIAKAAxADAALgAwAC8ANwAwAC4AMAAvADIAMAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADcAQwBcACIALAAgAFwAIgBIAEYAQwAtADMAMgAvAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEAXAAiACwAIABcACIAKAAyADMALgAwAC8AMgA1AC4AMAAvADUAMgAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADcARABcACIALAAgAFwAIgBIAEYAQwAtADMAMgAvAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEAXAAiACwAIABcACIAKAAxADUALgAwAC8AMQA1AC4AMAAvADcAMAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADcARQBcACIALAAgAFwAIgBIAEYAQwAtADMAMgAvAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEAXAAiACwAIABcACIAKAAyADUALgAwAC8AMQA1AC4AMAAvADYAMAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADgAQQBcACIALAAgAFwAIgBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADQAMwBhAC8ASABDAEYAQwAtADIAMgBcACIALAAgAFwAIgAoADcALgAwAC8ANAA2AC4AMAAvADQANwAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADkAQQBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8ASABDAEYAQwAtADEAMgA0AC8ASABDAEYAQwAtADEANAAyAGIAXAAiACwAIABcACIAKAA2ADAALgAwAC8AMgA1AC4AMAAvADEANQAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADkAQgBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8ASABDAEYAQwAtADEAMgA0AC8ASABDAEYAQwAtADEANAAyAGIAXAAiACwAIABcACIAKAA2ADUALgAwAC8AMgA1AC4AMAAvADEAMAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAxADAAQQBcACIALAAgAFwAIgBIAEYAQwAtADMAMgAvAEgARgBDAC0AMQAyADUAXAAiACwAIABcACIAKAA1ADAALgAwAC8ANQAwAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEAMABCAFwAIgAsACAAXAAiAEgARgBDAC0AMwAyAC8ASABGAEMALQAxADIANQBcACIALAAgAFwAIgAoADQANQAuADAALwA1ADUALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQAxAEEAXAAiACwAIABcACIASABDAC0AMQAyADcAMAAvAEgAQwBGAEMALQAyADIALwBIAEYAQwAtADEANQAyAGEAXAAiACwAIABcACIAKAAxAC4ANQAvADgANwAuADUALwAxADEALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQAxAEIAXAAiACwAIABcACIASABDAC0AMQAyADcAMAAvAEgAQwBGAEMALQAyADIALwBIAEYAQwAtADEANQAyAGEAXAAiACwAIABcACIAKAAzAC4AMAAvADkANAAuADAALwAzAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEAMQBDAFwAIgAsACAAXAAiAEgAQwAtADEAMgA3ADAALwBIAEMARgBDAC0AMgAyAC8ASABGAEMALQAxADUAMgBhAFwAIgAsACAAXAAiACgAMwAuADAALwA5ADUALgA1AC8AMQAuADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAxADIAQQBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8AUABGAEMALQAyADEAOAAvAEgAQwBGAEMALQAxADQAMgBiAFwAIgAsACAAXAAiACgANwAwAC4AMAAvADUALgAwAC8AMgA1AC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEAMwBBAFwAIgAsACAAXAAiAFAARgBDAC0AMgAxADgALwBIAEYAQwAtADEAMwA0AGEALwBIAEMALQA2ADAAMABhAFwAIgAsACAAXAAiACgAOQAuADAALwA4ADgALgAwAC8AMwAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAxADQAQQBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8ASABDAEYAQwAtADEAMgA0AC8ASABDAC0ANgAwADAAYQAvAEgAQwBGAEMALQAxADQAMgBiAFwAIgAsACAAXAAiACgANQAxAC4AMAAvADIAOAAuADUALwA0AC4AMAAvADEANgAuADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAxADQAQgBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8ASABDAEYAQwAtADEAMgA0AC8ASABDAC0ANgAwADAAYQAvAEgAQwBGAEMALQAxADQAMgBiAFwAIgAsACAAXAAiACgANQAwAC4AMAAvADMAOQAuADAALwAxAC4ANQAvADkALgA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQA1AEEAXAAiACwAIABcACIASABDAEYAQwAtADIAMgAvAEgARgBDAC0AMQA1ADIAYQBcACIALAAgAFwAIgAoADgAMgAuADAALwAxADgALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQA1AEIAXAAiACwAIABcACIASABDAEYAQwAtADIAMgAvAEgARgBDAC0AMQA1ADIAYQBcACIALAAgAFwAIgAoADIANQAuADAALwA3ADUALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQA2AEEAXAAiACwAIABcACIASABGAEMALQAxADMANABhAC8ASABDAEYAQwAtADEAMgA0AC8ASABDAC0ANgAwADAAXAAiACwAIABcACIAKAA1ADkALgAwAC8AMwA5AC4ANQAvADEALgA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQA3AEEAXAAiACwAIABcACIASABGAEMALQAxADIANQAvAEgARgBDAC0AMQAzADQAYQAvAEgAQwAtADYAMAAwAFwAIgAsACAAXAAiACgANAA2AC4ANgAvADUAMAAuADAALwAzAC4ANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEAOABBAFwAIgAsACAAXAAiAEgAQwAtADIAOQAwAC8ASABDAEYAQwAtADIAMgAvAEgARgBDAC0AMQA1ADIAYQBcACIALAAgAFwAIgAoADEALgA1AC8AOQA2AC4AMAAvADIALgA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQA5AEEAXAAiACwAIABcACIASABGAEMALQAxADIANQAvAEgARgBDAC0AMQAzADQAYQAvAEgARQAtAEUAMQA3ADAAXAAiACwAIABcACIAKAA3ADcALgAwAC8AMQA5AC4AMAAvADQALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMgAwAEEAXAAiACwAIABcACIASABGAEMALQAxADMANABhAC8ASABDAEYAQwAtADEANAAyAGIAXAAiACwAIABcACIAKAA4ADgALgAwAC8AMQAyAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADIAMQBBAFwAIgAsACAAXAAiAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEAXAAiACwAIABcACIAKAA1ADgALgAwAC8ANAAyAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADIAMgBBAFwAIgAsACAAXAAiAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEALwBIAEMALQA2ADAAMABhAFwAIgAsACAAXAAiACgAOAA1AC4AMQAvADEAMQAuADUALwAzAC4ANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADIAMgBCAFwAIgAsACAAXAAiAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEALwBIAEMALQA2ADAAMABhAFwAIgAsACAAXAAiACgANQA1AC4AMAAvADQAMgAuADAALwAzAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADIAMgBDAFwAIgAsACAAXAAiAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEALwBIAEMALQA2ADAAMABhAFwAIgAsACAAXAAiACgAOAAyAC4AMAAvADEANQAuADAALwAzAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA1ADAAMABcACIALAAgAFwAIgBDAEYAQwAtADEAMgAvAEgARgBDAC0AMQA1ADIAYQBcACIALAAgAFwAIgAoADcAMwAuADgALwAyADYALgAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADUAMAAxAFwAIgAsACAAXAAiAEgAQwBGAEMALQAyADIALwBDAEYAQwAtADEAMgBcACIALAAgAFwAIgAoADcANQAuADAALwAyADUALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADUAMAAyAFwAIgAsACAAXAAiAEgAQwBGAEMALQAyADIALwBDAEYAQwAtADEAMQA1AFwAIgAsACAAXAAiACgANAA4AC4AOAAvADUAMQAuADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANQAwADMAXAAiACwAIABcACIASABGAEMALQAyADMALwBDAEYAQwAtADEAMwBcACIALAAgAFwAIgAoADQAMAAuADEALwA1ADkALgA5ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADUAMAA0AFwAIgAsACAAXAAiAEgARgBDAC0AMwAyAC8AQwBGAEMALQAxADEANQBcACIALAAgAFwAIgAoADQAOAAuADIALwA1ADEALgA4ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADUAMAA1AFwAIgAsACAAXAAiAEMARgBDAC0AMQAyAC8ASABDAEYAQwAtADMAMQBcACIALAAgAFwAIgAoADcAOAAuADAALwAyADIALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADUAMAA2AFwAIgAsACAAXAAiAEMARgBDAC0AMwAxAC8AQwBGAEMALQAxADEANABcACIALAAgAFwAIgAoADUANQAuADEALwA0ADQALgA5ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADUAMAA3AEEAXAAiACwAIABcACIASABGAEMALQAxADIANQAvAEgARgBDAC0AMQA0ADMAYQBcACIALAAgAFwAIgAoADUAMAAuADAALwA1ADAALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADUAMAA4AEEAXAAiACwAIABcACIASABGAEMALQAyADMALwBQAEYAQwAtADEAMQA2AFwAIgAsACAAXAAiACgAMwA5AC4AMAAvADYAMQAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANQAwADgAQgBcACIALAAgAFwAIgBIAEYAQwAtADIAMwAvAFAARgBDAC0AMQAxADYAXAAiACwAIABcACIAKAA0ADYALgAwAC8ANQA0AC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA1ADAAOQBBAFwAIgAsACAAXAAiAEgAQwBGAEMALQAyADIALwBQAEYAQwAtADIAMQA4AFwAIgAsACAAXAAiACgANAA0AC4AMAAvADUANgAuADAAKQBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEIAbABlAG4AZABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAARgBpAHgAZQBkACAAdAB5AHAAbwAgAC0AIABjAGgAYQBuAGcAZQBkACAASABDADYAMAAwAGEAIAB0AG8AIABIAEMALQA2ADAAMABhACAAZgBvAHIAIABiAGwAZQBuAGQAIABSAC0ANAAxADQAQgAuACAARgBpAHgAZQBkACAAdAB5AHAAbwAgAGYAbwByACAAYgBsAGUAbgBkACAAUgAtADQAMAA1AEEAIAAtACAAQwBoAGEAbgBnAGUAZAAgAEgAQwBGAEMAMQA0ADIAYgAgAHQAbwAgAEgAQwBGAEMALQAxADQAMgBiAC4AXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ATABlAGEAawBhAGcAZQAgAHIAYQB0AGUAcwAgAGYAbwByACAAYwBvAG0AbQBvAG4AIAByAGUAZgByAGkAZwBlAHIAYQB0AGkAbwBuACAAYQBuAGQAIABhAGkAcgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBMAGUAYQBrAGEAZwBlAFIAYQB0AGUAcwBfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEkAbgBkAGkAYwBhAHQAaQB2AGUAIABsAGUAYQBrAGEAZwBlACAAcgBhAHQAZQBzACAAZgBvAHIAIABjAG8AbQBtAG8AbgAgAHIAZQBmAHIAaQBnAGUAcgBhAHQAaQBvAG4AIABhAG4AZAAgAGEAaQByACAALQAgAGMAbwBuAGQAaQB0AGkAbwBuAGkAbgBnACAAZQBxAHUAaQBwAG0AZQBuAHQAXAAiACkAKQA7AFwAbgBcAG4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBMAGUAYQBrAGEAZwBlAFIAYQB0AGUAcwBfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ATABlAGEAawBhAGcAZQBSAGEAdABlAHMAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAQQBjAGMAbwB1AG4AdABzACAARgBhAGMAdABvAHIAcwAgADIAMAAyADUAIAAtACAAVABhAGIAbABlACAAMQAwAFwAIgApACkAOwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ATABlAGEAawBhAGcAZQBSAGEAdABlAHMAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgAMQAsACAAMgAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAbABlAGEAawBhAGcAZQAgAHIAYQB0AGUAIAAoACUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAIAByAGUAZgByAGkAZwBlAHIAYQB0AG8AcgBzAFwAIgAsACAAMQAuADcAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAYQBuAHMAcABvAHIAdAAgAHIAZQBmAHIAaQBnAGUAcgBhAHQAaQBvAG4AXAAiACwAIAAxADUALgA3ADsAXABuACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjACAAQQAvAEMAIABwAG8AcgB0AGEAYgBsAGUAXAAiACwAIAAyAC4ANQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwAgAEEALwBDACAAcwBwAGwAaQB0AFwAIgAsACAAMwAuADUAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAIABBAC8AQwAgAHAAYQBjAGsAYQBnAGUAZABcACIALAAgADIALgA1ADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABpAGcAaAB0ACAAdgBlAGgAaQBjAGwAZQAgAEEALwBDAFwAIgAsACAANgAuADcAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAYQB2AHkAIAB2AGUAaABpAGMAbABlACAAQQAvAEMAXAAiACwAIAAxADAALgA4AFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEwAZQBhAGsAYQBnAGUAUgBhAHQAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBDAGEAbABjAHUAbABhAHQAZQBCAGwAZQBuAGQARwBXAFAAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAbwBuAHMAdABpAHQAdQBlAG4AdABGAGEAYwB0AGkAbwBuADEALAAgAEMAbwBuAHMAdABpAHQAdQBlAG4AdABHAFcAUAAxACwAIABcAG4AIAAgAEMAbwBuAHMAdABpAHQAdQBlAG4AdABGAGEAYwB0AGkAbwBuADIALAAgAEMAbwBuAHMAdABpAHQAdQBlAG4AdABHAFcAUAAyACwAIABcAG4AIAAgAEMAbwBuAHMAdABpAHQAdQBlAG4AdABGAGEAYwB0AGkAbwBuADMALAAgAEMAbwBuAHMAdABpAHQAdQBlAG4AdABHAFcAUAAzACwAIABcAG4AIAAgAEMAbwBuAHMAdABpAHQAdQBlAG4AdABGAGEAYwB0AGkAbwBuADQALAAgAEMAbwBuAHMAdABpAHQAdQBlAG4AdABHAFcAUAA0ACwAXABuACAAIAAoAEMAbwBuAHMAdABpAHQAdQBlAG4AdABGAGEAYwB0AGkAbwBuADEAIAAqACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEcAVwBQADEAKQAgACsAXABuACAAIAAoAEMAbwBuAHMAdABpAHQAdQBlAG4AdABGAGEAYwB0AGkAbwBuADIAIAAqACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEcAVwBQADIAKQAgACsAXABuACAAIAAoAEMAbwBuAHMAdABpAHQAdQBlAG4AdABGAGEAYwB0AGkAbwBuADMAIAAqACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEcAVwBQADMAKQAgACsAXABuACAAIAAoAEMAbwBuAHMAdABpAHQAdQBlAG4AdABGAGEAYwB0AGkAbwBuADQAIAAqACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEcAVwBQADQAKQBcAG4AKQA7ACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAEQAYQB0AGEAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVABpAHQAbABlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBTAG8AdQByAGMAZQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGEAdABhACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAFQAaQB0AGwAZQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBTAG8AdQByAGMAZQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8ARABhAHQAYQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQAXwBTAG8AdQByAGMAZQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAEQAYQB0AGEAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8AVABpAHQAbABlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AE8AZgBmAFIAbwBhAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AE8AZgBmAFIAbwBhAGQAXwBEAGEAdABhACIALAAiAEYAdQBlAGwAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBGAHUAZQBsAF8ARwBlAHQAVAByAGEAbgBzAHAAbwByAHQARgB1AGUAbABTAHQAcgBpAG4AZwAiACwAIgBGAHUAZQBsAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4ARgB1AGUAbABfAEcAZQB0AFMAdABhAHQAaQBvAG4AYQByAHkARgB1AGUAbABTAHQAcgBpAG4AZwAiACwAIgBGAHUAZQBsAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4ARgB1AGUAbABfAFQAbwB0AGEAbABDAG8AbgBzAHUAbQBwAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0ACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8AVQBuAGkAdAAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AVABpAHQAbABlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBVAG4AaQB0ACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AVABpAHQAbABlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAFUAbgBpAHQAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwBYAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAEcAZQBuAGUAcgBpAGMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AWABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBHAGUAbgBlAHIAaQBjAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfAFgAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4ARwBlAG4AZQByAGkAYwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcARwBXAFAAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAF8AVABpAHQAbABlACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAFUAbgBpAHQAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBTAG8AdQByAGMAZQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBSAGUAYQBkAGEAYgBsAGUARQBxAHUAYQB0AGkAbwBuACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcARwBXAFAAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABHAFcAUABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEcAVwBQAF8ARABhAHQAYQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABHAFcAUABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEIAbABlAG4AZABzAF8AVABpAHQAbABlACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEIAbABlAG4AZABzAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEIAbABlAG4AZABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBDAGgAZQBtAGkAYwBhAGwAQgBsAGUAbgBkAHMAXwBEAGEAdABhACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEIAbABlAG4AZABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBMAGUAYQBrAGEAZwBlAFIAYQB0AGUAcwBfAFQAaQB0AGwAZQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEwAZQBhAGsAYQBnAGUAUgBhAHQAZQBzAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ATABlAGEAawBhAGcAZQBSAGEAdABlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEwAZQBhAGsAYQBnAGUAUgBhAHQAZQBzAF8ARABhAHQAYQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEwAZQBhAGsAYQBnAGUAUgBhAHQAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAYQBsAGMAdQBsAGEAdABlAEIAbABlAG4AZABHAFcAUAAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -19514,7 +19501,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAG4AZAAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIAByAGUAdAB1AHIAbgBlAGQAIAB0AG8AIAB0AGgAZQAgAHMAbwBpAGwAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUARgBOAGkAIAAmACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAJgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACkAKgAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADIAKQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlACkAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwBlAGwAbAAsACAARABlAGwAaQBtAGkAdABlAHIALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEAXQAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgBdACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgBYAE0ATAAoAFwAbgAgACAAIAAgACAAIAAgACAAXAAiADwAdAA+ADwAcwA+AFwAIgAgACYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAPAAvAHMAPgA8AHMAPgBcACIAXABuACAAIAAgACAAIAAgACAAIAApACAAJgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AC8AcwA+ADwALwB0AD4AXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApADwAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkAKQA+AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQA+AD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkAKQA8AD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAPgA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPAA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQA+AD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApADwAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAPgA9AG0AYQBwAF8AcABlAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABBAEsARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgADEAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAE0AaQBuAEEAcgByAGEAeQAsACAATQBhAHgAQQByAHIAYQB5ACwAIABJAHQAZQBtAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AaQBuAEEAcgByAGEAeQApADwAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQA+AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8ACAAUwApACwAXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAD4AIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApADwAUwApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBiACAAcwB0AGEAcgB0AHMAIABhAGYAdABlAHIAIABFACwAaQB0ACAAYwBhAG4AJwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+AEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIAAmACAAXAAiACAAdABvACAAXAAiACAAJgAgAGUAbgBkAHMAVABlAHgAdAAgACYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAA+ADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjACcAXAAiACAAJgAgAHMAaAAgACYAIABcACIAJwAhAFwAIgAgACYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgACYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADEALAAgADIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADMALAAgADQAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAATQBNAFMALAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFwAbgAgACAAIAAgACAAIAAgACAATQBFAEQASQBBAE4AKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFUATgBEACgAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIAAwACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAE0ATQBTACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAaQB0AGwAZQBDAGUAbABsACwAIABTAG8AdQByAGMAZQBDAGUAbABsACwAXABuACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAEwARQBGAFQAKABTAG8AdQByAGMAZQBDAGUAbABsACwAIABGAEkATgBEACgAXAAiACwAXAAiACwAIABTAG8AdQByAGMAZQBDAGUAbABsACkAIAAtADEAKQAsACAAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFwAIgAsACAAXAAiAFwAIgApACAAJgAgAFwAIgAgAFwAIgAgACYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABTAHQAYQB0AGkAbwBuAGEAcgB5ACAAZwBhAHMAZQBvAHUAcwAgAGYAdQBlAGwAcwBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABTAHQAYQB0AGkAbwBuAGEAcgB5ACAAZwBhAHMAZQBvAHUAcwAgAGYAdQBlAGwAcwBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARABpAHIAZQBjAHQAIAAoAFMAYwBvAHAAZQAgADEAKQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAZwBhAHMAZQBvAHUAcwAgAGYAdQBlAGwAcwAgAGkAbgBjAGwAdQBkAGkAbgBnACAAbABpAHEAdQBlAGYAaQBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAIAAgAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAQQBjAGMAbwB1AG4AdABzACAARgBhAGMAdABvAHIAcwAgADIAMAAyADUAIAAtACAAVABhAGIAbABlACAANQBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADkALAAgADcALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIARgB1AGUAbAAgAGMAbwBtAGIAdQBzAHQAZQBkAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAQwBvAG4AdABlAG4AdAAgAEYAYQBjAHQAbwByACAAKABHAEoAIABwAGUAcgAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsACkAXAAiACwAIABcACIARgB1AGUAbAAgAHUAbgBpAHQAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBPADIAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBIADQAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAATgAyAE8AXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAAQwBvAG0AYgBpAG4AZQBkACAAZwBhAHMAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE4AYQB0AHUAcgBhAGwAIABnAGEAcwAgAGQAaQBzAHQAcgBpAGIAdQB0AGUAZAAgAGkAbgAgAGEAIABwAGkAcABlAGwAaQBuAGUAXAAiACwAIAAwAC4AMAAzADkAMwAsACAAXAAiAG0AMwBcACIALAAgADUAMQAuADQALAAgADAALgAxACwAIAAwAC4AMAAzACwAIAA1ADEALgA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AYQBsACAAcwBlAGEAbQAgAG0AZQB0AGgAYQBuAGUAIAB0AGgAYQB0ACAAaQBzACAAYwBhAHAAdAB1AHIAZQBkACAAZgBvAHIAIABjAG8AbQBiAHUAcwB0AGkAbwBuAFwAIgAsACAAMAAuADAAMwA3ADcALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAAwAC4AMgAsACAAMAAuADAAMwAsACAANQAxAC4ANgAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAGEAbAAgAG0AaQBuAGUAIAB3AGEAcwB0AGUAIABnAGEAcwAgAHQAaABhAHQAIABpAHMAIABjAGEAcAB0AHUAcgBlAGQAIABmAG8AcgAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AXAAiACwAIAAwAC4AMAAzADcANwAsACAAXAAiAG0AMwBcACIALAAgADUAMQAuADkALAAgADQALgA2ACwAIAAwAC4AMwAsACAANQA2AC4AOAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAcgBlAHMAcwBlAGQAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAKAByAGUAdgBlAHIAdABpAG4AZwAgAHQAbwAgAHMAdABhAG4AZABhAHIAZAAgAGMAbwBuAGQAaQB0AGkAbwBuAHMAKQBcACIALAAgADAALgAwADMAOQAzACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFUAbgBwAHIAbwBjAGUAcwBzAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwBcACIALAAgADAALgAwADMAOQAzACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEUAdABoAGEAbgBlAFwAIgAsACAAMAAuADAANgAyADkALAAgAFwAIgBtADMAXAAiACwAIAA1ADYALgA1ACwAIAAwAC4AMAAzACwAIAAwAC4AMAAzACwAIAA1ADYALgA1ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AawBlACAAbwB2AGUAbgAgAGcAYQBzAFwAIgAsACAAMAAuADAAMQA4ADEALAAgAFwAIgBtADMAXAAiACwAIAAzADcALgAwACwAIAAwAC4AMAAzACwAIAAwAC4AMAA1ACwAIAAzADcALgAwADgAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBCAGwAYQBzAHQAIABmAHUAcgBuAGEAYwBlACAAZwBhAHMAXAAiACwAIAAwAC4AMAAwADQAMAAsACAAXAAiAG0AMwBcACIALAAgADIAMwA0AC4AMAAsACAAMAAuADAAMwAsACAAMAAuADAAMgAsACAAMgAzADQALgAwADUAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAG8AdwBuACAAZwBhAHMAXAAiACwAIAAwAC4AMAAzADkAMAAsACAAXAAiAG0AMwBcACIALAAgADYAMAAuADIALAAgADAALgAwADQALAAgADAALgAwADMALAAgADYAMAAuADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAaQBxAHUAZQBmAGkAZQBkACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAFwAIgAsACAAMgA1AC4AMwAsACAAXAAiAGsATABcACIALAAgADUAMQAuADQALAAgADAALgAxACwAIAAwAC4AMAAzACwAIAA1ADEALgA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBHAGEAcwBlAG8AdQBzACAAZgBvAHMAcwBpAGwAIABmAHUAZQBsAHMAIABvAHQAaABlAHIAIAB0AGgAYQBuACAAdABoAG8AcwBlACAAbQBlAG4AdABpAG8AbgBlAGQAIABpAG4AIAB0AGgAZQAgAGkAdABlAG0AcwAgAGEAYgBvAHYAZQBcACIALAAgADAALgAwADMAOQAwACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4ANAAsACAAMAAuADEALAAgADAALgAwADMALAAgADUAMQAuADUAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbAAgAGIAaQBvAGcAYQBzACAAdABoAGEAdAAgAGkAcwAgAGMAYQBwAHQAdQByAGUAZAAgAGYAbwByACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgACgAbQBlAHQAaABhAG4AZQAgAG8AbgBsAHkAKQBcACIALAAgADAALgAwADMANwA3ACwAIABcACIAbQAzAFwAIgAsACAAMAAuADAALAAgADYALgA0ACwAIAAwAC4AMAAzACwAIAA2AC4ANAAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwBsAHUAZABnAGUAIABiAGkAbwBnAGEAcwAgAHQAaABhAHQAIABpAHMAIABjAGEAcAB0AHUAcgBlAGQAIABmAG8AcgAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIAAoAG0AZQB0AGgAYQBuAGUAIABvAG4AbAB5ACkAXAAiACwAIAAwAC4AMAAzADcANwAsACAAXAAiAG0AMwBcACIALAAgADAALgAwACwAIAA2AC4ANAAsACAAMAAuADAAMwAsACAANgAuADQAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAIABiAGkAbwBnAGEAcwAgAHQAaABhAHQAIABpAHMAIABjAGEAcAB0AHUAcgBlAGQAIABmAG8AcgAgAGMAbwBtAGIAdQBzAHQAaQBvAG4ALAAgAG8AdABoAGUAcgAgAHQAaABhAG4AIAB0AGgAbwBzAGUAIABtAGUAbgB0AGkAbwBuAGUAZAAgAGkAbgAgAHQAaABlACAAaQB0AGUAbQBzACAAYQBiAG8AdgBlAFwAIgAsACAAMAAuADAAMwA3ADAALAAgAFwAIgBtADMAXAAiACwAIAAwAC4AMAAsACAANgAuADQALAAgADAALgAwADMALAAgADYALgA0ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBCAGkAbwBtAGUAdABoAGEAbgBlAFwAIgAsACAAMAAuADAAMwA5ADMALAAgAFwAIgBtADMAXAAiACwAIAAwAC4AMAAsACAAMAAuADEALAAgADAALgAwADMALAAgADAALgAxADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAHkAZAByAG8AZwBlAG4AXAAiACwAIAAwAC4AMAAxADIAMgAsACAAXAAiAG0AMwBcACIALAAgADAALgAwACwAIAAwAC4AMAAsACAAMAAuADUALAAgADAALgA1ADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBhAHQAdQByAGEAbAAgAGcAYQBzACAAZABpAHMAdAByAGkAYgB1AHQAZQBkACAAaQBuACAAYQAgAHAAaQBwAGUAbABpAG4AZQAgAC0AIABHAGkAZwBhAGoAbwB1AGwAZQBzAFwAIgAsACAAMQAsACAAXAAiAEcASgBcACIALAAgADUAMQAuADQALAAgADAALgAxACwAIAAwAC4AMAAzACwAIAA1ADEALgA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAG8AdwBuACAAZwBhAHMAIAAtACAARwBpAGcAYQBqAG8AdQBsAGUAcwBcACIALAAgADEALAAgAFwAIgBHAEoAXAAiACwAIAA2ADAALgAyACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAzACwAIAA2ADAALgAyADcAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIAAnAE4AYQB0AHUAcgBhAGwAIABnAGEAcwAgAGQAaQBzAHQAcgBpAGIAdQB0AGUAZAAgAGkAbgAgAGEAIABwAGkAcABlAGwAaQBuAGUAIAAtACAARwBpAGcAYQBqAG8AdQBsAGUAcwAnACAAYQBuAGQAIAAnAFQAbwB3AG4AIABnAGEAcwAgAC0AIABHAGkAZwBhAGoAbwB1AGwAZQBzACcAIAB3AGUAcgBlACAAYQBkAGQAZQBkACwAIABlAGEAYwBoACAAdwBpAHQAaAAgAGEAbgAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAGYAYQBjAHQAbwByACAAbwBmACAAMQAgAEcASgAgAHAAZQByACAAdQBuAGkAdAAgAG8AZgAgAGYAdQBlAGwALgAgAFQAaABpAHMAIABpAHMAIABmAG8AcgAgAHUAcwBlAHIAcwAgAHcAaABvACAAaABhAHYAZQAgAGYAdQBlAGwAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABkAGEAdABhACAAaQBuACAARwBKACAAcgBhAHQAaABlAHIAIAB0AGgAYQBuACAAbQAzAC4AXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ARgB1AGUAbAAgAHMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARgB1AGUAbAAgAHMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABnAGEAcwBlAG8AdQBzACAAZgB1AGUAbABzAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBJAG4AZABpAHIAZQBjAHQAIAAoAFMAYwBvAHAAZQAgADMAKQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHQAaABlACAAYwBvAG4AcwB1AG0AcAB0AGkAbwBuACAAbwBmACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAC4AXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAA2AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAdABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMwAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIABmAG8AcgAgAE4AYQB0AHUAcgBhAGwAIABHAGEAcwAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAE0AZQB0AHIAbwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAcwAgAGYAbwByACAATgBhAHQAdQByAGEAbAAgAEcAYQBzACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApACAATgBvAG4AIAAtACAATQBlAHQAcgBvAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAMQAzAC4AMQAsACAAMQA0AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAQwBUAFwAIgAsACAAMQAzAC4AMQAsACAAMQA0AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgADQALgAwACwAIAA0AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIAA4AC4AOAAsACAANwAuADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgADEAMAAuADcALAAgADEAMAAuADYAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIAA0AC4AMQAsACAANAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIAA0AC4AMAAsACAANAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQBcACIALAAgADQALgAxACwAIAA0AC4AMABcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAE4AUwBXACAAYQBuAGQAIABBAEMAVAAgAHMAcABsAGkAdAAgAGkAbgB0AG8AIABzAGUAcABhAHIAYQB0AGUAIAByAG8AdwBzAC4AIAAnAEMAJwAgAFYAYQBsAHUAZQBzACAAZgBvAHIAIABUAGEAcwBtAGEAbgBpAGEAIABhAG4AZAAgAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5ACAAcgBlAHAAbABhAGMAZQBkACAAdwBpAHQAaAAgAHQAaABvAHMAZQAgAGYAbwByACAAVgBpAGMAdABvAHIAaQBhACAAYQBuAGQAIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAByAGUAcwBwAGUAYwB0AGkAdgBlAGwAeQAuACAAKABTAGUAZQAgAGEAcABwAGUAbgBkAGkAYwBlAHMAKQBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADIALAAgADIALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAFwAIgBBAHMAIABTAGMAbwBwAGUAIAAzACAAZgBhAGMAdABvAHIAcwAgAGEAcgBlACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGEAdAAgAHQAaABlACAAcABvAGkAbgB0ACAAdwBoAGUAcgBlACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzACAAaQBzACAAZABlAGwAaQB2AGUAcgBlAGQAIAB0AG8AIABlAG4AZAAgAHUAcwBlAHIAcwAsACAAaQB0ACAAaQBzACAAbgBlAGMAZQBzAHMAYQByAHkAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAGEAdAAgAGUAYQBjAGgAIABvAGYAIAB0AGgAZQAgAGwAbwBhAGQAIABjAGUAbgB0AHIAZQBzAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIARwBhAHMAIAByAGUAYQBjAGgAZQBzACAAZQBuAGQAIAB1AHMAZQByAHMAIABlAGkAdABoAGUAcgAgAGYAcgBvAG0AIAB0AGgAZQAgAG0AZQB0AHIAbwAgAGQAaQBzAHQAcgBpAGIAdQB0AGkAbwBuACAAbgBlAHQAdwBvAHIAawBzACAAbwByACAAZABpAHIAZQBjAHQAIABmAHIAbwBtACAAdABoAGUAIABoAGkAZwBoACAALQAgAHAAcgBlAHMAcwB1AHIAZQAgAGQAaQBzAHQAcgBpAGIAdQB0AGkAbwBuACAAcABpAHAAZQBsAGkAbgBlAHMALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBIAG8AdQBzAGUAaABvAGwAZABzACAAYQBuAGQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdQBzAGUAcgBzACAAdABlAG4AZAAgAHQAbwAgAGIAZQAgAHMAZQByAHYAZQBkACAAYgB5ACAAdABoAGUAIABmAG8AcgBtAGUAcgAsACAAYQBuAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAIABnAGUAbgBlAHIAYQB0AG8AcgBzACAAYQBuAGQAIABsAGEAcgBnAGUAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAcABsAGEAbgB0AHMAIABmAHIAbwBtACAAdABoAGUAIABsAGEAdAB0AGUAcgAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC0AXAAiACwAIABcACIATQBlAHQAcgBvACAAaQBzACAAZABlAGYAaQBuAGUAZAAgAGEAcwAgAGwAbwBjAGEAdABlAGQAIABvAG4AIABvAHIAIABlAGEAcwB0ACAAbwBmACAAdABoAGUAIABkAGkAdgBpAGQAaQBuAGcAIAByAGEAbgBnAGUAIABpAG4AIABOAFMAVwAsACAAaQBuAGMAbAB1AGQAaQBuAGcAIABDAGEAbgBiAGUAcgByAGEAIABhAG4AZAAgAFEAdQBlAGEAbgBiAGUAeQBhAG4ALAAgAE0AZQBsAGIAbwB1AHIAbgBlACwAIABCAHIAaQBzAGIAYQBuAGUALAAgAEEAZABlAGwAYQBpAGQAZQAgAG8AcgAgAFAAZQByAHQAaAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAE8AdABoAGUAcgB3AGkAcwBlACwAIAB0AGgAZQAgAG4AbwBuACAALQAgAG0AZQB0AHIAbwAgAGYAYQBjAHQAbwByACAAcwBoAG8AdQBsAGQAIABiAGUAIAB1AHMAZQBkAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAFwAIgBGAGEAYwB0AG8AcgBzACAAYQByAGUAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgBvAHIAIABhAGwAbAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwAgAGQAaQBzAHQAcgBpAGIAdQB0AGUAZAAgAGkAbgAgAGEAIABwAGkAcABlAGwAaQBuAGUAIAB3AGgAaQBjAGgAIABtAGEAeQAgAGkAbgBjAGwAdQBkAGUAIABjAG8AYQBsACAAcwBlAGEAbQAgAG0AZQB0AGgAYQBuAGUALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAtAFwAIgAsACAAXAAiAFQAYQBiAGwAZQAgADYAIABpAHMAIABuAG8AdAAgAGEAcABwAGwAaQBjAGEAYgBsAGUAIAB0AG8AIABlAHQAaABhAG4AZQAuACAAUwBlAGUAIABUAGEAYgBsAGUAIAA3ACAASQBuAGQAaQByAGUAYwB0ACAAKABTAGMAbwBwAGUAIAAzACkAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB0AGgAZQAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAG8AZgAgAGUAdABoAGEAbgBlAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAFwAIgBDACAAPQAgAEMAbwBuAGYAaQBkAGUAbgB0AGkAYQBsAC4AIABTAGMAbwBwAGUAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAVABhAHMAbQBhAG4AaQBhACAAYQBuAGQAIAB0AGgAZQAgAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5ACAAYQByAGUAIABuAG8AdAAgAGEAdgBhAGkAbABhAGIAbABlACAAZAB1AGUAIAB0AG8AIABjAG8AbgBmAGkAZABlAG4AdABpAGEAbABpAHQAeQAgAGMAbwBuAHMAdAByAGEAaQBuAHQAcwAgAHQAaABhAHQAIABhAHIAaQBzAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAZgByAG8AbQAgAHQAaABlACAAdQBzAGUAIABvAGYAIABhACAAbABpAG0AaQB0AGUAZAAgAG4AdQBtAGIAZQByACAAbwBmACAATgBHAEUAUgAgAGQAYQB0AGEAIABpAG4AcAB1AHQAcwAuACAASQB0ACAAaQBzACAAcwB1AGcAZwBlAHMAdABlAGQAIAB0AGgAYQB0ACAAZgBvAHIAIABUAGEAcwBtAGEAbgBpAGEAIAB0AGgAZQAgAHUAcwBlACAAbwBmACAAdABoAGUAIABWAGkAYwB0AG8AcgBpAGEAbgAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABpAHMAIABhAHAAcAByAG8AcAByAGkAYQB0AGUALABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgB3AGgAaQBsAGUAIABmAG8AcgAgAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5ACAAdABoAGUAIAB1AHMAZQAgAG8AZgAgAHQAaABlACAAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAaQBzACAAYQBwAHAAcgBvAHAAcgBpAGEAdABlAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIALQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGQAbwAgAG4AbwB0ACAAaQBuAGMAbAB1AGQAZQAgAGYAdQBnAGkAdABpAHYAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGwAZQBhAGsAYQBnAGUAIABmAHIAbwBtACAAbABvAHcAIABwAHIAZQBzAHMAdQByAGUAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAIABkAGkAcwB0AHIAaQBiAHUAdABpAG8AbgAgAHAAaQBwAGUAbABpAG4AZQAgAG4AZQB0AHcAbwByAGsAcwAgAHcAaABpAGwAZQAgAHQAaABvAHMAZQAgAGYAcgBvAG0AIABoAGkAZwBoACAAcAByAGUAcwBzAHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAGcAYQBzACAAbgBlAHQAdwBvAHIAawBzACAAYQByAGUAIABjAG8AbgBzAGkAZABlAHIAZQBkACAAbgBlAGcAbABpAGcAaQBiAGwAZQAuAFwAIgBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABhAG4AZAAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFMAdABhAHQAaQBvAG4AYQByAHkAIABsAGkAcQB1AGkAZAAgAGYAdQBlAGwAcwBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBGAHUAZQBsACAAcwBjAG8AcABlACAAMQAgAGEAbgBkACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAUwB0AGEAdABpAG8AbgBhAHIAeQAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzAFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARABpAHIAZQBjAHQAIAAoAFMAYwBvAHAAZQAgADEAKQAgAGEAbgBkACAAaQBuAGQAaQByAGUAYwB0ACAAKABzAGMAbwBwAGUAIAAzACkAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB0AGgAZQAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAG8AZgAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzACwAIABpAG4AYwBsAHUAZABpAG4AZwAgAGMAZQByAHQAYQBpAG4AIABwAGUAdAByAG8AbABlAHUAbQAgAGIAYQBzAGUAZAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzAC4AXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAQQBjAGMAbwB1AG4AdABzACAARgBhAGMAdABvAHIAcwAgADIAMAAyADUAIAAtACAAVABhAGIAbABlACAAOABcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgA1ACwAIAA4ACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAdQBlAGwAIABjAG8AbQBiAHUAcwB0AGUAZABcACIALAAgAFwAIgBFAG4AZQByAGcAeQAgAEMAbwBuAHQAZQBuAHQAIABGAGEAYwB0AG8AcgAgACgARwBKACAAcABlAHIAIAB1AG4AaQB0ACAAbwBmACAAZgB1AGUAbAApAFwAIgAsACAAXAAiAEYAdQBlAGwAIAB1AG4AaQB0AFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAEMATwAyAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAEMASAA0AFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAE4AMgBPAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgAgACgAawBnACAAQwBPADIAIAAtACAAZQAgAC8AIABHAEoAKQAgAEMAbwBtAGIAaQBuAGUAZAAgAGcAYQBzAGUAcwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABlAHQAcgBvAGwAZQB1AG0AIABiAGEAcwBlAGQAIABvAGkAbABzACAAKABvAHQAaABlAHIAIAB0AGgAYQBuACAAcABlAHQAcgBvAGwAZQB1AG0AIABiAGEAcwBlAGQAIABvAGkAbAAgAHUAcwBlAGQAIABhAHMAIABmAHUAZQBsACkALAAgAGUALgBnAC4AIABsAHUAYgByAGkAYwBhAG4AdABzAFwAIgAsACAAMwA4AC4AOAAsACAAXAAiAGsAbABcACIALAAgADEAMwAuADkALAAgADAALgAwACwAIAAwAC4AMAAsACAAMQAzAC4AOQAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAAZQB0AHIAbwBsAGUAdQBtACAAYgBhAHMAZQBkACAAZwByAGUAYQBzAGUAcwBcACIALAAgADMAOAAuADgALAAgAFwAIgBrAGwAXAAiACwAIAAzAC4ANQAsACAAMAAuADAALAAgADAALgAwACwAIAAzAC4ANQAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAcgB1AGQAZQAgAG8AaQBsACAAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAdQBkAGUAIABvAGkAbAAgAGMAbwBuAGQAZQBuAHMAYQB0AGUAcwBcACIALAAgADQANQAuADMALAAgAFwAIgB0AFwAIgAsACAANgA5AC4ANgAsACAAMAAuADAAOAAsACAAMAAuADIALAAgADYAOQAuADgAOAAsACAAXAAiAE4ARQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAIABuAGEAdAB1AHIAYQBsACAAZwBhAHMAIABsAGkAcQB1AGkAZABzAFwAIgAsACAANAA2AC4ANQAsACAAXAAiAHQAXAAiACwAIAA2ADEALgAwACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAANgAxAC4AMgA4ACwAIABcACIATgBFAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAdQB0AG8AbQBvAHQAaQB2AGUAIABnAGEAcwBvAGwAaQBuAGUAIAAvACAAcABlAHQAcgBvAGwAIAAoAG8AdABoAGUAcgAgAHQAaABhAG4AIABmAG8AcgAgAHUAcwBlACAAYQBzACAAZgB1AGUAbAAgAGkAbgAgAGEAbgAgAGEAaQByAGMAcgBhAGYAdAApAFwAIgAsACAAMwA0AC4AMgAsACAAXAAiAGsATABcACIALAAgADYANwAuADQALAAgADAALgAyACwAIAAwAC4AMgAsACAANgA3AC4AOAAwACwAIAAxADcALgAyADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQB2AGkAYQB0AGkAbwBuACAAZwBhAHMAbwBsAGkAbgBlAFwAIgAsACAAMwAzAC4AMQAsACAAXAAiAGsATABcACIALAAgADYANwAsACAAMAAuADIALAAgADAALgAyACwAIAA2ADcALgA0ADAALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBLAGUAcgBvAHMAZQBuAGUAIAAoAG8AdABoAGUAcgAgAHQAaABhAG4AIABmAG8AcgAgAHUAcwBlACAAYQBzACAAZgB1AGUAbAAgAGkAbgAgAGEAbgAgAGEAaQByAGMAcgBhAGYAdAApAFwAIgAsACAAMwA3AC4ANQAsACAAXAAiAGsATABcACIALAAgADYAOAAuADkALAAgADAALgAwADEALAAgADAALgAyACwAIAA2ADkALgAxADEALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAHYAaQBhAHQAaQBvAG4AIAB0AHUAcgBiAGkAbgBlACAAZgB1AGUAbAAgAC8AIABrAGUAcgBvAHMAZQBuAGUAXAAiACwAIAAzADYALgA4ACwAIABcACIAawBMAFwAIgAsACAANgA5AC4ANgAsACAAMAAuADAAMgAsACAAMAAuADIALAAgADYAOQAuADgAMgAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHQAaQBuAGcAIABvAGkAbABcACIALAAgADMANwAuADMALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA1ACwAIAAwAC4AMAAzACwAIAAwAC4AMgAsACAANgA5AC4ANwAzACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIARABpAGUAcwBlAGwAIABvAGkAbABcACIALAAgADMAOAAuADYALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA5ACwAIAAwAC4AMQAsACAAMAAuADIALAAgADcAMAAuADIAMAAsACAAMQA3AC4AMwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAdQBlAGwAIABvAGkAbABcACIALAAgADMAOQAuADcALAAgAFwAIgBrAEwAXAAiACwAIAA3ADMALgA2ACwAIAAwAC4AMAA0ACwAIAAwAC4AMgAsACAANwAzAC4AOAA0ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABhAHIAbwBtAGEAdABpAGMAIABoAHkAZAByAG8AYwBhAHIAYgBvAG4AcwBcACIALAAgADMANAAuADQALAAgAFwAIgBrAEwAXAAiACwAIAA2ADkALgA3ACwAIAAwAC4AMAAzACwAIAAwAC4AMgAsACAANgA5AC4AOQAzACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwBvAGwAdgBlAG4AdABzADoAIABtAGkAbgBlAHIAYQBsACAAdAB1AHIAcABlAG4AdABpAG4AZQAgAG8AcgAgAHcAaABpAHQAZQAgAHMAcABpAHIAaQB0AHMAXAAiACwAIAAzADQALgA0ACwAIABcACIAawBMAFwAIgAsACAANgA5AC4ANwAsACAAMAAuADAAMwAsACAAMAAuADIALAAgADYAOQAuADkAMwAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAaQBxAHUAZQBmAGkAZQBkACAAcABlAHQAcgBvAGwAZQB1AG0AIABnAGEAcwAgACgATABQAEcAKQBcACIALAAgADIANQAuADcALAAgAFwAIgBrAEwAXAAiACwAIAA2ADAALgAyACwAIAAwAC4AMgAsACAAMAAuADIALAAgADYAMAAuADYAMAAsACAAMgAwAC4AMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE4AYQBwAGgAdABoAGEAXAAiACwAIAAzADEALgA0ACwAIABcACIAawBMAFwAIgAsACAANgA5AC4AOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAANgA5AC4AOAAyACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABlAHQAcgBvAGwAZQB1AG0AIABjAG8AawBlAFwAIgAsACAAMwA0AC4AMgAsACAAXAAiAHQAXAAiACwAIAA5ADIALgA2ACwAIAAwAC4AMAA4ACwAIAAwAC4AMgAsACAAOQAyAC4AOAA4ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgBlAGYAaQBuAGUAcgB5ACAAZwBhAHMAIABhAG4AZAAgAGwAaQBxAHUAaQBkAHMAXAAiACwAIAA0ADIALgA5ACwAIABcACIAdABcACIALAAgADUANAAuADcALAAgADAALgAwADMALAAgADAALgAwADMALAAgADUANAAuADcANgAsACAAMQA4AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBmAGkAbgBlAHIAeQAgAGMAbwBrAGUAXAAiACwAIAAzADQALgAyACwAIABcACIAdABcACIALAAgADkAMgAuADYALAAgADAALgAwADgALAAgADAALgAyACwAIAA5ADIALgA4ADgALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAdAByAG8AbABlAHUAbQAgAGIAYQBzAGUAZAAgAHAAcgBvAGQAdQBjAHQAcwAgAG8AdABoAGUAcgAgAHQAaABhAG4AIABtAGUAbgB0AGkAbwBuAGUAZAAgAGkAbgAgAHQAaABlACAAaQB0AGUAbQBzACAAYQBiAG8AdgBlAFwAIgAsACAAMwA0AC4ANAAsACAAXAAiAGsATABcACIALAAgADYAOQAuADgALAAgADAALgAwADIALAAgADAALgAxACwAIAA2ADkALgA5ADIALAAgADEAOAAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBCAGkAbwBkAGkAZQBzAGUAbABcACIALAAgADMANAAuADYALAAgAFwAIgBrAEwAXAAiACwAIAAwAC4AMAAsACAAMAAuADAAOAAsACAAMAAuADIALAAgADAALgAyADgALAAgAFwAIgBOAEUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIARQB0AGgAYQBuAG8AbAAgAGYAbwByACAAdQBzAGUAIABhAHMAIABhACAAZgB1AGUAbAAgAGkAbgAgAGEAbgAgAGkAbgB0AGUAcgBuAGEAbAAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABlAG4AZwBpAG4AZQBcACIALAAgADIAMwAuADQALAAgAFwAIgBrAEwAXAAiACwAIAAwAC4AMAAsACAAMAAuADAAOAAsACAAMAAuADIALAAgADAALgAyADgALAAgAFwAIgBOAEUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQgBpAG8AZgB1AGUAbABzACAAbwB0AGgAZQByACAAdABoAGEAbgAgAHQAaABvAHMAZQAgAG0AZQBuAHQAaQBvAG4AZQBkACAAaQBuACAAdABoAGUAIABpAHQAZQBtAHMAIABhAGIAbwB2AGUAIABhAG4AZAAgAGIAZQBsAG8AdwBcACIALAAgADIAMwAuADQALAAgAFwAIgBrAEwAXAAiACwAIAAwAC4AMAAsACAAMAAuADAAOAAsACAAMAAuADIALAAgADAALgAyADgALAAgAFwAIgBOAEUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABhAHYAaQBhAHQAaQBvAG4AIABrAGUAcgBvAHMAZQBuAGUAXAAiACwAIAAzADYALgA4ACwAIABcACIAawBMAFwAIgAsACAAMAAuADAALAAgADAALgAwADIALAAgADAALgAyACwAIAAwAC4AMgAyACwAIABcACIATgBFAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBuAGUAdwBhAGIAbABlACAAZABpAGUAcwBlAGwAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBMAFwAIgAsACAAMAAuADAALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADMAMAAsACAAXAAiAE4ARQBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgACcATgBFACcAIAB2AGEAbAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAGEAcwAgAHoAZQByAG8AIABmAG8AcgAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgBzAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ARgB1AGUAbAAgAHMAYwBvAHAAZQAgADEAIABhAG4AZAAgADMAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAALQAgAFQAcgBhAG4AcwBwAG8AcgB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBGAHUAZQBsACAAcwBjAG8AcABlACAAMQAgAGEAbgBkACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAAVAByAGEAbgBzAHAAbwByAHQAXAAiACkAKQA7AFwAbgBcAG4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8ARABlAHMAYwByAGkAcAB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARABpAHIAZQBjAHQAIAAoAHMAYwBvAHAAZQAgADEAKQAgAGEAbgBkACAAaQBuAGQAaQByAGUAYwB0ACAAKABzAGMAbwBwAGUAIAAzACkAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIAB0AGgAZQAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAG8AZgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZgB1AGUAbABzACAAaQBuACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAcQB1AGkAcABtAGUAbgB0AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAA5AFwAIgApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgA2ACwAIAAxADAALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVAByAGEAbgBzAHAAbwByAHQAIAB0AHkAcABlAFwAIgAsACAAXAAiAEYAdQBlAGwAIABjAG8AbQBiAHUAcwB0AGUAZABcACIALAAgAFwAIgBFAG4AZQByAGcAeQAgAEMAbwBuAHQAZQBuAHQAIABGAGEAYwB0AG8AcgAoAEcASgAgAHAAZQByACAAdQBuAGkAdAAgAG8AZgAgAGYAdQBlAGwAKQBcACIALAAgAFwAIgBGAHUAZQBsACAAdQBuAGkAdABcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAE8AMgBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAEgANABcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABOADIATwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAIABDAG8AbQBiAGkAbgBlAGQAIABnAGEAcwBlAHMAXAAiACwAIABcACIAUwBjAG8AcABlACAAMwAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAEcASgApAFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAHMAIABhAG4AZAAgAGwAaQBnAGgAdAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIARwBhAHMAbwBsAGkAbgBlAFwAIgAsACAAMwA0AC4AMgAsACAAXAAiAGsAbABcACIALAAgADYANwAuADQALAAgADAALgAwADIALAAgADAALgAyACwAIAA2ADcALgA2ADIALAAgADEANwAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBzACAAYQBuAGQAIABsAGkAZwBoAHQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsACAAbwBpAGwAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBsAFwAIgAsACAANgA5AC4AOQAsACAAMAAuADAAMQAsACAAMAAuADUALAAgADcAMAAuADQAMQAsACAAMQA3AC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAHMAIABhAG4AZAAgAGwAaQBnAGgAdAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIATABpAHEAdQBlAGYAaQBlAGQAIABwAGUAdAByAG8AbABlAHUAbQAgAGcAYQBzACAAKABMAFAARwApAFwAIgAsACAAMgA2AC4AMgAsACAAXAAiAGsAbABcACIALAAgADYAMAAuADIALAAgADAALgA1ACwAIAAwAC4AMwAsACAANgAxAC4AMAAwACwAIAAyADAALgAyACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBGAHUAZQBsACAAbwBpAGwAXAAiACwAIAAzADkALgA3ACwAIABcACIAawBsAFwAIgAsACAANwAzAC4ANgAsACAAMAAuADAAOAAsACAAMAAuADUALAAgADcANAAuADEAOAAsACAAMQA4AC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAHMAIABhAG4AZAAgAGwAaQBnAGgAdAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIARQB0AGgAYQBuAG8AbABcACIALAAgADIAMwAuADQALAAgAFwAIgBrAGwAXAAiACwAIAAwAC4AMAAsACAAMAAuADIALAAgADAALgAyACwAIAAwAC4ANAAsACAAXAAiAE4ARQBcACIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAGEAcgBzACAAYQBuAGQAIABsAGkAZwBoAHQAIABjAG8AbQBtAGUAcgBjAGkAYQBsACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEIAaQBvAGQAaQBlAHMAZQBsAFwAIgAsACAAMwA0AC4ANgAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AOAAsACAAMQAuADcALAAgADIALgA1ACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAHMAIABhAG4AZAAgAGwAaQBnAGgAdAAgAGMAbwBtAG0AZQByAGMAaQBhAGwAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABkAGkAZQBzAGUAbABcACIALAAgADMAOAAuADYALAAgAFwAIgBrAGwAXAAiACwAIAAwAC4AMAAsACAAMAAuADAAMQAsACAAMAAuADUALAAgADAALgA1ADEALAAgAFwAIgBOAEUAXAAiACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBhAHIAcwAgAGEAbgBkACAAbABpAGcAaAB0ACAAYwBvAG0AbQBlAHIAYwBpAGEAbAAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBPAHQAaABlAHIAIABiAGkAbwBmAHUAZQBsAHMAXAAiACwAIAAyADMALgA0ACwAIABcACIAawBsAFwAIgAsACAAMAAuADAALAAgADAALgA4ACwAIAAxAC4ANwAsACAAMgAuADUALAAgAFwAIgBOAEUAXAAiACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABpAGcAaAB0ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBDAG8AbQBwAHIAZQBzAHMAZQBkACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAFwAIgAsACAAMAAuADAAMwA5ADMALAAgAFwAIgBtADMAXAAiACwAIAA1ADEALgA0ACwAIAA3AC4AMwAsACAAMAAuADMALAAgADUAOQAuADAALAAgADEAOAAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGkAZwBoAHQAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAZQBmAGkAZQBkACAAbgBhAHQAdQByAGEAbAAgAGcAYQBzAFwAIgAsACAAMgA1AC4AMwAsACAAXAAiAGsAbABcACIALAAgADUAMQAuADQALAAgADcALgAzACwAIAAwAC4AMwAsACAANQA5AC4AMAAsACAAMQA4AC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIAQwBvAG0AcAByAGUAcwBzAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwBcACIALAAgADAALgAwADMAOQAzACwAIABcACIAbQAzAFwAIgAsACAANQAxAC4ANAAsACAAMgAuADgALAAgADAALgAzACwAIAA1ADQALgA1ACwAIAAxADgALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABlAGEAdgB5ACAAZAB1AHQAeQAgAHYAZQBoAGkAYwBsAGUAcwBcACIALAAgAFwAIgBMAGkAcQB1AGUAZgBpAGUAZAAgAG4AYQB0AHUAcgBhAGwAIABnAGEAcwBcACIALAAgADIANQAuADMALAAgAFwAIgBrAGwAXAAiACwAIAA1ADEALgA0ACwAIAAyAC4AOAAsACAAMAAuADMALAAgADUANAAuADUALAAgADEAOAAuADAALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAYQB2AHkAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsACAAbwBpAGwAIAAtACAARQB1AHIAbwAgAGkAdgAgAG8AcgAgAGgAaQBnAGgAZQByAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADYAOQAuADkALAAgADAALgAwADcALAAgADAALgA0ACwAIAA3ADAALgAzADcALAAgADEANwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAYQB2AHkAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsACAAbwBpAGwAIAAtACAARQB1AHIAbwAgAGkAaQBpAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADYAOQAuADkALAAgADAALgAxACwAIAAwAC4ANAAsACAANwAwAC4ANAAsACAAMQA3AC4AMwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIARABpAGUAcwBlAGwAIABvAGkAbAAgAC0AIABFAHUAcgBvACAAaQBcACIALAAgADMAOAAuADYALAAgAFwAIgBrAGwAXAAiACwAIAA2ADkALgA5ACwAIAAwAC4AMgAsACAAMAAuADQALAAgADcAMAAuADUALAAgADEANwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAYQB2AHkAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAFIAZQBuAGUAdwBhAGIAbABlACAAZABpAGUAcwBlAGwAIAATICAARQB1AHIAbwAgAGkAdgAgAG8AcgAgAGgAaQBnAGgAZQByAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AMAA3ACwAIAAwAC4ANAAsACAAMAAuADQANwAsACAAXAAiAE4ARQBcACIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAYQB2AHkAIABkAHUAdAB5ACAAdgBlAGgAaQBjAGwAZQBzAFwAIgAsACAAXAAiAFIAZQBuAGUAdwBhAGIAbABlACAAZABpAGUAcwBlAGwAIAATICAARQB1AHIAbwAgAGkAaQBpAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AMQAsACAAMAAuADQALAAgADAALgA1ACwAIABcACIATgBFAFwAIgAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAGQAdQB0AHkAIAB2AGUAaABpAGMAbABlAHMAXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABkAGkAZQBzAGUAbAAgABMgIABFAHUAcgBvACAAaQBcACIALAAgADMAOAAuADYALAAgAFwAIgBrAGwAXAAiACwAIAAwAC4AMAAsACAAMAAuADIALAAgADAALgA0ACwAIAAwAC4ANgAsACAAXAAiAE4ARQBcACIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAHYAaQBhAHQAaQBvAG4AXAAiACwAIABcACIARwBhAHMAbwBsAGkAbgBlACAAZgBvAHIAIAB1AHMAZQAgAGEAcwAgAGYAdQBlAGwAIABpAG4AIABhAG4AIABhAGkAcgBjAHIAYQBmAHQAXAAiACwAIAAzADMALgAxACwAIABcACIAawBsAFwAIgAsACAANgA3AC4AMAAsACAAMAAuADAANgAsACAAMAAuADYALAAgADYANwAuADYANgAsACAAMQA4AC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ADoAIABUAGEAYgBsAGUAIAA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAdgBpAGEAdABpAG8AbgBcACIALAAgAFwAIgBLAGUAcgBvAHMAZQBuAGUAIABmAG8AcgAgAHUAcwBlACAAYQBzACAAZgB1AGUAbAAgAGkAbgAgAGEAbgAgAGEAaQByAGMAcgBhAGYAdABcACIALAAgADMANgAuADgALAAgAFwAIgBrAGwAXAAiACwAIAA2ADkALgA2ACwAIAAwAC4AMAAxACwAIAAwAC4ANgAsACAANwAwAC4AMgAxACwAIAAxADgALgAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAOgAgAFQAYQBiAGwAZQAgADkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQB2AGkAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFIAZQBuAGUAdwBhAGIAbABlACAAYQB2AGkAYQB0AGkAbwBuACAAawBlAHIAbwBzAGUAbgBlAFwAIgAsACAAMwA2AC4AOAAsACAAXAAiAGsAbABcACIALAAgADAALgAwACwAIAAwAC4AMAAxACwAIAAwAC4ANgAsACAAMAAuADYAMQAsACAAXAAiAE4ARQBcACIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQA6ACAAVABhAGIAbABlACAAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcwBzAGUAbABzAFwAIgAsACAAXAAiAEcAYQBzAG8AbABpAG4AZQBcACIALAAgADMANAAuADIALAAgAFwAIgBrAEwAXAAiACwAIAA2ADcALgA0ACwAIAAxADAALgAxACwAIAAwAC4AMwAsACAAXAAiAFwAIgAsACAAMQA3AC4AMgAsACAAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMgAuADEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBlAHMAcwBlAGwAcwBcACIALAAgAFwAIgBEAGkAZQBzAGUAbAAgAG8AaQBsAFwAIgAsACAAMwA4AC4ANgAsACAAXAAiAGsATABcACIALAAgADYAOQAuADkALAAgADAALgAyACwAIAAwAC4ANQAsACAAXAAiAFwAIgAsACAAMQA3AC4AMwAsACAAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMgAuADEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBlAHMAcwBlAGwAcwBcACIALAAgAFwAIgBGAHUAZQBsACAATwBpAGwAXAAiACwAIAAzADkALgA3ACwAIABcACIAawBMAFwAIgAsACAANwAzAC4ANgAsACAAMAAuADIALAAgADAALgA1ACwAIABcACIAXAAiACwAIAAxADgALgAwACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAyAC4AMQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBPAGYAZgAtAHIAbwBhAGQAIABBAGcAcgBpAGMAdQBsAHQAdQByAGUAIABhAG4AZAAgAGYAbwByAGUAcwB0AHIAeQAgAGUAcQB1AGkAcABtAGUAbgB0AFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsACAAbwBpAGwAXAAiACwAIAAzADgALgA2ACwAIABcACIAawBMAFwAIgAsACAANgA5AC4AOQAsACAAMAAuADMALAAgADAALgA1ACwAIABcACIAXAAiACwAIAAxADcALgAzACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAyAC4AMQBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIAAnAE4ARQAnACAAdgBhAGwAdQBlAHMAIAByAGUAdAB1AHIAbgBlAGQAIABhAHMAIAB6AGUAcgBvACAAZgBvAHIAIABjAGEAbABjAHUAbABhAHQAaQBvAG4AcwAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBGAHUAZQBsACAAcwBjAG8AcABlACAAMQAgAGEAbgBkACAAMwAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIAAtACAATwBmAGYALQByAGEAZAAgAGUAcQB1AGkAcABtAGUAbgB0ACAAYQBuAGQAIAB2AGUAcwBzAGUAbABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEYAdQBlAGwAIABzAGMAbwBwAGUAIAAxACAAYQBuAGQAIAAzACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAC0AIABPAGYAZgAtAHIAbwBhAGQAIABlAHEAdQBpAHAAbQBlAG4AdAAgAGEAbgBkACAAdgBlAHMAcwBlAGwAcwBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEQAaQByAGUAYwB0ACAAKABzAGMAbwBwAGUAIAAxACkAIABhAG4AZAAgAGkAbgBkAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMwApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIABmAHUAZQBsAHMAIABpAG4AIABvAGYAZgAtAHIAbwBhAGQAIABlAHEAdQBpAHAAbQBlAG4AdAAgAGEAbgBkACAAdgBlAHMAcwBlAGwAcwBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADQALgAyAC4AMQBcACIAKQApADsAXABuAFwAbgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAANwAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAYQBuAHMAcABvAHIAdAAgAHQAeQBwAGUAIAB0AFwAIgAsACAAXAAiAEYAdQBlAGwAIAB0AHkAcABlACAAcQBcACIALAAgAFwAIgBFAEMAVAByAGEAbgBzACwAcQAgACgARwBKAC8AawBMACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAEMATwAyACAARQBGAFQAcgBhAG4ALAAxACwAdABxAGcAIAAoAGsAZwAgAEMATwAyAC0AZQAvAEcASgApAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABDAEgANAAgAEUARgBUAHIAYQBuACwAMQAsAHQAZwBnACAAKABrAGcAIABDAE8AMgAtAGUALwBHAEoAKQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAxACAATgAyAE8AIABFAEYAVAByAGEAbgAsADEALAB0AGcAZwAgACgAawBnACAAQwBPADIALQBlAC8ARwBKACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMwAgAEUARgBUAHIAYQBuAHMALAAzACwAcQAgACgAawBnACAAQwBPADIALQBlAC8ARwBKACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBlAHMAcwBlAGwAXAAiACwAIABcACIAUABlAHQAcgBvAGwAXAAiACwAIAAzADQALgAyACwAIAA2ADcALgA0ACwAIAAxADAALgAxACwAIAAwAC4AMwAsACAAMQA3AC4AMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAZQBzAHMAZQBsAFwAIgAsACAAXAAiAEQAaQBlAHMAZQBsAFwAIgAsACAAMwA4AC4ANgAsACAANgA5AC4AOQAsACAAMAAuADIALAAgADAALgA1ACwAIAAxADcALgAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVgBlAHMAcwBlAGwAXAAiACwAIABcACIARgB1AGUAbAAgAE8AaQBsAFwAIgAsACAAMwA5AC4ANwAsACAANwAzAC4ANgAsACAAMAAuADIALAAgADAALgA1ACwAIAAxADgALgAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIATwBmAGYALQByAG8AYQBkACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACAAYQBuAGQAIABmAG8AcgBlAHMAdAByAHkAIABlAHEAdQBpAHAAbQBlAG4AdABcACIALAAgAFwAIgBEAGkAZQBzAGUAbABcACIALAAgADMAOAAuADYALAAgADYAOQAuADkALAAgADAALgAzACwAIAAwAC4ANQAsACAAMQA3AC4AMwBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEYAdQBlAGwAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBGAHUAZQBsAF8ARwBlAHQAVAByAGEAbgBzAHAAbwByAHQARgB1AGUAbABTAHQAcgBpAG4AZwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALABcAG4AIAAgACAAIABMAEUARgBUACgAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsACAAXAAiACwAQwBlAGwAbAApACAALQAxACkAXABuACkAOwBcAG4AXABuAEYAdQBlAGwAXwBHAGUAdABTAHQAYQB0AGkAbwBuAGEAcgB5AEYAdQBlAGwAUwB0AHIAaQBuAGcAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAXABuACAAIAAgACAAUgBJAEcASABUACgAQwBlAGwAbAAsAEwARQBOACgAQwBlAGwAbAApAC0ARgBJAE4ARAAoAFwAIgAsACAAXAAiACwAQwBlAGwAbAApACkAXABuACkAOwBcAG4AXABuAEYAdQBlAGwAXwBUAG8AdABhAGwAQwBvAG4AcwB1AG0AcAB0AGkAbwBuAFwAbgA9ACAATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABGAHUAZQBsAEMAbwBuAHMAdQBtAHAAdABpAG8AbgBBAHIAcgBhAHkALAAgAEYAdQBlAGwAVQBzAGUAQQByAHIAYQB5ACwAIABGAHUAZQBsAFUAcwBlACwAIABGAHUAZQBsAFQAeQBwAGUAQQByAHIAYQB5ACwAIABGAHUAZQBsAFQAeQBwAGUALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAUwBVAE0AKABcAG4AIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAEYAdQBlAGwAQwBvAG4AcwB1AG0AcAB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAKABGAHUAZQBsAFQAeQBwAGUAQQByAHIAYQB5ACAAPQAgAEYAdQBlAGwAVAB5AHAAZQApACAAKgAgAFwAbgAgACAAIAAgACAAIAAgACAAKABGAHUAZQBsAFUAcwBlAEEAcgByAGEAeQAgAD0AIABGAHUAZQBsAFUAcwBlACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQAsAFwAbgAgACAAIAAgADAAXABuACAAIAApAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AOAA6ACAARgB1AGUAbAAgAFUAcwBlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADgALgAxACAARgB1AGUAbAAgAFUAcwBlACAALQAgAFQAcgBhAG4AcwBwAG8AcgB0ACAAZgB1AGUAbABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRACwAIABFAEMALAAgAEUARgAsAFwAbgAgACAAIAAgACgAUQAgACoAIABFAEMAIAAqACAARQBGACkAIAAqACAAMQAwACAAXgAgAC0AIAAzAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBmACAAZgB1AGUAbABzACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzAFwAbgBRACAAOgAgAEEAbQBvAHUAbgB0ACAAbwBmACAAZgB1AGUAbAAgAHQAeQBwAGUAIABxACAAYwBvAG0AYgB1AHMAdABlAGQAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAIAA6ACAAawBMAFwAbgBFAEMAIAA6ACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAIAA6ACAARwBKAC8AawBMAFwAbgBFAEYAIAA6ACAAUwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzACAAZgBvAHIAIABlAGEAYwBoACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzACAAOgAgAGsAZwAgAEMATwAyAGUAIAAvACAARwBKAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwBUAHIAYQBuAHMAdABxACwAIABFAEMAXwBUAHIAYQBuAHMAcQAsACAARQBGAF8AVAByAGEAbgBzADEAdABxAGcALABcAG4AIAAgACAAIABWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACgAUQBfAFQAcgBhAG4AcwB0AHEALAAgAEUAQwBfAFQAcgBhAG4AcwBxACwAIABFAEYAXwBUAHIAYQBuAHMAMQB0AHEAZwApAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBmACAAZgB1AGUAbABzACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgAtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAOAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIAAyAC4AMwAgAEUAcwB0AGkAbQBhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB0AHIAYQBuAHMAcABvAHIAdAAgAGYAdQBlAGwAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBnAD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwB0ACAAXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBxAFwAXABsAGUAZgB0ACgAUQBfAHsAVAByAGEAbgBzACwAdABxAH0AXABcAHQAaQBtAGUAcwAgAEUAQwBfAHsAVAByAGEAbgBzACwAcQB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFQAcgBhAG4AcwAsADEALAB0AHEAZwB9AFwAXAByAGkAZwBoAHQAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAFQAcgBhAG4AcwB0AHEAXAAiACwAIABcACIAQQBtAG8AdQBuAHQAIABvAGYAIABmAHUAZQBsACAAdAB5AHAAZQAgAHEAIABjAG8AbQBiAHUAcwB0AGUAZAAgAGYAbwByACAAdAByAGEAbgBzAHAAbwByAHQAIABlAG4AZQByAGcAeQAgAHAAdQByAHAAbwBzAGUAcwBcACIALAAgAFwAIgBWAGEAcgBpAGUAcwAgAGIAYQBzAGUAZAAgAG8AbgAgAGYAdQBlAGwAIAB0AHkAcABlADoAIABrAEwALAAgAG0AMwAsACAARwBKAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAF8AVAByAGEAbgBzAHEAXAAiACwAIABcACIARQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAcgBhAG4AcwBwAG8AcgB0ACAAZQBuAGUAcgBnAHkAIABwAHUAcgBwAG8AcwBlAHMAXAAiACwAIABcACIARwBKACAALwAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AVAByAGEAbgBzADEAdABxAGcAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB0AHIAYQBuAHMAcABvAHIAdAAgAGUAbgBlAHIAZwB5ACAAcAB1AHIAcABvAHMAZQBzACAAZgBvAHIAIABlAGEAYwBoACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAGsAZwAgAEMATwAyAGUAIAAvACAARwBKAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcQBcACIALAAgAFwAIgBGAHUAZQBsACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBhAG4AcwBcACIALAAgAFwAIgBUAHIAYQBuAHMAcABvAHIAdAAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAXAAiACwAIABcACIAUwBjAG8AcABlACAAMQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgBvAHIAIABlAGEAYwBoACAARwBIAEcAIABmAHIAbwBtACAAdABoAGUAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AZgAgAGYAdQBlAGwAcwBcAG4AUQAgADoAIABBAG0AbwB1AG4AdAAgAG8AZgAgAGYAdQBlAGwAIAB0AHkAcABlACAAcQAgAHUAcwBlAGQAIABmAG8AcgAgAHMAdABhAHQAaQBvAG4AYQByAHkAIABjAG8AbQBiAHUAcwB0AGkAbwBuACAAbwBwAGUAcgBhAHQAaQBvAG4AcwAgADoAIABrAEwAXABuAEUAQwAgADoAIABFAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABvAHAAZQByAGEAdABpAG8AbgBzACAAOgAgAEcASgAvAGsATABcAG4ARQBGACAAOgAgAFMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIAA6ACAAawBnACAAQwBPADIAZQAgAC8AIABHAEoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AUwBDAHEALAAgAEUAQwBfAFMAQwBxACwAIABFAEYAXwBTAEMAMQBxAGcALABcAG4AIAAgACAAIABWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACgAUQBfAFMAQwBxACwAIABFAEMAXwBTAEMAcQAsACAARQBGAF8AUwBDADEAcQBnACkAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAbwByACAAZQBhAGMAaAAgAEcASABHACAAZgByAG8AbQAgAHQAaABlACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABvAGYAIABmAHUAZQBsAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGcAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgAtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA4AC4AMgAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABOAGEAdABpAG8AbgBhAGwAIABHAHIAZQBlAG4AaABvAHUAcwBlACAAQQBjAGMAbwB1AG4AdABzACAARgBhAGMAdABvAHIAcwAgADIAMAAyADUAIAAtACAAMgAuADIAIABFAHMAdABpAG0AYQB0AGkAbgBnACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGUAbgBlAHIAZwB5ACAAcwBvAHUAcgBjAGUAcwAgAC0AIABDAGEAbABjAHUAbABhAHQAaQBuAGcAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AZgAgAGwAaQBxAHUAaQBkACAAZgB1AGUAbABzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdAAgAFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AcQBcAFwAbABlAGYAdAAoAFEAXwB7AFMAQwAsAHEAfQBcAFwAdABpAG0AZQBzACAARQBDAF8AewBTAEMALABxAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAUwBDACwAMQAsAHEAZwB9AFwAXAByAGkAZwBoAHQAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AUwBDAHEAXAAiACwAIABcACIAQQBtAG8AdQBuAHQAIABvAGYAIABmAHUAZQBsACAAdAB5AHAAZQAgAHEAIAB1AHMAZQBkACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIAVgBhAHIAaQBlAHMAIABiAGEAcwBlAGQAIABvAG4AIABmAHUAZQBsACAAdAB5AHAAZQA6ACAAawBMACwAIABtADMALAAgAEcASgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBfAFMAQwBxAFwAIgAsACAAXAAiAEUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABzAHQAYQB0AGkAbwBuAGEAcgB5ACAAYwBvAG0AYgB1AHMAdABpAG8AbgAgAG8AcABlAHIAYQB0AGkAbwBuAHMAXAAiACwAIABcACIARwBKACAALwAgAHUAbgBpAHQAIABvAGYAIABmAHUAZQBsAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AUwBDADEAcQBnAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABpAG8AbgBhAHIAeQAgAGMAbwBtAGIAdQBzAHQAaQBvAG4AIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAawBnACAAQwBPADIAZQAgAC8AIABHAEoAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBxAFwAIgAsACAAXAAiAEYAdQBlAGwAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBDAFwAIgAsACAAXAAiAFMAdABhAHQAaQBvAG4AYQByAHkAIABjAG8AbQBiAHUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAZwBcACIALAAgAFwAIgBHAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADEAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADkAOgAgAFIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAFUAcwBlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADkALgAxACAAUgBlAGYAcgBpAGcAZQByAGEAbgB0ACAAVQBzAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXABuAFQAaABlACAAdABvAHQAYQBsACAAZQBtAGkAcwBzAGkAbwBuAHMAIABvAGYAIAByAGUAZgByAGkAZwBlAHIAYQBuAHQAIABsAGUAYQBrAGkAbgBnACAAZAB1AHIAaQBuAGcAIABvAHAAZQByAGEAdABpAG8AbgAgACgAbgBvAHQAIABkAHUAcgBpAG4AZwAgAGkAbgBzAHQAYQBsAGwAYQB0AGkAbwBuACAAbwByACAAZABpAHMAcABvAHMAYQBsACkAXABuAEcAVwBQAFIAIAA6ACAARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABvAGYAIAByAGUAZgByAGkAZwBlAHIAYQBuAHQAIABSACAAOgAgAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXABuAGMAaABhAHIAZwBlAF8AUgBhACAAOgAgAEEAbQBvAHUAbgB0ACAAbwBmACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0ACAAUgAgAGMAbwBuAHQAYQBpAG4AZQBkACAAaQBuACAAYQBwAHAAbABpAGEAbgBjAGUAIABhACAAOgAgAGsAZwBcAG4AbABlAGEAawBhAGcAZQByAGEAdABlAF8AYQAgADoAIABQAHIAYwBlAG4AdABhAGcAZQAgAG8AZgAgAHQAbwB0AGEAbAAgAGMAaABhAHIAZwBlACAAbABlAGEAawBlAGQAIABmAHIAbwBtACAAYQBwAHAAbABpAGEAbgBjAGUAIABhACAAZQBhAGMAaAAgAHkAZQBhAHIAIAA6ACAAUABlAHIAYwBlAG4AdABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYwBoAGEAcgBnAGUAXwBSAGEALAAgAGwAZQBhAGsAYQBnAGUAcgBhAHQAZQBfAGEALABcAG4AIAAgACAAIAAoAGMAaABhAHIAZwBlAF8AUgBhACAAKgAgACgAbABlAGEAawBhAGcAZQByAGEAdABlAF8AYQAvADEAMAAwACkAKQAgACoAIAAxADAAIABeACAALQAgADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBHAFcAUABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AUgAsACAARwBXAFAAXwBSACwAXABuACAAIAAgACAAKAAoAEUAXwBSACAAKgAgADEAMABeADMAKQAgACoAIABHAFcAUABfAFIAKQAgACoAIAAxADAAXgAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABoAGUAIAB0AG8AdABhAGwAIABlAG0AaQBzAHMAaQBvAG4AcwAgAG8AZgAgAHIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAGwAZQBhAGsAaQBuAGcAIABkAHUAcgBpAG4AZwAgAG8AcABlAHIAYQB0AGkAbwBuACAAKABuAG8AdAAgAGQAdQByAGkAbgBnACAAaQBuAHMAdABhAGwAbABhAHQAaQBvAG4AIABvAHIAIABkAGkAcwBwAG8AcwBhAGwAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAGwAZQBhAGsAYQBnAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAQwBPADIALQBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAFIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0ACAAZwBhAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAC0AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAOQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIAAzAC4AMQAgAEUAcwB0AGkAbQBhAHQAaQBuAGcAIABpAG4AZAB1AHMAdAByAGkAYQBsACAAcAByAG8AYwBlAHMAcwBlAHMAIABlAG0AaQBzAHMAaQBvAG4AcwAgAC0AIABSAGUAZgByAGkAZwBlAHIAYQBuAHQAIABsAGUAYQBrAGEAZwBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAFIAZQBhAGQAYQBiAGwAZQBFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGMAaABhAHIAZwBlAF8AUgBhACAAKgAgACgAbABlAGEAawBhAGcAZQByAGEAdABlAF8AYQAvADEAMAAwACkAIAAqACAAMQAwACAAXgAgAC0AIAAzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBSACAAPQAgAFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AYQAgAFwAXABsAGUAZgB0ACgAIABjAGgAYQByAGcAZQBfAHsAUgBhAH0AIABcAFwAdABpAG0AZQBzACAAXABcAGYAcgBhAGMAewBsAGUAYQBrAGEAZwBlAFwAXAAsAHIAYQB0AGUAXwBhAH0AewAxADAAMAB9ACAAXABcAHIAaQBnAGgAdAApACAAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAEMATwAyAGUAIAA9ACAAXABcAGwAZQBmAHQAKABFAF8AUgAgAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7ADMAfQAgAFwAXAByAGkAZwBoAHQAKQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAFIAIABcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGMAaABhAHIAZwBlAF8AUgBhAFwAIgAsACAAXAAiAEEAbQBvAHUAbgB0ACAAbwBmACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0ACAAUgAgAGMAbwBuAHQAYQBpAG4AZQBkACAAaQBuACAAYQBwAHAAbABpAGEAbgBjAGUAIABhAFwAIgAsACAAXAAiAGsAZwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGwAZQBhAGsAYQBnAGUAcgBhAHQAZQBfAGEAXAAiACwAIABcACIAUAByAGMAZQBuAHQAYQBnAGUAIABvAGYAIAB0AG8AdABhAGwAIABjAGgAYQByAGcAZQAgAGwAZQBhAGsAZQBkACAAZgByAG8AbQAgAGEAcABwAGwAaQBhAG4AYwBlACAAYQAgAGUAYQBjAGgAIAB5AGUAYQByAFwAIgAsACAAXAAiAFAAZQByAGMAZQBuAHQAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBhAFwAIgAsACAAXAAiAEEAcABwAGwAaQBhAG4AYwBlACAAdAB5AHAAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAXAAiACwAIABcACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAF8AUgBcACIALAAgAFwAIgBUAG8AdABhAGwAIABlAG0AaQBzAHMAaQBvAG4AcwAgAG8AZgAgAHIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAFIAXAAiACwAIABcACIAdAAgAHIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAGcAYQBzAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAOQAuADEALgAxACAAKAAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAF8AUgBcACIALAAgAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAG8AZgAgAHIAZQBmAHIAaQBnAGUAcgBhAG4AdAAgAFIAXAAiACwAIABcACIARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABlAHEAdQBhAHQAaQBvAG4AIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0ACAAUgAgAHQAbwAgAEMATwAyAC0AZQAgAHUAcwBpAG4AZwAgAHQAaABlACAAcgBlAGYAcgBpAGcAZQByAGEAbgB0ACcAcwAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAKABHAFcAUAApAC4AXAAiACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AQQBwAHAAZQBuAGQAaQB4ACAAMgAgAEcAbABvAGIAYQBsACAAVwBhAHIAbQBpAG4AZwAgAFAAbwB0AGUAbgB0AGkAYQBsAHMAOgAgAFQAYQBiAGwAZQAgADIAMwAgAEcAbABvAGIAYQBsACAAVwBhAHIAbQBpAG4AZwAgAFAAbwB0AGUAbgB0AGkAYQBsAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEcAVwBQAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARwBsAG8AYgBhAGwAIABXAGEAcgBtAGkAbgBnACAAUABvAHQAZQBuAHQAaQBhAGwAcwBcACIAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABHAFcAUABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAALQAgAEEAcABwAGUAbgBkAGkAeAAgADIAIAAtACAAVABhAGIAbABlACAAMgAzAFwAIgApACkAOwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEcAVwBQAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzADkALAAgADUALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBoAGUAbQBpAGMAYQBsACAAZgBvAHIAbQB1AGwAYQBcACIALAAgAFwAIgBHAGwAbwBiAGEAbAAgAFcAYQByAG0AaQBuAGcAIABQAG8AdABlAG4AdABpAGEAbAAgACgAQQBSADUAKQBcACIALAAgAFwAIgBHAGEAcwAgAC0AIABGAEMAIABuAGEAbQBlAFwAIgAsACAAXAAiAEEAZABpAHQAaQBvAG4AYQBsACAAZABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQBcACIALAAgAFwAIgBDAE8AMgBcACIALAAgADEALAAgAFwAIgBDAE8AMgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBNAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAEMASAA0AFwAIgAsACAAMgA4ACwAIABcACIAQwBIADQAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQBcACIALAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ACwAIABcACIATgAyAE8AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwB1AGwAcABoAHUAcgAgAGgAZQB4AGEAZgBsAHUAbwByAGkAZABlAFwAIgAsACAAXAAiAFMARgA2AFwAIgAsACAAMgAzADUAMAAwACwAIABcACIAUwBGADYAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQAyADMAIAAoAFIALQAyADMAKQBcACIALAAgAFwAIgBDAEgARgAzAFwAIgAsACAAIAAxADIANAAwADAALAAgAFwAIgBIAEYAQwAtADIAMwBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEYAQwAtADMAMgAgACgAUgAtADMAMgApAFwAIgAsACAAXAAiAEMASAAyAEYAMgBcACIALAAgADYANwA3ACwAIABcACIASABGAEMALQAzADIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQA0ADEAIAAoAFIALQA0ADEAKQBcACIALAAgAFwAIgBDAEgAMwBGAFwAIgAsACAAIAAxADEANgAsACAAXAAiAEgARgBDAC0ANAAxAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgARgBDAC0ANAAzAC0AMQAwAG0AZQBlACAAKABSAC0ANAAzADEAMABtAGUAZQApAFwAIgAsACAAXAAiAEMANQBIADIARgAxADAAXAAiACwAIAAxADYANQAwACwAIABcACIASABGAEMALQA0ADMALQAxADAAbQBlAGUAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQAxADIANQAgACgAUgAtADEAMgA1ACkAXAAiACwAIABcACIAQwAyAEgARgA1AFwAIgAsACAAIAAzADEANwAwACwAIABcACIASABGAEMALQAxADIANQBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEYAQwAtADEAMwA0ACAAKABSAC0AMQAzADQAKQBcACIALAAgAFwAIgBDADIASAAyAEYANAAgACgAQwBIAEYAMgBDAEgARgAyACkAXAAiACwAIAAgADEAMQAyADAALAAgAFwAIgBIAEYAQwAtADEAMwA0AFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgARgBDAC0AMQAzADQAYQAgACgAUgAtADEAMwA0AGEAKQBcACIALAAgAFwAIgBDADIASAAyAEYANAAgACgAQwBIADIARgBDAEYAMwApAFwAIgAsACAAMQAzADAAMAAsACAAXAAiAEgARgBDAC0AMQAzADQAYQBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEYAQwAtADEANAAzACAAKABSAC0AMQA0ADMAKQBcACIALAAgAFwAIgBDADIASAAzAEYAMwAgACgAQwBIAEYAMgBDAEgAMgBGACkAXAAiACwAIAAzADIAOAAsACAAXAAiAEgARgBDAC0AMQA0ADMAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQAxADQAMwBhACAAKABSAC0AMQA0ADMAYQApAFwAIgAsACAAXAAiAEMAMgBIADMARgAzACAAKABDAEYAMwBDAEgAMwApAFwAIgAsACAANAA4ADAAMAAsACAAXAAiAEgARgBDAC0AMQA0ADMAYQBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEYAQwAtADEANQAyAGEAIAAoAFIALQAxADUAMgBhACkAXAAiACwAIABcACIAQwAyAEgANABGADIAIAAoAEMASAAzAEMASABGADIAKQBcACIALAAgADEAMwA4ACwAIABcACIASABGAEMALQAxADUAMgBhAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgARgBDAC0AMgAyADcAZQBhACAAKABSAC0AMgAyADcAZQBhACkAXAAiACwAIABcACIAQwAzAEgARgA3AFwAIgAsACAAMwAzADUAMAAsACAAXAAiAEgARgBDAC0AMgAyADcAZQBhAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgARgBDAC0AMgAzADYAZgBhACAAKABSAC0AMgAzADYAZgBhACkAXAAiACwAIABcACIAQwAzAEgAMgBGADYAXAAiACwAIAA4ADAANgAwACwAIABcACIASABGAEMALQAyADMANgBmAGEAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQAyADQANQBjAGEAIAAoAFIALQAyADQANQBjAGEAKQBcACIALAAgAFwAIgBDADMASAAzAEYANQBcACIALAAgADcAMQA2ACwAIABcACIASABGAEMALQAyADQANQBjAGEAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABGAEMALQAyADQANQBmAGEAIAAoAFIALQAyADQANQBmAGEAKQBcACIALAAgAFwAIgBDAEgARgAyAEMASAAyAEMARgAzAFwAIgAsACAAOAA1ADgALAAgAFwAIgBIAEYAQwAtADIANAA1AGYAYQBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEYAQwAtADMANgA1AG0AZgBjACAAKABSAC0AMwA2ADUAbQBmAGMAKQBcACIALAAgAFwAIgBDAEgAMwBDAEYAMgBDAEgAMgBDAEYAMwBcACIALAAgADgAMAA0ACwAIABcACIASABGAEMALQAzADYANQBtAGYAYwBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEMARgBDAC0AMgAyACAAKABSAC0AMgAyACkAXAAiACwAIABcACIAQwBIAEMAbABGADIAXAAiACwAIAAxADcANgAwACwAIABcACIASABDAEYAQwAtADIAMgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEMARgBDAC0AMQAyADMAIAAoAFIALQAxADIAMwApAFwAIgAsACAAXAAiAEMASABDAGwAMgAyAEMARgAzAFwAIgAsACAANwA5ACwAIABcACIASABDAEYAQwAtADEAMgAzAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAQwBGAEMALQAxADIANAAgACgAUgAtADEAMgA0ACkAXAAiACwAIABcACIAQwBIAEMAbABGAEMARgAzAFwAIgAsACAANQAyADcALAAgAFwAIgBIAEMARgBDAC0AMQAyADQAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABDAEYAQwAtADEANAAxAGIAIAAoAFIALQAxADQAMQBiACkAXAAiACwAIABcACIAQwBIADMAQwBDAGwAMgBGAFwAIgAsACAANwA4ADIALAAgAFwAIgBIAEMARgBDAC0AMQA0ADEAYgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEMARgBDAC0AMQA0ADIAYgAgACgAUgAtADEANAAyAGIAKQBcACIALAAgAFwAIgBDAEgAMgBDAEMAbABGADIAXAAiACwAIAAxADkAOAAwACwAIABcACIASABDAEYAQwAtADEANAAyAGIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASABDAEYAQwAtADIAMgA1AGMAYQAgACgAUgAtADIAMgA1AGMAYQApAFwAIgAsACAAXAAiAEMASABDAGwAMgBDAEYAMgBDAEYAMwBcACIALAAgADEAMgA3ACwAIABcACIASABDAEYAQwAtADIAMgA1AGMAYQBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBIAEMARgBDAC0AMgAyADUAYwBiACAAKABSAC0AMgAyADUAYwBiACkAXAAiACwAIABcACIAQwBIAEMAbABGAEMARgAyAEMAQwBJAEYAMgBcACIALAAgADUAMgA1ACwAIABcACIASABDAEYAQwAtADIAMgA1AGMAYgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAQwAtADEANAAgAFAAZQByAGYAbAB1AG8AcgBvAG0AZQB0AGgAYQBuAGUAIAAoAHQAZQB0AHIAYQBmAGwAdQBvAHIAbwBtAGUAdABoAGEAbgBlACkAXAAiACwAIABcACIAQwBGADQAXAAiACwAIAA2ADYAMwAwACwAIABcACIAUABGAEMALQAxADQAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABGAEMALQAxADEANgAgAFAAZQByAGYAbAB1AG8AcgBvAGUAdABoAGEAbgBlACAAKABoAGUAeABhAGYAbAB1AG8AcgBvAGUAdABoAGEAbgBlACkAXAAiACwAIABcACIAQwAyAEYANgBcACIALAAgADEAMQAxADAAMAAsACAAXAAiAFAARgBDAC0AMQAxADYAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABGAEMALQAyADEAOAAgAFAAZQByAGYAbAB1AG8AcgBvAHAAcgBvAHAAYQBuAGUAXAAiACwAIABcACIAQwAzAEYAOABcACIALAAgADgAOQAwADAALAAgAFwAIgBQAEYAQwAtADIAMQA4AFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAARgBDAC0AMwAxAC0AMQAwACAAUABlAHIAZgBsAHUAbwByAG8AYgB1AHQAYQBuAGUAXAAiACwAIABcACIAQwA0AEYAMQAwAFwAIgAsACAAOQAyADAAMAAsACAAXAAiAFAARgBDAC0AMwAxAC0AMQAwAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAARgBDAC0AMwAxADgAIABQAGUAcgBmAGwAdQBvAHIAbwBjAHkAYwBsAG8AYgB1AHQAYQBuAGUAXAAiACwAIABcACIAYwAtAEMANABGADgAXAAiACwAIAA5ADUANAAwACwAIABcACIAUABGAEMALQAzADEAOABcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAQwAtADQAMQAtADEAMgAgAFAAZQByAGYAbAB1AG8AcgBvAHAAZQBuAHQAYQBuAGUAXAAiACwAIABcACIAQwA1AEYAMQAyAFwAIgAsACAAOAA1ADUAMAAsACAAXAAiAFAARgBDAC0ANAAxAC0AMQAyAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAARgBDAC0ANQAxAC0AMQA0ACAAUABlAHIAZgBsAHUAbwByAG8AaABlAHgAYQBuAGUAXAAiACwAIABcACIAQwA2AEYAMQA0AFwAIgAsACAANwA5ADEAMAAsACAAXAAiAFAARgBDAC0ANQAxAC0AMQA0AFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAARgBDAC0AOQAxAC0AMQA4ACAAUABlAHIAZgBsAHUAbgBhAGYAZQBuAGUAXAAiACwAIABcACIAQwAxADAARgAxADgAXAAiACwAIAA3ADEAOQAwACwAIABcACIAUABGAEMALQA5ADEALQAxADgAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBGAEMALQAxADIAXAAiACwAIABcACIAQwBDAGwAMgBGADIAXAAiACwAIAAxADAAMgAwADAALAAgAFwAIgBDAEYAQwAtADEAMgBcACIALAAgAFwAIgBJAFAAQwBDACAARwBsAG8AYgBhAGwAIABXAGEAcgBtAGkAbgBnACAAUABvAHQAZQBuAHQAaQBhAGwAIABWAGEAbAB1AGUAcwAgAHYAMgAuADAAIAAtACAAKABBAFIANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMARgBDAC0AMQAzAFwAIgAsACAAXAAiAEMAQwBsAEYAMwBcACIALAAgADEAMwA5ADAAMAAsACAAXAAiAEMARgBDAC0AMQAzAFwAIgAsACAAXAAiAEkAUABDAEMAIABHAGwAbwBiAGEAbAAgAFcAYQByAG0AaQBuAGcAIABQAG8AdABlAG4AdABpAGEAbAAgAFYAYQBsAHUAZQBzACAAdgAyAC4AMAAgAC0AIAAoAEEAUgA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBGAEMALQAxADEANABcACIALAAgAFwAIgBDAEMAbABGADIAQwBDAGwARgAyAFwAIgAsACAAOAA1ADkAMAAsACAAXAAiAEMARgBDAC0AMQAxADQAXAAiACwAIABcACIASQBQAEMAQwAgAEcAbABvAGIAYQBsACAAVwBhAHIAbQBpAG4AZwAgAFAAbwB0AGUAbgB0AGkAYQBsACAAVgBhAGwAdQBlAHMAIAB2ADIALgAwACAALQAgACgAQQBSADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAEYAQwAtADEAMQA1AFwAIgAsACAAXAAiAEMAQwBsAEYAMgBDAEYAMwBcACIALAAgADcANgA3ADAALAAgAFwAIgBDAEYAQwAtADEAMQA1AFwAIgAsACAAXAAiAEkAUABDAEMAIABHAGwAbwBiAGEAbAAgAFcAYQByAG0AaQBuAGcAIABQAG8AdABlAG4AdABpAGEAbAAgAFYAYQBsAHUAZQBzACAAdgAyAC4AMAAgAC0AIAAoAEEAUgA1ACkAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABHAFcAUABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgACcARwBBAFMAIAAtACAARgBDACAAbgBhAG0AZQAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAdAByAHUAbgBjAGEAdABlAGQAIABnAGEAcwAgAG4AYQBtAGUAIAB0AG8AIABhAGwAbABvAHcAIABtAGEAdABjAGgAaQBuAGcAIAB3AGkAdABoACAAbwB0AGgAZQByACAAdABhAGIAbABlAHMALgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAGcAYQBzAGUAcwAgAGYAcgBvAG0AIABJAFAAQwBDACAARwBsAG8AYgBhAGwAIABXAGEAcgBtAGkAbgBnACAAUABvAHQAZQBuAHQAaQBhAGwAIABWAGEAbAB1AGUAcwAgAHYAMgAuADAAIAAtACAAKABBAFIANQApAC4AIABBAGQAZABlAGQAIAAnAEEAZABkAGkAdABpAG8AbgBhAGwAIABkAGEAdABhACAAcwBvAHUAcgBjAGUAJwAgAGMAbwBsAHUAbQBuAC4AXAAiACkAKQA7AFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBBAHAAcABlAG4AZABpAHgAIAAyACAARwBsAG8AYgBhAGwAIABXAGEAcgBtAGkAbgBnACAAUABvAHQAZQBuAHQAaQBhAGwAcwA6ACAAQgBsAGUAbgBkAGUAZAAgAHIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABCAGwAZQBuAGQAcwBfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEIAbABlAG4AZABlAGQAIAByAGUAZgByAGkAZwBlAHIAYQBuAHQAcwAgACgAbQBhAG4AeQAgAGMAbwBuAHQAYQBpAG4AaQBuAGcAIABIAEYAQwBTACAAYQBuAGQALwBvAHIAIABQAEYAQwBTACkAXAAiACkAKQA7AFwAbgBcAG4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBDAGgAZQBtAGkAYwBhAGwAQgBsAGUAbgBkAHMAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABCAGwAZQBuAGQAcwBfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABBAHAAcABlAG4AZABpAHgAIAAyACAALQAgAFQAYQBiAGwAZQAgADIANABcACIAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABCAGwAZQBuAGQAcwBfAEQAYQB0AGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAxACwAIAAzACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEIAbABlAG4AZABcACIALAAgAFwAIgBDAG8AbgBzAHQAaQB0AHUAZQBuAHQAcwBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwBpAHQAaQBvAG4AIAAoACUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADAAXAAiACwAIABcACIAQwBGAEMALQAxADIALwBDAEYAQwAtADEAMQA0AFwAIgAsACAAXAAiAFIALQA0ADAAMAAgAGMAYQBuACAAaABhAHYAZQAgAHYAYQByAGkAbwB1AHMAIABwAHIAbwBwAG8AcgB0AGkAbwBuAHMAIABvAGYAIABDAEYAQwAtADEAMgAgAGEAbgBkACAAQwBGAEMALQAxADEANAAuACAAVABoAGUAIABlAHgAYQBjAHQAIABjAG8AbQBwAG8AcwBpAHQAaQBvAG4AIABuAGUAZQBkAHMAIAB0AG8AIABiAGUAIABzAHAAZQBjAGkAZgBpAGUAZAAsACAAZQAuAGcALgAsACAAUgAtADQAMAAwACAAKAA2ADAALwA0ADAAKQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADAAMQBBAFwAIgAsACAAXAAiAEgAQwBGAEMALQAyADIALwBIAEYAQwAtADEANQAyAGEALwBIAEMARgBDAC0AMQAyADQAXAAiACwAIABcACIAKAA1ADMALgAwAC8AMQAzAC4AMAAvADMANAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADEAQgBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8ASABGAEMALQAxADUAMgBhAC8ASABDAEYAQwAtADEAMgA0AFwAIgAsACAAXAAiACgANgAxAC4AMAAvADEAMQAuADAALwAyADgALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAAxAEMAXAAiACwAIABcACIASABDAEYAQwAtADIAMgAvAEgARgBDAC0AMQA1ADIAYQAvAEgAQwBGAEMALQAxADIANABcACIALAAgAFwAIgAoADMAMwAuADAALwAxADUALgAwAC8ANQAyAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADAAMgBBAFwAIgAsACAAXAAiAEgARgBDAC0AMQAyADUALwBIAEMALQAyADkAMAAvAEgAQwBGAEMALQAyADIAXAAiACwAIABcACIAKAA2ADAALgAwAC8AMgAuADAALwAzADgALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAAyAEIAXAAiACwAIABcACIASABGAEMALQAxADIANQAvAEgAQwAtADIAOQAwAC8ASABDAEYAQwAtADIAMgBcACIALAAgAFwAIgAoADMAOAAuADAALwAyAC4AMAAvADYAMAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADMAQQBcACIALAAgAFwAIgBIAEMALQAyADkAMAAvAEgAQwBGAEMALQAyADIALwBQAEYAQwAtADIAMQA4AFwAIgAsACAAXAAiACgANQAuADAALwA3ADUALgAwAC8AMgAwAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADAAMwBCAFwAIgAsACAAXAAiAEgAQwAtADIAOQAwAC8ASABDAEYAQwAtADIAMgAvAFAARgBDAC0AMgAxADgAXAAiACwAIABcACIAKAA1AC4AMAAvADUANgAuADAALwAzADkALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAA0AEEAXAAiACwAIABcACIASABGAEMALQAxADIANQAvAEgARgBDAC0AMQA0ADMAYQAvAEgARgBDAC0AMQAzADQAYQBcACIALAAgAFwAIgAoADQANAAuADAALwA1ADIALgAwAC8ANAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADUAQQBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8AIABIAEYAQwAtADEANQAyAGEALwBIAEMARgBDAC0AMQA0ADIAYgAvAFAARgBDAC0AMwAxADgAXAAiACwAIABcACIAKAA0ADUALgAwAC8ANwAuADAALwA1AC4ANQAvADQAMgAuADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAwADYAQQBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8ASABDAC0ANgAwADAAYQAvAEgAQwBGAEMALQAxADQAMgBiAFwAIgAsACAAXAAiACgANQA1AC4AMAAvADEANAAuADAALwA0ADEALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAA3AEEAXAAiACwAIABcACIASABGAEMALQAzADIALwBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADMANABhAFwAIgAsACAAXAAiACgAMgAwAC4AMAAvADQAMAAuADAALwA0ADAALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAA3AEIAXAAiACwAIABcACIASABGAEMALQAzADIALwBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADMANABhAFwAIgAsACAAXAAiACgAMQAwAC4AMAAvADcAMAAuADAALwAyADAALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAA3AEMAXAAiACwAIABcACIASABGAEMALQAzADIALwBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADMANABhAFwAIgAsACAAXAAiACgAMgAzAC4AMAAvADIANQAuADAALwA1ADIALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAA3AEQAXAAiACwAIABcACIASABGAEMALQAzADIALwBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADMANABhAFwAIgAsACAAXAAiACgAMQA1AC4AMAAvADEANQAuADAALwA3ADAALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAA3AEUAXAAiACwAIABcACIASABGAEMALQAzADIALwBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADMANABhAFwAIgAsACAAXAAiACgAMgA1AC4AMAAvADEANQAuADAALwA2ADAALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAA4AEEAXAAiACwAIABcACIASABGAEMALQAxADIANQAvAEgARgBDAC0AMQA0ADMAYQAvAEgAQwBGAEMALQAyADIAXAAiACwAIABcACIAKAA3AC4AMAAvADQANgAuADAALwA0ADcALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAA5AEEAXAAiACwAIABcACIASABDAEYAQwAtADIAMgAvAEgAQwBGAEMALQAxADIANAAvAEgAQwBGAEMALQAxADQAMgBiAFwAIgAsACAAXAAiACgANgAwAC4AMAAvADIANQAuADAALwAxADUALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMAA5AEIAXAAiACwAIABcACIASABDAEYAQwAtADIAMgAvAEgAQwBGAEMALQAxADIANAAvAEgAQwBGAEMALQAxADQAMgBiAFwAIgAsACAAXAAiACgANgA1AC4AMAAvADIANQAuADAALwAxADAALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQAwAEEAXAAiACwAIABcACIASABGAEMALQAzADIALwBIAEYAQwAtADEAMgA1AFwAIgAsACAAXAAiACgANQAwAC4AMAAvADUAMAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAxADAAQgBcACIALAAgAFwAIgBIAEYAQwAtADMAMgAvAEgARgBDAC0AMQAyADUAXAAiACwAIABcACIAKAA0ADUALgAwAC8ANQA1AC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEAMQBBAFwAIgAsACAAXAAiAEgAQwAtADEAMgA3ADAALwBIAEMARgBDAC0AMgAyAC8ASABGAEMALQAxADUAMgBhAFwAIgAsACAAXAAiACgAMQAuADUALwA4ADcALgA1AC8AMQAxAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEAMQBCAFwAIgAsACAAXAAiAEgAQwAtADEAMgA3ADAALwBIAEMARgBDAC0AMgAyAC8ASABGAEMALQAxADUAMgBhAFwAIgAsACAAXAAiACgAMwAuADAALwA5ADQALgAwAC8AMwAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAxADEAQwBcACIALAAgAFwAIgBIAEMALQAxADIANwAwAC8ASABDAEYAQwAtADIAMgAvAEgARgBDAC0AMQA1ADIAYQBcACIALAAgAFwAIgAoADMALgAwAC8AOQA1AC4ANQAvADEALgA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQAyAEEAXAAiACwAIABcACIASABDAEYAQwAtADIAMgAvAFAARgBDAC0AMgAxADgALwBIAEMARgBDAC0AMQA0ADIAYgBcACIALAAgAFwAIgAoADcAMAAuADAALwA1AC4AMAAvADIANQAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAxADMAQQBcACIALAAgAFwAIgBQAEYAQwAtADIAMQA4AC8ASABGAEMALQAxADMANABhAC8ASABDAC0ANgAwADAAYQBcACIALAAgAFwAIgAoADkALgAwAC8AOAA4AC4AMAAvADMALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQA0AEEAXAAiACwAIABcACIASABDAEYAQwAtADIAMgAvAEgAQwBGAEMALQAxADIANAAvAEgAQwAtADYAMAAwAGEALwBIAEMARgBDAC0AMQA0ADIAYgBcACIALAAgAFwAIgAoADUAMQAuADAALwAyADgALgA1AC8ANAAuADAALwAxADYALgA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADQAMQA0AEIAXAAiACwAIABcACIASABDAEYAQwAtADIAMgAvAEgAQwBGAEMALQAxADIANAAvAEgAQwAtADYAMAAwAGEALwBIAEMARgBDAC0AMQA0ADIAYgBcACIALAAgAFwAIgAoADUAMAAuADAALwAzADkALgAwAC8AMQAuADUALwA5AC4ANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEANQBBAFwAIgAsACAAXAAiAEgAQwBGAEMALQAyADIALwBIAEYAQwAtADEANQAyAGEAXAAiACwAIABcACIAKAA4ADIALgAwAC8AMQA4AC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEANQBCAFwAIgAsACAAXAAiAEgAQwBGAEMALQAyADIALwBIAEYAQwAtADEANQAyAGEAXAAiACwAIABcACIAKAAyADUALgAwAC8ANwA1AC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEANgBBAFwAIgAsACAAXAAiAEgARgBDAC0AMQAzADQAYQAvAEgAQwBGAEMALQAxADIANAAvAEgAQwAtADYAMAAwAFwAIgAsACAAXAAiACgANQA5AC4AMAAvADMAOQAuADUALwAxAC4ANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEANwBBAFwAIgAsACAAXAAiAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEALwBIAEMALQA2ADAAMABcACIALAAgAFwAIgAoADQANgAuADYALwA1ADAALgAwAC8AMwAuADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAxADgAQQBcACIALAAgAFwAIgBIAEMALQAyADkAMAAvAEgAQwBGAEMALQAyADIALwBIAEYAQwAtADEANQAyAGEAXAAiACwAIABcACIAKAAxAC4ANQAvADkANgAuADAALwAyAC4ANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADEAOQBBAFwAIgAsACAAXAAiAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEAMwA0AGEALwBIAEUALQBFADEANwAwAFwAIgAsACAAXAAiACgANwA3AC4AMAAvADEAOQAuADAALwA0AC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA0ADIAMABBAFwAIgAsACAAXAAiAEgARgBDAC0AMQAzADQAYQAvAEgAQwBGAEMALQAxADQAMgBiAFwAIgAsACAAXAAiACgAOAA4AC4AMAAvADEAMgAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAyADEAQQBcACIALAAgAFwAIgBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADMANABhAFwAIgAsACAAXAAiACgANQA4AC4AMAAvADQAMgAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAyADIAQQBcACIALAAgAFwAIgBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADMANABhAC8ASABDAC0ANgAwADAAYQBcACIALAAgAFwAIgAoADgANQAuADEALwAxADEALgA1AC8AMwAuADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAyADIAQgBcACIALAAgAFwAIgBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADMANABhAC8ASABDAC0ANgAwADAAYQBcACIALAAgAFwAIgAoADUANQAuADAALwA0ADIALgAwAC8AMwAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANAAyADIAQwBcACIALAAgAFwAIgBIAEYAQwAtADEAMgA1AC8ASABGAEMALQAxADMANABhAC8ASABDAC0ANgAwADAAYQBcACIALAAgAFwAIgAoADgAMgAuADAALwAxADUALgAwAC8AMwAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANQAwADAAXAAiACwAIABcACIAQwBGAEMALQAxADIALwBIAEYAQwAtADEANQAyAGEAXAAiACwAIABcACIAKAA3ADMALgA4AC8AMgA2AC4AMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA1ADAAMQBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8AQwBGAEMALQAxADIAXAAiACwAIABcACIAKAA3ADUALgAwAC8AMgA1AC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA1ADAAMgBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8AQwBGAEMALQAxADEANQBcACIALAAgAFwAIgAoADQAOAAuADgALwA1ADEALgAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADUAMAAzAFwAIgAsACAAXAAiAEgARgBDAC0AMgAzAC8AQwBGAEMALQAxADMAXAAiACwAIABcACIAKAA0ADAALgAxAC8ANQA5AC4AOQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA1ADAANABcACIALAAgAFwAIgBIAEYAQwAtADMAMgAvAEMARgBDAC0AMQAxADUAXAAiACwAIABcACIAKAA0ADgALgAyAC8ANQAxAC4AOAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA1ADAANQBcACIALAAgAFwAIgBDAEYAQwAtADEAMgAvAEgAQwBGAEMALQAzADEAXAAiACwAIABcACIAKAA3ADgALgAwAC8AMgAyAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA1ADAANgBcACIALAAgAFwAIgBDAEYAQwAtADMAMQAvAEMARgBDAC0AMQAxADQAXAAiACwAIABcACIAKAA1ADUALgAxAC8ANAA0AC4AOQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA1ADAANwBBAFwAIgAsACAAXAAiAEgARgBDAC0AMQAyADUALwBIAEYAQwAtADEANAAzAGEAXAAiACwAIABcACIAKAA1ADAALgAwAC8ANQAwAC4AMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIALQA1ADAAOABBAFwAIgAsACAAXAAiAEgARgBDAC0AMgAzAC8AUABGAEMALQAxADEANgBcACIALAAgAFwAIgAoADMAOQAuADAALwA2ADEALgAwACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUgAtADUAMAA4AEIAXAAiACwAIABcACIASABGAEMALQAyADMALwBQAEYAQwAtADEAMQA2AFwAIgAsACAAXAAiACgANAA2AC4AMAAvADUANAAuADAAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBSAC0ANQAwADkAQQBcACIALAAgAFwAIgBIAEMARgBDAC0AMgAyAC8AUABGAEMALQAyADEAOABcACIALAAgAFwAIgAoADQANAAuADAALwA1ADYALgAwACkAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABCAGwAZQBuAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAYwBoAGEAbgBnAGUAZAAgAEgAQwA2ADAAMABhACAAdABvACAASABDAC0ANgAwADAAYQAgAGYAbwByACAAYgBsAGUAbgBkACAAUgAtADQAMQA0AEIALgAgAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABmAG8AcgAgAGIAbABlAG4AZAAgAFIALQA0ADAANQBBACAALQAgAEMAaABhAG4AZwBlAGQAIABIAEMARgBDADEANAAyAGIAIAB0AG8AIABIAEMARgBDAC0AMQA0ADIAYgAuAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEwAZQBhAGsAYQBnAGUAIAByAGEAdABlAHMAIABmAG8AcgAgAGMAbwBtAG0AbwBuACAAcgBlAGYAcgBpAGcAZQByAGEAdABpAG8AbgAgAGEAbgBkACAAYQBpAHIAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ATABlAGEAawBhAGcAZQBSAGEAdABlAHMAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBJAG4AZABpAGMAYQB0AGkAdgBlACAAbABlAGEAawBhAGcAZQAgAHIAYQB0AGUAcwAgAGYAbwByACAAYwBvAG0AbQBvAG4AIAByAGUAZgByAGkAZwBlAHIAYQB0AGkAbwBuACAAYQBuAGQAIABhAGkAcgAgAC0AIABjAG8AbgBkAGkAdABpAG8AbgBpAG4AZwAgAGUAcQB1AGkAcABtAGUAbgB0AFwAIgApACkAOwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ATABlAGEAawBhAGcAZQBSAGEAdABlAHMAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEwAZQBhAGsAYQBnAGUAUgBhAHQAZQBzAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAALQAgAFQAYQBiAGwAZQAgADEAMABcACIAKQApADsAXABuAFwAbgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEwAZQBhAGsAYQBnAGUAUgBhAHQAZQBzAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIABsAGUAYQBrAGEAZwBlACAAcgBhAHQAZQAgACgAJQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwAgAHIAZQBmAHIAaQBnAGUAcgBhAHQAbwByAHMAXAAiACwAIAAxAC4ANwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBhAG4AcwBwAG8AcgB0ACAAcgBlAGYAcgBpAGcAZQByAGEAdABpAG8AbgBcACIALAAgADEANQAuADcAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAIABBAC8AQwAgAHAAbwByAHQAYQBiAGwAZQBcACIALAAgADIALgA1ADsAXABuACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjACAAQQAvAEMAIABzAHAAbABpAHQAXAAiACwAIAAzAC4ANQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwAgAEEALwBDACAAcABhAGMAawBhAGcAZQBkAFwAIgAsACAAMgAuADUAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGkAZwBoAHQAIAB2AGUAaABpAGMAbABlACAAQQAvAEMAXAAiACwAIAA2AC4ANwA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBhAHYAeQAgAHYAZQBoAGkAYwBsAGUAIABBAC8AQwBcACIALAAgADEAMAAuADgAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ATABlAGEAawBhAGcAZQBSAGEAdABlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAYQBsAGMAdQBsAGEAdABlAEIAbABlAG4AZABHAFcAUABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEYAYQBjAHQAaQBvAG4AMQAsACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEcAVwBQADEALAAgAFwAbgAgACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEYAYQBjAHQAaQBvAG4AMgAsACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEcAVwBQADIALAAgAFwAbgAgACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEYAYQBjAHQAaQBvAG4AMwAsACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEcAVwBQADMALAAgAFwAbgAgACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEYAYQBjAHQAaQBvAG4ANAAsACAAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEcAVwBQADQALABcAG4AIAAgACgAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEYAYQBjAHQAaQBvAG4AMQAgACoAIABDAG8AbgBzAHQAaQB0AHUAZQBuAHQARwBXAFAAMQApACAAKwBcAG4AIAAgACgAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEYAYQBjAHQAaQBvAG4AMgAgACoAIABDAG8AbgBzAHQAaQB0AHUAZQBuAHQARwBXAFAAMgApACAAKwBcAG4AIAAgACgAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEYAYQBjAHQAaQBvAG4AMwAgACoAIABDAG8AbgBzAHQAaQB0AHUAZQBuAHQARwBXAFAAMwApACAAKwBcAG4AIAAgACgAQwBvAG4AcwB0AGkAdAB1AGUAbgB0AEYAYQBjAHQAaQBvAG4ANAAgACoAIABDAG8AbgBzAHQAaQB0AHUAZQBuAHQARwBXAFAANAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFQAaQB0AGwAZQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8ARABhAHQAYQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEcAYQBzAGUAbwB1AHMAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8ARABlAHMAYwByAGkAcAB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkARwBhAHMAZQBvAHUAcwBfAEQAYQB0AGEAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBHAGEAcwBlAG8AdQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBTAHQAYQB0AGkAbwBuAGEAcgB5AEwAaQBxAHUAaQBkAF8AVABpAHQAbABlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAUwB0AGEAdABpAG8AbgBhAHIAeQBMAGkAcQB1AGkAZABfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBEAGEAdABhACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFMAdABhAHQAaQBvAG4AYQByAHkATABpAHEAdQBpAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFQAaQB0AGwAZQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFMAbwB1AHIAYwBlACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AF8ARABhAHQAYQAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARgB1AGUAbABfAFMAYwBvAHAAZQAxAFMAYwBvAHAAZQAzAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAFQAcgBhAG4AcwBwAG8AcgB0AE8AZgBmAFIAbwBhAGQAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEYAdQBlAGwAXwBTAGMAbwBwAGUAMQBTAGMAbwBwAGUAMwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBUAHIAYQBuAHMAcABvAHIAdABPAGYAZgBSAG8AYQBkAF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBGAHUAZQBsAF8AUwBjAG8AcABlADEAUwBjAG8AcABlADMARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMAVAByAGEAbgBzAHAAbwByAHQATwBmAGYAUgBvAGEAZABfAEQAYQB0AGEAIgAsACIARgB1AGUAbABfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEYAdQBlAGwAXwBHAGUAdABUAHIAYQBuAHMAcABvAHIAdABGAHUAZQBsAFMAdAByAGkAbgBnACIALAAiAEYAdQBlAGwAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBGAHUAZQBsAF8ARwBlAHQAUwB0AGEAdABpAG8AbgBhAHIAeQBGAHUAZQBsAFMAdAByAGkAbgBnACIALAAiAEYAdQBlAGwAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBGAHUAZQBsAF8AVABvAHQAYQBsAEMAbwBuAHMAdQBtAHAAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAFQAaQB0AGwAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBVAG4AaQB0ACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAxAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AVAByAGEAbgBzAHAAbwByAHQAXwBTAG8AdQByAGMAZQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMQBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFQAcgBhAG4AcwBwAG8AcgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADEAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBUAHIAYQBuAHMAcABvAHIAdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBUAGkAdABsAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEYAdQBlAGwAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADgAXwAyAF8AMQBfADEAXwBfADEAXwBGAHUAZQBsAEMAbwBtAGIAdQBzAHQAaQBvAG4AUwB0AGEAdABpAG8AbgBhAHIAeQBfAFUAbgBpAHQAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8AUwBvAHUAcgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARgB1AGUAbABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOABfADIAXwAxAF8AMQBfAF8AMQBfAEYAdQBlAGwAQwBvAG0AYgB1AHMAdABpAG8AbgBTAHQAYQB0AGkAbwBuAGEAcgB5AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBGAHUAZQBsAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA4AF8AMgBfADEAXwAxAF8AXwAxAF8ARgB1AGUAbABDAG8AbQBiAHUAcwB0AGkAbwBuAFMAdABhAHQAaQBvAG4AYQByAHkAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBfAFQAaQB0AGwAZQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBVAG4AaQB0ACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBHAFcAUABfAFUAbgBpAHQAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAF8AUwBvAHUAcgBjAGUAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAF8AUgBlAGEAZABhAGIAbABlAEUAcQB1AGEAdABpAG8AbgAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AOQBfADEAXwAxAF8AXwAxAF8AUgBlAGYAcgBpAGcAZQByAGEAbgB0AEwAZQBhAGsAaQBuAGcAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA5AF8AMQBfADEAXwBfADEAXwBSAGUAZgByAGkAZwBlAHIAYQBuAHQATABlAGEAawBpAG4AZwBHAFcAUABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAEcAVwBQAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADkAXwAxAF8AMQBfAF8AMQBfAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABMAGUAYQBrAGkAbgBnAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBDAGgAZQBtAGkAYwBhAGwARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBDAGgAZQBtAGkAYwBhAGwARwBXAFAAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBDAGgAZQBtAGkAYwBhAGwARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABHAFcAUABfAEQAYQB0AGEAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBDAGgAZQBtAGkAYwBhAGwARwBXAFAAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABCAGwAZQBuAGQAcwBfAFQAaQB0AGwAZQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABCAGwAZQBuAGQAcwBfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABCAGwAZQBuAGQAcwBfAFMAbwB1AHIAYwBlACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AQwBoAGUAbQBpAGMAYQBsAEIAbABlAG4AZABzAF8ARABhAHQAYQAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEMAaABlAG0AaQBjAGEAbABCAGwAZQBuAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ATABlAGEAawBhAGcAZQBSAGEAdABlAHMAXwBUAGkAdABsAGUAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBMAGUAYQBrAGEAZwBlAFIAYQB0AGUAcwBfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgAiACwAIgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBSAGUAZgByAGkAZwBlAHIAYQBuAHQAcwBfAEwAZQBhAGsAYQBnAGUAUgBhAHQAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBMAGUAYQBrAGEAZwBlAFIAYQB0AGUAcwBfAEQAYQB0AGEAIgAsACIAUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBMAGUAYQBrAGEAZwBlAFIAYQB0AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFIAZQBmAHIAaQBnAGUAcgBhAG4AdABzAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AUgBlAGYAcgBpAGcAZQByAGEAbgB0AHMAXwBDAGEAbABjAHUAbABhAHQAZQBCAGwAZQBuAGQARwBXAFAAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -19525,23 +19524,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19558,4 +19541,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>